<commit_message>
Add human-readable UP/DOWN recommendation scenario engine
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -18,6 +18,8 @@
     <sheet name="BasketSummary" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Validation" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Log" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="ScenarioText_UP" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="ScenarioText_DOWN" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -804,12 +806,775 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1">
-        <f>"NEXT ACTION UP:"&amp;CHAR(10)&amp;BasketSummary!B13&amp;CHAR(10)&amp;"NEXT ACTION DOWN:"&amp;CHAR(10)&amp;BasketSummary!C13</f>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TailBefore</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>TailClosed</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>TailAfter</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>RecoveryBefore</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>RecoveryAfter</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>ReserveAfter</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>NOW()</f>
+        <v/>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ScenarioText_UP</t>
+        </is>
+      </c>
+      <c r="D2">
+        <f>BasketSummary!B13</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>TailRecovery_UP!B3</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>TailRecovery_UP!B10</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>MAX(E2-F2,0)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>TailRecovery_UP!B5</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>TailRecovery_UP!B7</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>SectionCalculator_UP!B35</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>IF(OR(SectionCalculator_UP!B12&lt;&gt;"YES",SectionCalculator_UP!B13&lt;&gt;"YES"),"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>NOW()</f>
+        <v/>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ScenarioText_DOWN</t>
+        </is>
+      </c>
+      <c r="D3">
+        <f>BasketSummary!C13</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>TailRecovery_DOWN!B3</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>TailRecovery_DOWN!B10</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>MAX(E3-F3,0)</f>
+        <v/>
+      </c>
+      <c r="H3">
+        <f>TailRecovery_DOWN!B5</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>TailRecovery_DOWN!B7</f>
+        <v/>
+      </c>
+      <c r="J3">
+        <f>SectionCalculator_DOWN!B35</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>IF(OR(SectionCalculator_DOWN!B12&lt;&gt;"YES",SectionCalculator_DOWN!B13&lt;&gt;"YES"),"YES","NO")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ScenarioTitle</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>"SCENARIO: PRICE MOVES UP"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CurrentPrice</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>Scenario_UP!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NextTriggerLevel</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SectionCalculator_UP!B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DistancePoints</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>ROUND(ABS(B4-B3)*10000,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BigPosition</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>"SELL "&amp;TEXT(TailRecovery_UP!B16,"0.00")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SmallHedge</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>"BUY "&amp;TEXT(TailRecovery_UP!B17,"0.00")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SectionLevel</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>SectionCalculator_UP!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(SectionCalculator_UP!B12="YES","Reached level; tail found; risk limits OK","Waiting level/risk gate")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RiskChecks</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CanOpenSection</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>SectionCalculator_UP!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NoOppositeCascade</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>SectionCalculator_UP!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CanCloseSection</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>SectionCalculator_UP!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CanCloseTail</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>TailRecovery_UP!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CycleProfit</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>SectionCalculator_UP!B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ReserveAdd</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>TailRecovery_UP!B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RecoveryAdd</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>TailRecovery_UP!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DetectedTailType</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>TailRecovery_UP!B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TailLot</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>TailRecovery_UP!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TailLoss</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>TailRecovery_UP!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RecoveryFundBefore</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>TailRecovery_UP!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CloseLotRaw</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>TailRecovery_UP!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CloseLotRounded</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>TailRecovery_UP!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CloseLotFinal</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>TailRecovery_UP!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TailLotAfter</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>MAX(B22-B27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RecoveryFundAfter</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>TailRecovery_UP!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HumanReadableAction</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>TEXTJOIN(CHAR(10),TRUE,B2,"Current Price: "&amp;TEXT(B3,"0.00000"),"Next trigger level: "&amp;TEXT(B4,"0.00000")&amp;" ("&amp;TEXT(B5,"0")&amp;" points)","Open section: "&amp;B6&amp;" + "&amp;B7,"Section level: "&amp;TEXT(B8,"0"),"CycleProfit: "&amp;TEXT(B17,"0.00"),"Reserve += "&amp;TEXT(B18,"0.00")&amp;"; Recovery += "&amp;TEXT(B19,"0.00"),"Tail: "&amp;B21&amp;" "&amp;TEXT(B22,"0.00")&amp;"; Close "&amp;TEXT(B27,"0.00")&amp;"; Remain "&amp;TEXT(B28,"0.00"),"CanCloseBasket: "&amp;BasketSummary!B10,"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ScenarioTitle</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>"SCENARIO: PRICE MOVES DOWN"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CurrentPrice</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>Scenario_DOWN!B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>NextTriggerLevel</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>SectionCalculator_DOWN!B15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DistancePoints</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>ROUND(ABS(B4-B3)*10000,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BigPosition</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>"SELL "&amp;TEXT(TailRecovery_DOWN!B16,"0.00")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SmallHedge</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>"BUY "&amp;TEXT(TailRecovery_DOWN!B17,"0.00")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SectionLevel</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>SectionCalculator_DOWN!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Reason</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(SectionCalculator_DOWN!B12="YES","Reached level; tail found; risk limits OK","Waiting level/risk gate")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RiskChecks</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>CanOpenSection</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>SectionCalculator_DOWN!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NoOppositeCascade</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>SectionCalculator_DOWN!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CanCloseSection</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>SectionCalculator_DOWN!B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CanCloseTail</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>TailRecovery_DOWN!B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CycleProfit</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>SectionCalculator_DOWN!B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ReserveAdd</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>TailRecovery_DOWN!B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>RecoveryAdd</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>TailRecovery_DOWN!B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DetectedTailType</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>TailRecovery_DOWN!B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TailLot</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>TailRecovery_DOWN!B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TailLoss</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>TailRecovery_DOWN!B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>RecoveryFundBefore</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>TailRecovery_DOWN!B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CloseLotRaw</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>TailRecovery_DOWN!B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>CloseLotRounded</t>
+        </is>
+      </c>
+      <c r="B26">
+        <f>TailRecovery_DOWN!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>CloseLotFinal</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>TailRecovery_DOWN!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TailLotAfter</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>MAX(B22-B27,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RecoveryFundAfter</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>TailRecovery_DOWN!B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>HumanReadableAction</t>
+        </is>
+      </c>
+      <c r="B31">
+        <f>TEXTJOIN(CHAR(10),TRUE,B2,"Current Price: "&amp;TEXT(B3,"0.00000"),"Next trigger level: "&amp;TEXT(B4,"0.00000")&amp;" ("&amp;TEXT(B5,"0")&amp;" points)","Open section: "&amp;B6&amp;" + "&amp;B7,"Section level: "&amp;TEXT(B8,"0"),"CycleProfit: "&amp;TEXT(B17,"0.00"),"Reserve += "&amp;TEXT(B18,"0.00")&amp;"; Recovery += "&amp;TEXT(B19,"0.00"),"Tail: "&amp;B21&amp;" "&amp;TEXT(B22,"0.00")&amp;"; Close "&amp;TEXT(B27,"0.00")&amp;"; Remain "&amp;TEXT(B28,"0.00"),"CanCloseBasket: "&amp;BasketSummary!C10,"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
         <v/>
       </c>
     </row>
@@ -19984,7 +20749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20184,6 +20949,21 @@
         <v/>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HumanReadableAction</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>ScenarioText_UP!B31</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>ScenarioText_DOWN!B31</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Russian UP/DOWN recommendation engine and safe text outputs
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -29,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,13 +40,23 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="13"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -61,9 +71,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -812,52 +825,52 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Timestamp</t>
+          <t>Время</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Direction</t>
+          <t>Направление</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Scenario</t>
+          <t>Сценарий</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Действие</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>TailBefore</t>
+          <t>Хвост до закрытия</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>TailClosed</t>
+          <t>Закрываемый лот хвоста</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>TailAfter</t>
+          <t>Хвост после закрытия</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>RecoveryBefore</t>
+          <t>RecoveryFund до</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>RecoveryAfter</t>
+          <t>RecoveryFund после</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>ReserveAfter</t>
+          <t>Резерв после</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -873,7 +886,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>UP</t>
+          <t>ВВЕРХ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -910,7 +923,7 @@
         <v/>
       </c>
       <c r="K2">
-        <f>IF(OR(SectionCalculator_UP!B12&lt;&gt;"YES",SectionCalculator_UP!B13&lt;&gt;"YES"),"YES","NO")</f>
+        <f>IF(OR(SectionCalculator_UP!B14&lt;&gt;"YES",SectionCalculator_UP!B13&lt;&gt;"YES"),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -921,7 +934,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DOWN</t>
+          <t>ВНИЗ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -958,7 +971,7 @@
         <v/>
       </c>
       <c r="K3">
-        <f>IF(OR(SectionCalculator_DOWN!B12&lt;&gt;"YES",SectionCalculator_DOWN!B13&lt;&gt;"YES"),"YES","NO")</f>
+        <f>IF(OR(SectionCalculator_DOWN!B14&lt;&gt;"YES",SectionCalculator_DOWN!B13&lt;&gt;"YES"),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -973,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -991,113 +1004,113 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ScenarioTitle</t>
+          <t>Название сценария</t>
         </is>
       </c>
       <c r="B2">
-        <f>"SCENARIO: PRICE MOVES UP"</f>
+        <f>"СЦЕНАРИЙ: ЦЕНА ИДЕТ ВВЕРХ"</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CurrentPrice</t>
+          <t>Текущая цена</t>
         </is>
       </c>
       <c r="B3">
-        <f>Scenario_UP!B4</f>
+        <f>IFERROR(Scenario_UP!B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NextTriggerLevel</t>
+          <t>Следующий уровень</t>
         </is>
       </c>
       <c r="B4">
-        <f>SectionCalculator_UP!B15</f>
+        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!E4,IF(SectionCalculator_UP!B4=2,Scenario_UP!E5,IF(SectionCalculator_UP!B4=3,Scenario_UP!E6,IF(SectionCalculator_UP!B4=4,Scenario_UP!E7,"")))),"")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DistancePoints</t>
+          <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
       <c r="B5">
-        <f>ROUND(ABS(B4-B3)*10000,0)</f>
+        <f>IF(OR(B4="",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BigPosition</t>
+          <t>Большая позиция</t>
         </is>
       </c>
       <c r="B6">
-        <f>"SELL "&amp;TEXT(TailRecovery_UP!B16,"0.00")</f>
+        <f>IFERROR(IF(TailRecovery_UP!B16&gt;0,IF("UP"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_UP!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SmallHedge</t>
+          <t>Малая защитная позиция</t>
         </is>
       </c>
       <c r="B7">
-        <f>"BUY "&amp;TEXT(TailRecovery_UP!B17,"0.00")</f>
+        <f>IFERROR(IF(TailRecovery_UP!B17&gt;0,IF("UP"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_UP!B17,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SectionLevel</t>
+          <t>Уровень секции</t>
         </is>
       </c>
       <c r="B8">
-        <f>SectionCalculator_UP!B16</f>
+        <f>IFERROR(SectionCalculator_UP!B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Причина</t>
         </is>
       </c>
       <c r="B9">
-        <f>IF(SectionCalculator_UP!B12="YES","Reached level; tail found; risk limits OK","Waiting level/risk gate")</f>
+        <f>IF(SectionCalculator_UP!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция сейчас недоступна: уровень/риск-гейт/хвост")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RiskChecks</t>
+          <t>Проверки риска</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CanOpenSection</t>
+          <t>Можно открыть секцию</t>
         </is>
       </c>
       <c r="B12">
-        <f>SectionCalculator_UP!B12</f>
+        <f>SectionCalculator_UP!B14</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NoOppositeCascade</t>
+          <t>Нет встречного каскада</t>
         </is>
       </c>
       <c r="B13">
@@ -1108,7 +1121,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CanCloseSection</t>
+          <t>Можно закрыть секцию</t>
         </is>
       </c>
       <c r="B14">
@@ -1119,7 +1132,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CanCloseTail</t>
+          <t>Можно закрыть хвост</t>
         </is>
       </c>
       <c r="B15">
@@ -1130,132 +1143,132 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CycleProfit</t>
+          <t>Прибыль цикла</t>
         </is>
       </c>
       <c r="B17">
-        <f>SectionCalculator_UP!B31</f>
+        <f>IFERROR(SectionCalculator_UP!B31,0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ReserveAdd</t>
+          <t>Добавить в резерв</t>
         </is>
       </c>
       <c r="B18">
-        <f>TailRecovery_UP!B6</f>
+        <f>IFERROR(TailRecovery_UP!B6,0)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RecoveryAdd</t>
+          <t>Добавить в RecoveryFund</t>
         </is>
       </c>
       <c r="B19">
-        <f>TailRecovery_UP!B8</f>
+        <f>IFERROR(TailRecovery_UP!B8,0)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DetectedTailType</t>
+          <t>Тип хвоста</t>
         </is>
       </c>
       <c r="B21">
-        <f>TailRecovery_UP!B2</f>
+        <f>IF(OR(TailRecovery_UP!B2="",TailRecovery_UP!B2="N/A"),"Хвост не найден",TailRecovery_UP!B2)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TailLot</t>
+          <t>Лот хвоста</t>
         </is>
       </c>
       <c r="B22">
-        <f>TailRecovery_UP!B3</f>
+        <f>IFERROR(IF(TailRecovery_UP!B3&gt;0,TailRecovery_UP!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TailLoss</t>
+          <t>Убыток хвоста</t>
         </is>
       </c>
       <c r="B23">
-        <f>TailRecovery_UP!B12</f>
+        <f>IFERROR(TailRecovery_UP!B12,0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RecoveryFundBefore</t>
+          <t>RecoveryFund до закрытия</t>
         </is>
       </c>
       <c r="B24">
-        <f>TailRecovery_UP!B5</f>
+        <f>IFERROR(TailRecovery_UP!B5,0)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CloseLotRaw</t>
+          <t>Расчётный лот закрытия</t>
         </is>
       </c>
       <c r="B25">
-        <f>TailRecovery_UP!B9</f>
+        <f>IFERROR(TailRecovery_UP!B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CloseLotRounded</t>
+          <t>Округлённый лот закрытия</t>
         </is>
       </c>
       <c r="B26">
-        <f>TailRecovery_UP!B10</f>
+        <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CloseLotFinal</t>
+          <t>Итоговый лот закрытия</t>
         </is>
       </c>
       <c r="B27">
-        <f>TailRecovery_UP!B10</f>
+        <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TailLotAfter</t>
+          <t>Остаток хвоста</t>
         </is>
       </c>
       <c r="B28">
-        <f>MAX(B22-B27,0)</f>
+        <f>IF(OR(B22="Хвост не найден",NOT(ISNUMBER(B22))),"Хвост не найден",MAX(B22-B27,0))</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RecoveryFundAfter</t>
+          <t>RecoveryFund после закрытия</t>
         </is>
       </c>
       <c r="B29">
-        <f>TailRecovery_UP!B7</f>
+        <f>IFERROR(TailRecovery_UP!B7,0)</f>
         <v/>
       </c>
     </row>
@@ -1266,11 +1279,33 @@
         </is>
       </c>
       <c r="B31">
-        <f>TEXTJOIN(CHAR(10),TRUE,B2,"Current Price: "&amp;TEXT(B3,"0.00000"),"Next trigger level: "&amp;TEXT(B4,"0.00000")&amp;" ("&amp;TEXT(B5,"0")&amp;" points)","Open section: "&amp;B6&amp;" + "&amp;B7,"Section level: "&amp;TEXT(B8,"0"),"CycleProfit: "&amp;TEXT(B17,"0.00"),"Reserve += "&amp;TEXT(B18,"0.00")&amp;"; Recovery += "&amp;TEXT(B19,"0.00"),"Tail: "&amp;B21&amp;" "&amp;TEXT(B22,"0.00")&amp;"; Close "&amp;TEXT(B27,"0.00")&amp;"; Remain "&amp;TEXT(B28,"0.00"),"CanCloseBasket: "&amp;BasketSummary!B10,"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
-        <v/>
-      </c>
-    </row>
+        <f>TEXTJOIN(CHAR(10),TRUE,"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ:",B2,"Если цена дойдет до: "&amp;IF(B4="","уровень не рассчитан",TEXT(B4,"0.00000")),"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5),"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7,"Прибыль цикла: "&amp;TEXT(B17,"0.00")&amp;"; Резерв +"&amp;TEXT(B18,"0.00")&amp;"; RecoveryFund +"&amp;TEXT(B19,"0.00"),"Хвост: "&amp;B21&amp;"; закрыть: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;"; останется: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28),"RecoveryFund после: "&amp;TEXT(B29,"0.00"),"Итоговое действие: "&amp;IF(BasketSummary!B10="YES","BASKET_CLOSE",IF(B12&lt;&gt;"YES","WAIT",IF(B14="YES",IF(B15="YES","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION"))),"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2">
+        <f>B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A32:H45"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1281,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1299,113 +1334,113 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ScenarioTitle</t>
+          <t>Название сценария</t>
         </is>
       </c>
       <c r="B2">
-        <f>"SCENARIO: PRICE MOVES DOWN"</f>
+        <f>"СЦЕНАРИЙ: ЦЕНА ИДЕТ ВНИЗ"</f>
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CurrentPrice</t>
+          <t>Текущая цена</t>
         </is>
       </c>
       <c r="B3">
-        <f>Scenario_DOWN!B4</f>
+        <f>IFERROR(Scenario_DOWN!B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NextTriggerLevel</t>
+          <t>Следующий уровень</t>
         </is>
       </c>
       <c r="B4">
-        <f>SectionCalculator_DOWN!B15</f>
+        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!E9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!E10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!E11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!E12,"")))),"")</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DistancePoints</t>
+          <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
       <c r="B5">
-        <f>ROUND(ABS(B4-B3)*10000,0)</f>
+        <f>IF(OR(B4="",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BigPosition</t>
+          <t>Большая позиция</t>
         </is>
       </c>
       <c r="B6">
-        <f>"SELL "&amp;TEXT(TailRecovery_DOWN!B16,"0.00")</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B16&gt;0,IF("DOWN"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_DOWN!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SmallHedge</t>
+          <t>Малая защитная позиция</t>
         </is>
       </c>
       <c r="B7">
-        <f>"BUY "&amp;TEXT(TailRecovery_DOWN!B17,"0.00")</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B17&gt;0,IF("DOWN"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_DOWN!B17,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SectionLevel</t>
+          <t>Уровень секции</t>
         </is>
       </c>
       <c r="B8">
-        <f>SectionCalculator_DOWN!B16</f>
+        <f>IFERROR(SectionCalculator_DOWN!B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Причина</t>
         </is>
       </c>
       <c r="B9">
-        <f>IF(SectionCalculator_DOWN!B12="YES","Reached level; tail found; risk limits OK","Waiting level/risk gate")</f>
+        <f>IF(SectionCalculator_DOWN!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция сейчас недоступна: уровень/риск-гейт/хвост")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>RiskChecks</t>
+          <t>Проверки риска</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CanOpenSection</t>
+          <t>Можно открыть секцию</t>
         </is>
       </c>
       <c r="B12">
-        <f>SectionCalculator_DOWN!B12</f>
+        <f>SectionCalculator_DOWN!B14</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>NoOppositeCascade</t>
+          <t>Нет встречного каскада</t>
         </is>
       </c>
       <c r="B13">
@@ -1416,7 +1451,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CanCloseSection</t>
+          <t>Можно закрыть секцию</t>
         </is>
       </c>
       <c r="B14">
@@ -1427,7 +1462,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CanCloseTail</t>
+          <t>Можно закрыть хвост</t>
         </is>
       </c>
       <c r="B15">
@@ -1438,132 +1473,132 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CycleProfit</t>
+          <t>Прибыль цикла</t>
         </is>
       </c>
       <c r="B17">
-        <f>SectionCalculator_DOWN!B31</f>
+        <f>IFERROR(SectionCalculator_DOWN!B31,0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ReserveAdd</t>
+          <t>Добавить в резерв</t>
         </is>
       </c>
       <c r="B18">
-        <f>TailRecovery_DOWN!B6</f>
+        <f>IFERROR(TailRecovery_DOWN!B6,0)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RecoveryAdd</t>
+          <t>Добавить в RecoveryFund</t>
         </is>
       </c>
       <c r="B19">
-        <f>TailRecovery_DOWN!B8</f>
+        <f>IFERROR(TailRecovery_DOWN!B8,0)</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DetectedTailType</t>
+          <t>Тип хвоста</t>
         </is>
       </c>
       <c r="B21">
-        <f>TailRecovery_DOWN!B2</f>
+        <f>IF(OR(TailRecovery_DOWN!B2="",TailRecovery_DOWN!B2="N/A"),"Хвост не найден",TailRecovery_DOWN!B2)</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TailLot</t>
+          <t>Лот хвоста</t>
         </is>
       </c>
       <c r="B22">
-        <f>TailRecovery_DOWN!B3</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B3&gt;0,TailRecovery_DOWN!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TailLoss</t>
+          <t>Убыток хвоста</t>
         </is>
       </c>
       <c r="B23">
-        <f>TailRecovery_DOWN!B12</f>
+        <f>IFERROR(TailRecovery_DOWN!B12,0)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RecoveryFundBefore</t>
+          <t>RecoveryFund до закрытия</t>
         </is>
       </c>
       <c r="B24">
-        <f>TailRecovery_DOWN!B5</f>
+        <f>IFERROR(TailRecovery_DOWN!B5,0)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CloseLotRaw</t>
+          <t>Расчётный лот закрытия</t>
         </is>
       </c>
       <c r="B25">
-        <f>TailRecovery_DOWN!B9</f>
+        <f>IFERROR(TailRecovery_DOWN!B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CloseLotRounded</t>
+          <t>Округлённый лот закрытия</t>
         </is>
       </c>
       <c r="B26">
-        <f>TailRecovery_DOWN!B10</f>
+        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CloseLotFinal</t>
+          <t>Итоговый лот закрытия</t>
         </is>
       </c>
       <c r="B27">
-        <f>TailRecovery_DOWN!B10</f>
+        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TailLotAfter</t>
+          <t>Остаток хвоста</t>
         </is>
       </c>
       <c r="B28">
-        <f>MAX(B22-B27,0)</f>
+        <f>IF(OR(B22="Хвост не найден",NOT(ISNUMBER(B22))),"Хвост не найден",MAX(B22-B27,0))</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RecoveryFundAfter</t>
+          <t>RecoveryFund после закрытия</t>
         </is>
       </c>
       <c r="B29">
-        <f>TailRecovery_DOWN!B7</f>
+        <f>IFERROR(TailRecovery_DOWN!B7,0)</f>
         <v/>
       </c>
     </row>
@@ -1574,11 +1609,33 @@
         </is>
       </c>
       <c r="B31">
-        <f>TEXTJOIN(CHAR(10),TRUE,B2,"Current Price: "&amp;TEXT(B3,"0.00000"),"Next trigger level: "&amp;TEXT(B4,"0.00000")&amp;" ("&amp;TEXT(B5,"0")&amp;" points)","Open section: "&amp;B6&amp;" + "&amp;B7,"Section level: "&amp;TEXT(B8,"0"),"CycleProfit: "&amp;TEXT(B17,"0.00"),"Reserve += "&amp;TEXT(B18,"0.00")&amp;"; Recovery += "&amp;TEXT(B19,"0.00"),"Tail: "&amp;B21&amp;" "&amp;TEXT(B22,"0.00")&amp;"; Close "&amp;TEXT(B27,"0.00")&amp;"; Remain "&amp;TEXT(B28,"0.00"),"CanCloseBasket: "&amp;BasketSummary!C10,"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
-        <v/>
-      </c>
-    </row>
+        <f>TEXTJOIN(CHAR(10),TRUE,"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ:",B2,"Если цена дойдет до: "&amp;IF(B4="","уровень не рассчитан",TEXT(B4,"0.00000")),"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5),"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7,"Прибыль цикла: "&amp;TEXT(B17,"0.00")&amp;"; Резерв +"&amp;TEXT(B18,"0.00")&amp;"; RecoveryFund +"&amp;TEXT(B19,"0.00"),"Хвост: "&amp;B21&amp;"; закрыть: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;"; останется: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28),"RecoveryFund после: "&amp;TEXT(B29,"0.00"),"Итоговое действие: "&amp;IF(BasketSummary!C10="YES","BASKET_CLOSE",IF(B12&lt;&gt;"YES","WAIT",IF(B14="YES",IF(B15="YES","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION"))),"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2">
+        <f>B31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
+    <row r="43"/>
+    <row r="44"/>
+    <row r="45"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A32:H45"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Ensure non-empty Russian HumanReadableAction and filled recommendation block
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!E4,IF(SectionCalculator_UP!B4=2,Scenario_UP!E5,IF(SectionCalculator_UP!B4=3,Scenario_UP!E6,IF(SectionCalculator_UP!B4=4,Scenario_UP!E7,"")))),"")</f>
+        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!E4,IF(SectionCalculator_UP!B4=2,Scenario_UP!E5,IF(SectionCalculator_UP!B4=3,Scenario_UP!E6,IF(SectionCalculator_UP!B4=4,Scenario_UP!E7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(B4="",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
+        <f>IF(OR(B4="Уровень не рассчитан",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
         <v/>
       </c>
     </row>
@@ -1103,7 +1103,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>SectionCalculator_UP!B14</f>
+        <f>IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>SectionCalculator_UP!B13</f>
+        <f>IF(SectionCalculator_UP!B13="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>SectionCalculator_UP!B32</f>
+        <f>IF(SectionCalculator_UP!B32="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>TailRecovery_UP!B11</f>
+        <f>IF(TailRecovery_UP!B11="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="B31">
-        <f>TEXTJOIN(CHAR(10),TRUE,"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ:",B2,"Если цена дойдет до: "&amp;IF(B4="","уровень не рассчитан",TEXT(B4,"0.00000")),"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5),"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7,"Прибыль цикла: "&amp;TEXT(B17,"0.00")&amp;"; Резерв +"&amp;TEXT(B18,"0.00")&amp;"; RecoveryFund +"&amp;TEXT(B19,"0.00"),"Хвост: "&amp;B21&amp;"; закрыть: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;"; останется: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28),"RecoveryFund после: "&amp;TEXT(B29,"0.00"),"Итоговое действие: "&amp;IF(BasketSummary!B10="YES","BASKET_CLOSE",IF(B12&lt;&gt;"YES","WAIT",IF(B14="YES",IF(B15="YES","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION"))),"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B4),TEXT(B4,"0.00000"),B4)&amp;"."&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5)&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Проверки: открыть секцию="&amp;B12&amp;", встречный каскад="&amp;B13&amp;", закрыть секцию="&amp;B14&amp;", закрыть хвост="&amp;B15&amp;"."&amp;CHAR(10)&amp;"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7&amp;"."&amp;CHAR(10)&amp;"Хвост: "&amp;B21&amp;". Лот хвоста: "&amp;IF(ISNUMBER(B22),TEXT(B22,"0.00"),B22)&amp;"."&amp;CHAR(10)&amp;"Рекомендованный лот закрытия: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;". Остаток хвоста: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28)&amp;"."&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B29,"0.00")&amp;". Резерв после: "&amp;TEXT(B18,"0.00")&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Итоговое действие: "&amp;IF(BasketSummary!B10="YES","BASKET_CLOSE",IF(B12="НЕТ","WAIT",IF(B14="ДА",IF(B15="ДА","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION")))&amp;" / "&amp;IF(OR(B12="НЕТ",B13="НЕТ"),"SAFE","NORMAL")</f>
         <v/>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!E9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!E10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!E11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!E12,"")))),"")</f>
+        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!E9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!E10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!E11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!E12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(B4="",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
+        <f>IF(OR(B4="Уровень не рассчитан",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
         <v/>
       </c>
     </row>
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>SectionCalculator_DOWN!B14</f>
+        <f>IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
         </is>
       </c>
       <c r="B13">
-        <f>SectionCalculator_DOWN!B13</f>
+        <f>IF(SectionCalculator_DOWN!B13="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>SectionCalculator_DOWN!B32</f>
+        <f>IF(SectionCalculator_DOWN!B32="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1466,7 +1466,7 @@
         </is>
       </c>
       <c r="B15">
-        <f>TailRecovery_DOWN!B11</f>
+        <f>IF(TailRecovery_DOWN!B11="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
         </is>
       </c>
       <c r="B31">
-        <f>TEXTJOIN(CHAR(10),TRUE,"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ:",B2,"Если цена дойдет до: "&amp;IF(B4="","уровень не рассчитан",TEXT(B4,"0.00000")),"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5),"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7,"Прибыль цикла: "&amp;TEXT(B17,"0.00")&amp;"; Резерв +"&amp;TEXT(B18,"0.00")&amp;"; RecoveryFund +"&amp;TEXT(B19,"0.00"),"Хвост: "&amp;B21&amp;"; закрыть: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;"; останется: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28),"RecoveryFund после: "&amp;TEXT(B29,"0.00"),"Итоговое действие: "&amp;IF(BasketSummary!C10="YES","BASKET_CLOSE",IF(B12&lt;&gt;"YES","WAIT",IF(B14="YES",IF(B15="YES","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION"))),"SAFE: "&amp;IF(OR(B12&lt;&gt;"YES",B13&lt;&gt;"YES"),"YES","NO"))</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B4),TEXT(B4,"0.00000"),B4)&amp;"."&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5)&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Проверки: открыть секцию="&amp;B12&amp;", встречный каскад="&amp;B13&amp;", закрыть секцию="&amp;B14&amp;", закрыть хвост="&amp;B15&amp;"."&amp;CHAR(10)&amp;"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7&amp;"."&amp;CHAR(10)&amp;"Хвост: "&amp;B21&amp;". Лот хвоста: "&amp;IF(ISNUMBER(B22),TEXT(B22,"0.00"),B22)&amp;"."&amp;CHAR(10)&amp;"Рекомендованный лот закрытия: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;". Остаток хвоста: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28)&amp;"."&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B29,"0.00")&amp;". Резерв после: "&amp;TEXT(B18,"0.00")&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Итоговое действие: "&amp;IF(BasketSummary!C10="YES","BASKET_CLOSE",IF(B12="НЕТ","WAIT",IF(B14="ДА",IF(B15="ДА","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION")))&amp;" / "&amp;IF(OR(B12="НЕТ",B13="НЕТ"),"SAFE","NORMAL")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix RU scenario text outputs and guarantee non-empty recommendation blocks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -986,7 +986,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1019,256 +1019,256 @@
         </is>
       </c>
       <c r="B3">
-        <f>IFERROR(Scenario_UP!B4,0)</f>
+        <f>IFERROR(CurrentPositions!F2,0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Следующий уровень</t>
+          <t>Сценарная цена</t>
         </is>
       </c>
       <c r="B4">
-        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!E4,IF(SectionCalculator_UP!B4=2,Scenario_UP!E5,IF(SectionCalculator_UP!B4=3,Scenario_UP!E6,IF(SectionCalculator_UP!B4=4,Scenario_UP!E7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
+        <f>IFERROR(Scenario_UP!B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Расстояние до уровня, пунктов</t>
+          <t>Следующий уровень открытия</t>
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(B4="Уровень не рассчитан",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
+        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!E4,IF(SectionCalculator_UP!B4=2,Scenario_UP!E5,IF(SectionCalculator_UP!B4=3,Scenario_UP!E6,IF(SectionCalculator_UP!B4=4,Scenario_UP!E7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Большая позиция</t>
+          <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
       <c r="B6">
-        <f>IFERROR(IF(TailRecovery_UP!B16&gt;0,IF("UP"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_UP!B16,"0.00"),"Не открывать"),"Не открывать")</f>
+        <f>IF(OR(B5="Уровень не рассчитан",B4=""),"Расстояние не рассчитано",ROUND(ABS(B5-B4)*10000,0))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Малая защитная позиция</t>
+          <t>Большая позиция</t>
         </is>
       </c>
       <c r="B7">
-        <f>IFERROR(IF(TailRecovery_UP!B17&gt;0,IF("UP"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_UP!B17,"0.00"),"Не открывать"),"Не открывать")</f>
+        <f>IFERROR(IF(TailRecovery_UP!B16&gt;0,IF("UP"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_UP!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Уровень секции</t>
+          <t>Малая защитная позиция</t>
         </is>
       </c>
       <c r="B8">
-        <f>IFERROR(SectionCalculator_UP!B4,0)</f>
+        <f>IFERROR(IF(TailRecovery_UP!B17&gt;0,IF("UP"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_UP!B17,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Уровень секции</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IFERROR(SectionCalculator_UP!B4,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Причина</t>
         </is>
       </c>
-      <c r="B9">
-        <f>IF(SectionCalculator_UP!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция сейчас недоступна: уровень/риск-гейт/хвост")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Проверки риска</t>
-        </is>
+      <c r="B10">
+        <f>IF(SectionCalculator_UP!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция недоступна: уровень/риск-гейт/хвост")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Можно открыть секцию</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")</f>
-        <v/>
+          <t>Проверки риска</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Нет встречного каскада</t>
+          <t>Можно открыть секцию</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(SectionCalculator_UP!B13="YES","ДА","НЕТ")</f>
+        <f>IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Можно закрыть секцию</t>
+          <t>Нет встречного каскада</t>
         </is>
       </c>
       <c r="B14">
-        <f>IF(SectionCalculator_UP!B32="YES","ДА","НЕТ")</f>
+        <f>IF(SectionCalculator_UP!B13="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Можно закрыть секцию</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(SectionCalculator_UP!B32="YES","ДА","НЕТ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Можно закрыть хвост</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B16">
         <f>IF(TailRecovery_UP!B11="YES","ДА","НЕТ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Прибыль цикла</t>
-        </is>
-      </c>
-      <c r="B17">
-        <f>IFERROR(SectionCalculator_UP!B31,0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Добавить в резерв</t>
+          <t>Прибыль цикла</t>
         </is>
       </c>
       <c r="B18">
-        <f>IFERROR(TailRecovery_UP!B6,0)</f>
+        <f>IFERROR(SectionCalculator_UP!B31,0)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Добавить в резерв</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>IFERROR(TailRecovery_UP!B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Добавить в RecoveryFund</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B20">
         <f>IFERROR(TailRecovery_UP!B8,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Тип хвоста</t>
-        </is>
-      </c>
-      <c r="B21">
-        <f>IF(OR(TailRecovery_UP!B2="",TailRecovery_UP!B2="N/A"),"Хвост не найден",TailRecovery_UP!B2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Лот хвоста</t>
-        </is>
-      </c>
-      <c r="B22">
-        <f>IFERROR(IF(TailRecovery_UP!B3&gt;0,TailRecovery_UP!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Убыток хвоста</t>
+          <t>Тип хвоста</t>
         </is>
       </c>
       <c r="B23">
-        <f>IFERROR(TailRecovery_UP!B12,0)</f>
+        <f>IF(OR(TailRecovery_UP!B2="",TailRecovery_UP!B2="N/A"),"Хвост не найден",TailRecovery_UP!B2)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RecoveryFund до закрытия</t>
+          <t>Лот хвоста</t>
         </is>
       </c>
       <c r="B24">
-        <f>IFERROR(TailRecovery_UP!B5,0)</f>
+        <f>IFERROR(IF(TailRecovery_UP!B3&gt;0,TailRecovery_UP!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Расчётный лот закрытия</t>
+          <t>Убыток хвоста</t>
         </is>
       </c>
       <c r="B25">
-        <f>IFERROR(TailRecovery_UP!B9,0)</f>
+        <f>IFERROR(TailRecovery_UP!B12,0)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Округлённый лот закрытия</t>
+          <t>RecoveryFund до закрытия</t>
         </is>
       </c>
       <c r="B26">
-        <f>IFERROR(TailRecovery_UP!B10,0)</f>
+        <f>IFERROR(TailRecovery_UP!B5,0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Итоговый лот закрытия</t>
+          <t>Расчётный лот закрытия</t>
         </is>
       </c>
       <c r="B27">
-        <f>IFERROR(TailRecovery_UP!B10,0)</f>
+        <f>IFERROR(TailRecovery_UP!B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Остаток хвоста</t>
+          <t>Округлённый лот закрытия</t>
         </is>
       </c>
       <c r="B28">
-        <f>IF(OR(B22="Хвост не найден",NOT(ISNUMBER(B22))),"Хвост не найден",MAX(B22-B27,0))</f>
+        <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RecoveryFund после закрытия</t>
+          <t>Итоговый лот закрытия</t>
         </is>
       </c>
       <c r="B29">
-        <f>IFERROR(TailRecovery_UP!B7,0)</f>
+        <f>IFERROR(TailRecovery_UP!B10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Остаток хвоста</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>IF(OR(B24="Хвост не найден",NOT(ISNUMBER(B24))),"Хвост не найден",MAX(B24-B29,0))</f>
         <v/>
       </c>
     </row>
@@ -1279,13 +1279,13 @@
         </is>
       </c>
       <c r="B31">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B4),TEXT(B4,"0.00000"),B4)&amp;"."&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5)&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Проверки: открыть секцию="&amp;B12&amp;", встречный каскад="&amp;B13&amp;", закрыть секцию="&amp;B14&amp;", закрыть хвост="&amp;B15&amp;"."&amp;CHAR(10)&amp;"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7&amp;"."&amp;CHAR(10)&amp;"Хвост: "&amp;B21&amp;". Лот хвоста: "&amp;IF(ISNUMBER(B22),TEXT(B22,"0.00"),B22)&amp;"."&amp;CHAR(10)&amp;"Рекомендованный лот закрытия: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;". Остаток хвоста: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28)&amp;"."&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B29,"0.00")&amp;". Резерв после: "&amp;TEXT(B18,"0.00")&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Итоговое действие: "&amp;IF(BasketSummary!B10="YES","BASKET_CLOSE",IF(B12="НЕТ","WAIT",IF(B14="ДА",IF(B15="ДА","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION")))&amp;" / "&amp;IF(OR(B12="НЕТ",B13="НЕТ"),"SAFE","NORMAL")</f>
+        <f>IF(B13="ДА","ОТКРЫТЬ СЕКЦИЮ",IF(B15="ДА",IF(B16="ДА","ЗАКРЫТЬ СЕКЦИЮ + ЗАКРЫТЬ ХВОСТ","ЗАКРЫТЬ СЕКЦИЮ"),"ЖДАТЬ / НИЧЕГО НЕ ДЕЛАТЬ"))</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <f>B31</f>
+        <f>B46</f>
         <v/>
       </c>
     </row>
@@ -1302,6 +1302,12 @@
     <row r="43"/>
     <row r="44"/>
     <row r="45"/>
+    <row r="46">
+      <c r="B46">
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A32:H45"/>
@@ -1316,7 +1322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1349,256 +1355,256 @@
         </is>
       </c>
       <c r="B3">
-        <f>IFERROR(Scenario_DOWN!B4,0)</f>
+        <f>IFERROR(CurrentPositions!F2,0)</f>
         <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Следующий уровень</t>
+          <t>Сценарная цена</t>
         </is>
       </c>
       <c r="B4">
-        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!E9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!E10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!E11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!E12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
+        <f>IFERROR(Scenario_DOWN!B4,0)</f>
         <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Расстояние до уровня, пунктов</t>
+          <t>Следующий уровень открытия</t>
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(B4="Уровень не рассчитан",B3=""),"Уровень не рассчитан",ROUND(ABS(B4-B3)*10000,0))</f>
+        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!E9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!E10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!E11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!E12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Большая позиция</t>
+          <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
       <c r="B6">
-        <f>IFERROR(IF(TailRecovery_DOWN!B16&gt;0,IF("DOWN"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_DOWN!B16,"0.00"),"Не открывать"),"Не открывать")</f>
+        <f>IF(OR(B5="Уровень не рассчитан",B4=""),"Расстояние не рассчитано",ROUND(ABS(B5-B4)*10000,0))</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Малая защитная позиция</t>
+          <t>Большая позиция</t>
         </is>
       </c>
       <c r="B7">
-        <f>IFERROR(IF(TailRecovery_DOWN!B17&gt;0,IF("DOWN"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_DOWN!B17,"0.00"),"Не открывать"),"Не открывать")</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B16&gt;0,IF("DOWN"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_DOWN!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Уровень секции</t>
+          <t>Малая защитная позиция</t>
         </is>
       </c>
       <c r="B8">
-        <f>IFERROR(SectionCalculator_DOWN!B4,0)</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B17&gt;0,IF("DOWN"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_DOWN!B17,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Уровень секции</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IFERROR(SectionCalculator_DOWN!B4,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Причина</t>
         </is>
       </c>
-      <c r="B9">
-        <f>IF(SectionCalculator_DOWN!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция сейчас недоступна: уровень/риск-гейт/хвост")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Проверки риска</t>
-        </is>
+      <c r="B10">
+        <f>IF(SectionCalculator_DOWN!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция недоступна: уровень/риск-гейт/хвост")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Можно открыть секцию</t>
-        </is>
-      </c>
-      <c r="B12">
-        <f>IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")</f>
-        <v/>
+          <t>Проверки риска</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Нет встречного каскада</t>
+          <t>Можно открыть секцию</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(SectionCalculator_DOWN!B13="YES","ДА","НЕТ")</f>
+        <f>IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Можно закрыть секцию</t>
+          <t>Нет встречного каскада</t>
         </is>
       </c>
       <c r="B14">
-        <f>IF(SectionCalculator_DOWN!B32="YES","ДА","НЕТ")</f>
+        <f>IF(SectionCalculator_DOWN!B13="YES","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Можно закрыть секцию</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(SectionCalculator_DOWN!B32="YES","ДА","НЕТ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Можно закрыть хвост</t>
         </is>
       </c>
-      <c r="B15">
+      <c r="B16">
         <f>IF(TailRecovery_DOWN!B11="YES","ДА","НЕТ")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Прибыль цикла</t>
-        </is>
-      </c>
-      <c r="B17">
-        <f>IFERROR(SectionCalculator_DOWN!B31,0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Добавить в резерв</t>
+          <t>Прибыль цикла</t>
         </is>
       </c>
       <c r="B18">
-        <f>IFERROR(TailRecovery_DOWN!B6,0)</f>
+        <f>IFERROR(SectionCalculator_DOWN!B31,0)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Добавить в резерв</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>IFERROR(TailRecovery_DOWN!B6,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Добавить в RecoveryFund</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B20">
         <f>IFERROR(TailRecovery_DOWN!B8,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Тип хвоста</t>
-        </is>
-      </c>
-      <c r="B21">
-        <f>IF(OR(TailRecovery_DOWN!B2="",TailRecovery_DOWN!B2="N/A"),"Хвост не найден",TailRecovery_DOWN!B2)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Лот хвоста</t>
-        </is>
-      </c>
-      <c r="B22">
-        <f>IFERROR(IF(TailRecovery_DOWN!B3&gt;0,TailRecovery_DOWN!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Убыток хвоста</t>
+          <t>Тип хвоста</t>
         </is>
       </c>
       <c r="B23">
-        <f>IFERROR(TailRecovery_DOWN!B12,0)</f>
+        <f>IF(OR(TailRecovery_DOWN!B2="",TailRecovery_DOWN!B2="N/A"),"Хвост не найден",TailRecovery_DOWN!B2)</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RecoveryFund до закрытия</t>
+          <t>Лот хвоста</t>
         </is>
       </c>
       <c r="B24">
-        <f>IFERROR(TailRecovery_DOWN!B5,0)</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B3&gt;0,TailRecovery_DOWN!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Расчётный лот закрытия</t>
+          <t>Убыток хвоста</t>
         </is>
       </c>
       <c r="B25">
-        <f>IFERROR(TailRecovery_DOWN!B9,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B12,0)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Округлённый лот закрытия</t>
+          <t>RecoveryFund до закрытия</t>
         </is>
       </c>
       <c r="B26">
-        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B5,0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Итоговый лот закрытия</t>
+          <t>Расчётный лот закрытия</t>
         </is>
       </c>
       <c r="B27">
-        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Остаток хвоста</t>
+          <t>Округлённый лот закрытия</t>
         </is>
       </c>
       <c r="B28">
-        <f>IF(OR(B22="Хвост не найден",NOT(ISNUMBER(B22))),"Хвост не найден",MAX(B22-B27,0))</f>
+        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RecoveryFund после закрытия</t>
+          <t>Итоговый лот закрытия</t>
         </is>
       </c>
       <c r="B29">
-        <f>IFERROR(TailRecovery_DOWN!B7,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Остаток хвоста</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>IF(OR(B24="Хвост не найден",NOT(ISNUMBER(B24))),"Хвост не найден",MAX(B24-B29,0))</f>
         <v/>
       </c>
     </row>
@@ -1609,13 +1615,13 @@
         </is>
       </c>
       <c r="B31">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B4),TEXT(B4,"0.00000"),B4)&amp;"."&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0")&amp;" пунктов",B5)&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Проверки: открыть секцию="&amp;B12&amp;", встречный каскад="&amp;B13&amp;", закрыть секцию="&amp;B14&amp;", закрыть хвост="&amp;B15&amp;"."&amp;CHAR(10)&amp;"Рекомендация по открытию: "&amp;B6&amp;" и "&amp;B7&amp;"."&amp;CHAR(10)&amp;"Хвост: "&amp;B21&amp;". Лот хвоста: "&amp;IF(ISNUMBER(B22),TEXT(B22,"0.00"),B22)&amp;"."&amp;CHAR(10)&amp;"Рекомендованный лот закрытия: "&amp;IF(ISNUMBER(B27),TEXT(B27,"0.00"),"0.00")&amp;". Остаток хвоста: "&amp;IF(ISNUMBER(B28),TEXT(B28,"0.00"),B28)&amp;"."&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B29,"0.00")&amp;". Резерв после: "&amp;TEXT(B18,"0.00")&amp;"."&amp;CHAR(10)&amp;CHAR(10)&amp;"Итоговое действие: "&amp;IF(BasketSummary!C10="YES","BASKET_CLOSE",IF(B12="НЕТ","WAIT",IF(B14="ДА",IF(B15="ДА","CLOSE_SECTION+CLOSE_TAIL","CLOSE_SECTION"),"OPEN_SECTION")))&amp;" / "&amp;IF(OR(B12="НЕТ",B13="НЕТ"),"SAFE","NORMAL")</f>
+        <f>IF(B13="ДА","ОТКРЫТЬ СЕКЦИЮ",IF(B15="ДА",IF(B16="ДА","ЗАКРЫТЬ СЕКЦИЮ + ЗАКРЫТЬ ХВОСТ","ЗАКРЫТЬ СЕКЦИЮ"),"ЖДАТЬ / НИЧЕГО НЕ ДЕЛАТЬ"))</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <f>B31</f>
+        <f>B46</f>
         <v/>
       </c>
     </row>
@@ -1632,6 +1638,12 @@
     <row r="43"/>
     <row r="44"/>
     <row r="45"/>
+    <row r="46">
+      <c r="B46">
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A32:H45"/>

</xml_diff>

<commit_message>
Restore workbook calculation sync and robust RU scenario recommendations
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -785,11 +785,11 @@
         </is>
       </c>
       <c r="B5">
-        <f>IF(OR(SectionCalculator_UP!B14="NO",SectionCalculator_UP!B12="YES"),"OK","ERROR")</f>
+        <f>IF(SectionCalculator_UP!B12="YES","OK",IF(SectionCalculator_UP!B14="NO","BLOCKED","ERROR"))</f>
         <v/>
       </c>
       <c r="C5">
-        <f>IF(OR(SectionCalculator_DOWN!B14="NO",SectionCalculator_DOWN!B12="YES"),"OK","ERROR")</f>
+        <f>IF(SectionCalculator_DOWN!B12="YES","OK",IF(SectionCalculator_DOWN!B14="NO","BLOCKED","ERROR"))</f>
         <v/>
       </c>
     </row>
@@ -800,11 +800,11 @@
         </is>
       </c>
       <c r="B6">
-        <f>IF(SectionCalculator_UP!B13="YES","OK","ERROR")</f>
+        <f>IF(SectionCalculator_UP!B13="YES","OK","BLOCKED")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>IF(SectionCalculator_DOWN!B13="YES","OK","ERROR")</f>
+        <f>IF(SectionCalculator_DOWN!B13="YES","OK","BLOCKED")</f>
         <v/>
       </c>
     </row>
@@ -895,31 +895,31 @@
         </is>
       </c>
       <c r="D2">
-        <f>BasketSummary!B13</f>
+        <f>IF(BasketSummary!B13="WAIT","ЖДАТЬ",IF(BasketSummary!B13="SAFE","SAFE",IF(BasketSummary!B13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(AND(TailRecovery_UP!B10&gt;0,TailRecovery_UP!B10&lt;TailRecovery_UP!B3),"ЗАКРЫТЬ ХВОСТ ЧАСТИЧНО","ЗАКРЫТЬ СЕКЦИЮ"))))</f>
         <v/>
       </c>
       <c r="E2">
-        <f>TailRecovery_UP!B3</f>
+        <f>IFERROR(TailRecovery_UP!B3,0)</f>
         <v/>
       </c>
       <c r="F2">
-        <f>TailRecovery_UP!B10</f>
+        <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
       <c r="G2">
-        <f>MAX(E2-F2,0)</f>
+        <f>IF(OR(NOT(ISNUMBER(E2)),NOT(ISNUMBER(F2))),"Хвост не найден",MAX(E2-F2,0))</f>
         <v/>
       </c>
       <c r="H2">
-        <f>TailRecovery_UP!B5</f>
+        <f>IFERROR(TailRecovery_UP!B5,0)</f>
         <v/>
       </c>
       <c r="I2">
-        <f>TailRecovery_UP!B7</f>
+        <f>IFERROR(TailRecovery_UP!B7,0)</f>
         <v/>
       </c>
       <c r="J2">
-        <f>SectionCalculator_UP!B35</f>
+        <f>IFERROR(SectionCalculator_UP!B35,0)</f>
         <v/>
       </c>
       <c r="K2">
@@ -943,31 +943,31 @@
         </is>
       </c>
       <c r="D3">
-        <f>BasketSummary!C13</f>
+        <f>IF(BasketSummary!C13="WAIT","ЖДАТЬ",IF(BasketSummary!C13="SAFE","SAFE",IF(BasketSummary!C13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(AND(TailRecovery_DOWN!B10&gt;0,TailRecovery_DOWN!B10&lt;TailRecovery_DOWN!B3),"ЗАКРЫТЬ ХВОСТ ЧАСТИЧНО","ЗАКРЫТЬ СЕКЦИЮ"))))</f>
         <v/>
       </c>
       <c r="E3">
-        <f>TailRecovery_DOWN!B3</f>
+        <f>IFERROR(TailRecovery_DOWN!B3,0)</f>
         <v/>
       </c>
       <c r="F3">
-        <f>TailRecovery_DOWN!B10</f>
+        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
       <c r="G3">
-        <f>MAX(E3-F3,0)</f>
+        <f>IF(OR(NOT(ISNUMBER(E3)),NOT(ISNUMBER(F3))),"Хвост не найден",MAX(E3-F3,0))</f>
         <v/>
       </c>
       <c r="H3">
-        <f>TailRecovery_DOWN!B5</f>
+        <f>IFERROR(TailRecovery_DOWN!B5,0)</f>
         <v/>
       </c>
       <c r="I3">
-        <f>TailRecovery_DOWN!B7</f>
+        <f>IFERROR(TailRecovery_DOWN!B7,0)</f>
         <v/>
       </c>
       <c r="J3">
-        <f>SectionCalculator_DOWN!B35</f>
+        <f>IFERROR(SectionCalculator_DOWN!B35,0)</f>
         <v/>
       </c>
       <c r="K3">
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="E1">
-        <f>IFERROR(SUMPRODUCT((B7:B206="BUY")*E7:E206*D7:D206)/SUMIFS(D7:D206,B7:B206,"BUY"),0)</f>
+        <f>IFERROR(SUMPRODUCT((B7:B206="BUY")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"BUY")),0)</f>
         <v/>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
         </is>
       </c>
       <c r="E2">
-        <f>IFERROR(SUMPRODUCT((B7:B206="SELL")*E7:E206*D7:D206)/SUMIFS(D7:D206,B7:B206,"SELL"),0)</f>
+        <f>IFERROR(SUMPRODUCT((B7:B206="SELL")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"SELL")),0)</f>
         <v/>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="E4">
-        <f>E3+1*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
         </is>
       </c>
       <c r="E5">
-        <f>E3+2*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <f>E3+3*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+3*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -2048,7 +2048,7 @@
         </is>
       </c>
       <c r="E7">
-        <f>E3+4*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F7">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="E9">
-        <f>E3-1*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F9">
@@ -2176,7 +2176,7 @@
         </is>
       </c>
       <c r="E10">
-        <f>E3-2*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F10">
@@ -2219,7 +2219,7 @@
         </is>
       </c>
       <c r="E11">
-        <f>E3-3*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-3*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F11">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="E12">
-        <f>E3-4*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F12">
@@ -10532,7 +10532,7 @@
         </is>
       </c>
       <c r="E1">
-        <f>IFERROR(SUMPRODUCT((B7:B206="BUY")*E7:E206*D7:D206)/SUMIFS(D7:D206,B7:B206,"BUY"),0)</f>
+        <f>IFERROR(SUMPRODUCT((B7:B206="BUY")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"BUY")),0)</f>
         <v/>
       </c>
     </row>
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="E2">
-        <f>IFERROR(SUMPRODUCT((B7:B206="SELL")*E7:E206*D7:D206)/SUMIFS(D7:D206,B7:B206,"SELL"),0)</f>
+        <f>IFERROR(SUMPRODUCT((B7:B206="SELL")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"SELL")),0)</f>
         <v/>
       </c>
     </row>
@@ -10591,7 +10591,7 @@
         </is>
       </c>
       <c r="E4">
-        <f>E3+1*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10602,7 +10602,7 @@
         </is>
       </c>
       <c r="E5">
-        <f>E3+2*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10628,7 +10628,7 @@
         </is>
       </c>
       <c r="E6" s="1">
-        <f>E3+3*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+3*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F6" s="1" t="inlineStr">
@@ -10676,7 +10676,7 @@
         </is>
       </c>
       <c r="E7">
-        <f>E3+4*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3+4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F7">
@@ -10761,7 +10761,7 @@
         </is>
       </c>
       <c r="E9">
-        <f>E3-1*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F9">
@@ -10804,7 +10804,7 @@
         </is>
       </c>
       <c r="E10">
-        <f>E3-2*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F10">
@@ -10847,7 +10847,7 @@
         </is>
       </c>
       <c r="E11">
-        <f>E3-3*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-3*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F11">
@@ -10890,7 +10890,7 @@
         </is>
       </c>
       <c r="E12">
-        <f>E3-4*Settings!$B$5*Settings!$B$3</f>
+        <f>IF(E3=0,"Уровень не рассчитан",E3-4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
       <c r="F12">
@@ -19216,7 +19216,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>FLOOR(B3*B5,Settings!$B$7)</f>
+        <f>IF(B3&lt;=0,0,FLOOR(B3*B5,Settings!$B$7))</f>
         <v/>
       </c>
     </row>
@@ -19227,7 +19227,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>FLOOR(B3*B6,Settings!$B$7)</f>
+        <f>IF(B3&lt;=0,0,FLOOR(B3*B6,Settings!$B$7))</f>
         <v/>
       </c>
     </row>
@@ -19293,7 +19293,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES",B13="YES"),"YES","NO")</f>
+        <f>IF(B3&lt;=0,"NO",IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES",B13="YES"),"YES","NO"))</f>
         <v/>
       </c>
     </row>
@@ -19853,7 +19853,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>FLOOR(B3*B5,Settings!$B$7)</f>
+        <f>IF(B3&lt;=0,0,FLOOR(B3*B5,Settings!$B$7))</f>
         <v/>
       </c>
     </row>
@@ -19864,7 +19864,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>FLOOR(B3*B6,Settings!$B$7)</f>
+        <f>IF(B3&lt;=0,0,FLOOR(B3*B6,Settings!$B$7))</f>
         <v/>
       </c>
     </row>
@@ -19930,7 +19930,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES",B13="YES"),"YES","NO")</f>
+        <f>IF(B3&lt;=0,"NO",IF(AND(B7&gt;=Settings!$B$6,B8&gt;=Settings!$B$6,B8&lt;B7,B7&lt;=B3,B9&lt;Settings!$B$8,B10&lt;=Settings!$B$15,B11&lt;=Settings!$B$16,B12="YES",B13="YES"),"YES","NO"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor scenario architecture, add workbook validator, and regenerate synced workbooks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -20,6 +20,7 @@
     <sheet name="Log" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="ScenarioText_UP" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="ScenarioText_DOWN" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="FormulaDependencyMap" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1041,7 +1042,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!E4,IF(SectionCalculator_UP!B4=2,Scenario_UP!E5,IF(SectionCalculator_UP!B4=3,Scenario_UP!E6,IF(SectionCalculator_UP!B4=4,Scenario_UP!E7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
+        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!N4,IF(SectionCalculator_UP!B4=2,Scenario_UP!N5,IF(SectionCalculator_UP!B4=3,Scenario_UP!N6,IF(SectionCalculator_UP!B4=4,Scenario_UP!N7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
@@ -1377,7 +1378,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!E9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!E10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!E11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!E12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
+        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!N9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!N10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!N11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!N12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
@@ -1652,6 +1653,105 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Cell</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>DependsOn</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>UsedBy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B4</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>Scenario_UP!B2+Scenario_UP!B3*Settings!B3</f>
+        <v/>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B2, Scenario_UP!B3, Settings!B3</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B12, ScenarioText_UP!B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Scenario_DOWN!B4</t>
+        </is>
+      </c>
+      <c r="B3">
+        <f>Scenario_DOWN!B2-Scenario_DOWN!B3*Settings!B3</f>
+        <v/>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Scenario_DOWN!B2, Scenario_DOWN!B3, Settings!B3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SectionCalculator_DOWN!B12, ScenarioText_DOWN!B4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TailRecovery_UP!B10</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>IF(B6="YES",MIN(B9,B4),0)</f>
+        <v/>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TailRecovery_UP!B9, TailRecovery_UP!B4, TailRecovery_UP!B6</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>BasketSummary!B7, Log!F2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1884,7 +1984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J225"/>
+  <dimension ref="A1:N225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1898,12 +1998,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>AverageBuyPrice</t>
         </is>
       </c>
-      <c r="E1">
+      <c r="N1">
         <f>IFERROR(SUMPRODUCT((B7:B206="BUY")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"BUY")),0)</f>
         <v/>
       </c>
@@ -1918,12 +2018,12 @@
         <f>CurrentPositions!F2</f>
         <v/>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>AverageSellPrice</t>
         </is>
       </c>
-      <c r="E2">
+      <c r="N2">
         <f>IFERROR(SUMPRODUCT((B7:B206="SELL")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"SELL")),0)</f>
         <v/>
       </c>
@@ -1937,13 +2037,13 @@
       <c r="B3" t="n">
         <v>100</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Center</t>
         </is>
       </c>
-      <c r="E3">
-        <f>(E1+E2)/2</f>
+      <c r="N3">
+        <f>(N1+N2)/2</f>
         <v/>
       </c>
     </row>
@@ -1957,24 +2057,24 @@
         <f>B2+B3*Settings!$B$3</f>
         <v/>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>UpperLevel1</t>
         </is>
       </c>
-      <c r="E4">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+1*Settings!$B$5*Settings!$B$3)</f>
+      <c r="N4">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="D5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>UpperLevel2</t>
         </is>
       </c>
-      <c r="E5">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+2*Settings!$B$5*Settings!$B$3)</f>
+      <c r="N5">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -1996,37 +2096,47 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>OpenPrice</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>ScenarioPrice</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>ScenarioPointsPnL</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>ScenarioMoneyPnL</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>IsTail</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>SectionID</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>UpperLevel3</t>
         </is>
       </c>
-      <c r="E6" s="1">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+3*Settings!$B$5*Settings!$B$3)</f>
-        <v/>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>ScenarioPrice</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="inlineStr">
-        <is>
-          <t>ScenarioPointsPnL</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>ScenarioMoneyPnL</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="inlineStr">
-        <is>
-          <t>IsTail</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>SectionID</t>
-        </is>
+      <c r="N6">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+3*Settings!$B$5*Settings!$B$3)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -2042,13 +2152,12 @@
         <f>CurrentPositions!C2</f>
         <v/>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>UpperLevel4</t>
-        </is>
+      <c r="D7">
+        <f>CurrentPositions!D2</f>
+        <v/>
       </c>
       <c r="E7">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+4*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E2</f>
         <v/>
       </c>
       <c r="F7">
@@ -2069,6 +2178,15 @@
       </c>
       <c r="J7">
         <f>CurrentPositions!J2</f>
+        <v/>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>UpperLevel4</t>
+        </is>
+      </c>
+      <c r="N7">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -2127,13 +2245,12 @@
         <f>CurrentPositions!C4</f>
         <v/>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>LowerLevel1</t>
-        </is>
+      <c r="D9">
+        <f>CurrentPositions!D4</f>
+        <v/>
       </c>
       <c r="E9">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-1*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E4</f>
         <v/>
       </c>
       <c r="F9">
@@ -2154,6 +2271,15 @@
       </c>
       <c r="J9">
         <f>CurrentPositions!J4</f>
+        <v/>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>LowerLevel1</t>
+        </is>
+      </c>
+      <c r="N9">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -2170,13 +2296,12 @@
         <f>CurrentPositions!C5</f>
         <v/>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LowerLevel2</t>
-        </is>
+      <c r="D10">
+        <f>CurrentPositions!D5</f>
+        <v/>
       </c>
       <c r="E10">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-2*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E5</f>
         <v/>
       </c>
       <c r="F10">
@@ -2197,6 +2322,15 @@
       </c>
       <c r="J10">
         <f>CurrentPositions!J5</f>
+        <v/>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>LowerLevel2</t>
+        </is>
+      </c>
+      <c r="N10">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -2213,13 +2347,12 @@
         <f>CurrentPositions!C6</f>
         <v/>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>LowerLevel3</t>
-        </is>
+      <c r="D11">
+        <f>CurrentPositions!D6</f>
+        <v/>
       </c>
       <c r="E11">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-3*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E6</f>
         <v/>
       </c>
       <c r="F11">
@@ -2240,6 +2373,15 @@
       </c>
       <c r="J11">
         <f>CurrentPositions!J6</f>
+        <v/>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>LowerLevel3</t>
+        </is>
+      </c>
+      <c r="N11">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-3*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -2256,13 +2398,12 @@
         <f>CurrentPositions!C7</f>
         <v/>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>LowerLevel4</t>
-        </is>
+      <c r="D12">
+        <f>CurrentPositions!D7</f>
+        <v/>
       </c>
       <c r="E12">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-4*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E7</f>
         <v/>
       </c>
       <c r="F12">
@@ -2283,6 +2424,15 @@
       </c>
       <c r="J12">
         <f>CurrentPositions!J7</f>
+        <v/>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>LowerLevel4</t>
+        </is>
+      </c>
+      <c r="N12">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10512,7 +10662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J225"/>
+  <dimension ref="A1:N225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10526,12 +10676,12 @@
           <t>Value</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>AverageBuyPrice</t>
         </is>
       </c>
-      <c r="E1">
+      <c r="N1">
         <f>IFERROR(SUMPRODUCT((B7:B206="BUY")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"BUY")),0)</f>
         <v/>
       </c>
@@ -10546,12 +10696,12 @@
         <f>CurrentPositions!F2</f>
         <v/>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>AverageSellPrice</t>
         </is>
       </c>
-      <c r="E2">
+      <c r="N2">
         <f>IFERROR(SUMPRODUCT((B7:B206="SELL")*E7:E206*D7:D206)/MAX(0.0000001,SUMIFS(D7:D206,B7:B206,"SELL")),0)</f>
         <v/>
       </c>
@@ -10565,13 +10715,13 @@
       <c r="B3" t="n">
         <v>100</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Center</t>
         </is>
       </c>
-      <c r="E3">
-        <f>(E1+E2)/2</f>
+      <c r="N3">
+        <f>(N1+N2)/2</f>
         <v/>
       </c>
     </row>
@@ -10585,24 +10735,24 @@
         <f>B2-B3*Settings!$B$3</f>
         <v/>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>UpperLevel1</t>
         </is>
       </c>
-      <c r="E4">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+1*Settings!$B$5*Settings!$B$3)</f>
+      <c r="N4">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="D5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>UpperLevel2</t>
         </is>
       </c>
-      <c r="E5">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+2*Settings!$B$5*Settings!$B$3)</f>
+      <c r="N5">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10624,37 +10774,47 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
+          <t>Lot</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>OpenPrice</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>ScenarioPrice</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>ScenarioPointsPnL</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>ScenarioMoneyPnL</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>IsTail</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>SectionID</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>UpperLevel3</t>
         </is>
       </c>
-      <c r="E6" s="1">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+3*Settings!$B$5*Settings!$B$3)</f>
-        <v/>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>ScenarioPrice</t>
-        </is>
-      </c>
-      <c r="G6" s="1" t="inlineStr">
-        <is>
-          <t>ScenarioPointsPnL</t>
-        </is>
-      </c>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>ScenarioMoneyPnL</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="inlineStr">
-        <is>
-          <t>IsTail</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>SectionID</t>
-        </is>
+      <c r="N6">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+3*Settings!$B$5*Settings!$B$3)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -10670,13 +10830,12 @@
         <f>CurrentPositions!C2</f>
         <v/>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>UpperLevel4</t>
-        </is>
+      <c r="D7">
+        <f>CurrentPositions!D2</f>
+        <v/>
       </c>
       <c r="E7">
-        <f>IF(E3=0,"Уровень не рассчитан",E3+4*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E2</f>
         <v/>
       </c>
       <c r="F7">
@@ -10697,6 +10856,15 @@
       </c>
       <c r="J7">
         <f>CurrentPositions!J2</f>
+        <v/>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>UpperLevel4</t>
+        </is>
+      </c>
+      <c r="N7">
+        <f>IF(N3=0,"Уровень не рассчитан",N3+4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10755,13 +10923,12 @@
         <f>CurrentPositions!C4</f>
         <v/>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>LowerLevel1</t>
-        </is>
+      <c r="D9">
+        <f>CurrentPositions!D4</f>
+        <v/>
       </c>
       <c r="E9">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-1*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E4</f>
         <v/>
       </c>
       <c r="F9">
@@ -10782,6 +10949,15 @@
       </c>
       <c r="J9">
         <f>CurrentPositions!J4</f>
+        <v/>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>LowerLevel1</t>
+        </is>
+      </c>
+      <c r="N9">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-1*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10798,13 +10974,12 @@
         <f>CurrentPositions!C5</f>
         <v/>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>LowerLevel2</t>
-        </is>
+      <c r="D10">
+        <f>CurrentPositions!D5</f>
+        <v/>
       </c>
       <c r="E10">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-2*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E5</f>
         <v/>
       </c>
       <c r="F10">
@@ -10825,6 +11000,15 @@
       </c>
       <c r="J10">
         <f>CurrentPositions!J5</f>
+        <v/>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>LowerLevel2</t>
+        </is>
+      </c>
+      <c r="N10">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-2*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10841,13 +11025,12 @@
         <f>CurrentPositions!C6</f>
         <v/>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>LowerLevel3</t>
-        </is>
+      <c r="D11">
+        <f>CurrentPositions!D6</f>
+        <v/>
       </c>
       <c r="E11">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-3*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E6</f>
         <v/>
       </c>
       <c r="F11">
@@ -10868,6 +11051,15 @@
       </c>
       <c r="J11">
         <f>CurrentPositions!J6</f>
+        <v/>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>LowerLevel3</t>
+        </is>
+      </c>
+      <c r="N11">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-3*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -10884,13 +11076,12 @@
         <f>CurrentPositions!C7</f>
         <v/>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>LowerLevel4</t>
-        </is>
+      <c r="D12">
+        <f>CurrentPositions!D7</f>
+        <v/>
       </c>
       <c r="E12">
-        <f>IF(E3=0,"Уровень не рассчитан",E3-4*Settings!$B$5*Settings!$B$3)</f>
+        <f>CurrentPositions!E7</f>
         <v/>
       </c>
       <c r="F12">
@@ -10911,6 +11102,15 @@
       </c>
       <c r="J12">
         <f>CurrentPositions!J7</f>
+        <v/>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>LowerLevel4</t>
+        </is>
+      </c>
+      <c r="N12">
+        <f>IF(N3=0,"Уровень не рассчитан",N3-4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
     </row>
@@ -19271,7 +19471,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>IF(Scenario_UP!B4&gt;=IF(B4=1,Scenario_UP!E4,IF(B4=2,Scenario_UP!E5,IF(B4=3,Scenario_UP!E6,Scenario_UP!E7))),"YES","NO")</f>
+        <f>IF(Scenario_UP!B4&gt;=IF(B4=1,Scenario_UP!N4,IF(B4=2,Scenario_UP!N5,IF(B4=3,Scenario_UP!N6,Scenario_UP!N7))),"YES","NO")</f>
         <v/>
       </c>
     </row>
@@ -19908,7 +20108,7 @@
         </is>
       </c>
       <c r="B12">
-        <f>IF(Scenario_DOWN!B4&lt;=IF(B4=1,Scenario_DOWN!E9,IF(B4=2,Scenario_DOWN!E10,IF(B4=3,Scenario_DOWN!E11,Scenario_DOWN!E12))),"YES","NO")</f>
+        <f>IF(Scenario_DOWN!B4&lt;=IF(B4=1,Scenario_DOWN!N9,IF(B4=2,Scenario_DOWN!N10,IF(B4=3,Scenario_DOWN!N11,Scenario_DOWN!N12))),"YES","NO")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix tail ticket logic and sync ScenarioText action priority with BasketSummary
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -29,7 +29,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -72,9 +74,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -714,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -806,6 +811,81 @@
       </c>
       <c r="C6">
         <f>IF(SectionCalculator_DOWN!B13="YES","OK","BLOCKED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tail exists when loss exists</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>IF(OR(Scenario_UP!B221&gt;=0,Scenario_UP!B222&lt;&gt;"N/A"),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>IF(OR(Scenario_DOWN!B221&gt;=0,Scenario_DOWN!B222&lt;&gt;"N/A"),"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ScenarioText action equals BasketSummary action</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>IF(OR(AND(BasketSummary!B13="BASKET_CLOSE",ScenarioText_UP!B31="ЗАКРЫТЬ ВСЮ КОРЗИНУ"),BasketSummary!B13&lt;&gt;"BASKET_CLOSE"),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>IF(OR(AND(BasketSummary!C13="BASKET_CLOSE",ScenarioText_DOWN!B31="ЗАКРЫТЬ ВСЮ КОРЗИНУ"),BasketSummary!C13&lt;&gt;"BASKET_CLOSE"),"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>NextTriggerLevel is numeric</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>IF(OR(ISNUMBER(ScenarioText_UP!B5),ScenarioText_UP!B5="Уровень не рассчитан"),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>IF(OR(ISNUMBER(ScenarioText_DOWN!B5),ScenarioText_DOWN!B5="Уровень не рассчитан"),"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DistancePoints is numeric</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>IF(OR(ISNUMBER(ScenarioText_UP!B6),ScenarioText_UP!B6="Расстояние не рассчитано"),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>IF(OR(ISNUMBER(ScenarioText_DOWN!B6),ScenarioText_DOWN!B6="Расстояние не рассчитано"),"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HumanReadableAction not empty</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>IF(AND(ScenarioText_UP!B31&lt;&gt;"",ISNUMBER(ScenarioText_UP!B4)),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>IF(AND(ScenarioText_DOWN!B31&lt;&gt;"",ISNUMBER(ScenarioText_DOWN!B4)),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -1019,7 +1099,7 @@
           <t>Текущая цена</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <f>IFERROR(CurrentPositions!F2,0)</f>
         <v/>
       </c>
@@ -1030,7 +1110,7 @@
           <t>Сценарная цена</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <f>IFERROR(Scenario_UP!B4,0)</f>
         <v/>
       </c>
@@ -1041,7 +1121,7 @@
           <t>Следующий уровень открытия</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!N4,IF(SectionCalculator_UP!B4=2,Scenario_UP!N5,IF(SectionCalculator_UP!B4=3,Scenario_UP!N6,IF(SectionCalculator_UP!B4=4,Scenario_UP!N7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
@@ -1052,7 +1132,7 @@
           <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <f>IF(OR(B5="Уровень не рассчитан",B4=""),"Расстояние не рассчитано",ROUND(ABS(B5-B4)*10000,0))</f>
         <v/>
       </c>
@@ -1063,7 +1143,7 @@
           <t>Большая позиция</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <f>IFERROR(IF(TailRecovery_UP!B16&gt;0,IF("UP"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_UP!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
@@ -1074,7 +1154,7 @@
           <t>Малая защитная позиция</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" s="4">
         <f>IFERROR(IF(TailRecovery_UP!B17&gt;0,IF("UP"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_UP!B17,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
@@ -1202,7 +1282,7 @@
           <t>Лот хвоста</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B24" s="4">
         <f>IFERROR(IF(TailRecovery_UP!B3&gt;0,TailRecovery_UP!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
@@ -1235,7 +1315,7 @@
           <t>Расчётный лот закрытия</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B27" s="4">
         <f>IFERROR(TailRecovery_UP!B9,0)</f>
         <v/>
       </c>
@@ -1246,7 +1326,7 @@
           <t>Округлённый лот закрытия</t>
         </is>
       </c>
-      <c r="B28">
+      <c r="B28" s="4">
         <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
@@ -1257,7 +1337,7 @@
           <t>Итоговый лот закрытия</t>
         </is>
       </c>
-      <c r="B29">
+      <c r="B29" s="4">
         <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
@@ -1268,7 +1348,7 @@
           <t>Остаток хвоста</t>
         </is>
       </c>
-      <c r="B30">
+      <c r="B30" s="4">
         <f>IF(OR(B24="Хвост не найден",NOT(ISNUMBER(B24))),"Хвост не найден",MAX(B24-B29,0))</f>
         <v/>
       </c>
@@ -1280,18 +1360,20 @@
         </is>
       </c>
       <c r="B31">
-        <f>IF(B13="ДА","ОТКРЫТЬ СЕКЦИЮ",IF(B15="ДА",IF(B16="ДА","ЗАКРЫТЬ СЕКЦИЮ + ЗАКРЫТЬ ХВОСТ","ЗАКРЫТЬ СЕКЦИЮ"),"ЖДАТЬ / НИЧЕГО НЕ ДЕЛАТЬ"))</f>
+        <f>IF(BasketSummary!B13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(BasketSummary!B13="CLOSE_SECTION+CLOSE_TAIL","ЗАКРЫТЬ СЕКЦИЮ + ЗАКРЫТЬ ХВОСТ",IF(BasketSummary!B13="CLOSE_SECTION","ЗАКРЫТЬ СЕКЦИЮ",IF(BasketSummary!B13="OPEN_SECTION","ОТКРЫТЬ СЕКЦИЮ",IF(BasketSummary!B13="SAFE","SAFE",IF(BasketSummary!B13="WAIT","ЖДАТЬ","BLOCKED"))))))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2">
+      <c r="A32" s="5">
         <f>B46</f>
         <v/>
       </c>
     </row>
     <row r="33"/>
-    <row r="34"/>
+    <row r="34">
+      <c r="B34" s="4" t="n"/>
+    </row>
     <row r="35"/>
     <row r="36"/>
     <row r="37"/>
@@ -1305,7 +1387,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", до="&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;", закрыть="&amp;TEXT(B29,"0.00")&amp;", остаток="&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B26,"0.00")&amp;" / "&amp;TEXT(B34,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1355,7 +1437,7 @@
           <t>Текущая цена</t>
         </is>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <f>IFERROR(CurrentPositions!F2,0)</f>
         <v/>
       </c>
@@ -1366,7 +1448,7 @@
           <t>Сценарная цена</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <f>IFERROR(Scenario_DOWN!B4,0)</f>
         <v/>
       </c>
@@ -1377,7 +1459,7 @@
           <t>Следующий уровень открытия</t>
         </is>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!N9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!N10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!N11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!N12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
@@ -1388,7 +1470,7 @@
           <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
-      <c r="B6">
+      <c r="B6" s="3">
         <f>IF(OR(B5="Уровень не рассчитан",B4=""),"Расстояние не рассчитано",ROUND(ABS(B5-B4)*10000,0))</f>
         <v/>
       </c>
@@ -1399,7 +1481,7 @@
           <t>Большая позиция</t>
         </is>
       </c>
-      <c r="B7">
+      <c r="B7" s="4">
         <f>IFERROR(IF(TailRecovery_DOWN!B16&gt;0,IF("DOWN"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_DOWN!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
@@ -1410,7 +1492,7 @@
           <t>Малая защитная позиция</t>
         </is>
       </c>
-      <c r="B8">
+      <c r="B8" s="4">
         <f>IFERROR(IF(TailRecovery_DOWN!B17&gt;0,IF("DOWN"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_DOWN!B17,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
@@ -1538,7 +1620,7 @@
           <t>Лот хвоста</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B24" s="4">
         <f>IFERROR(IF(TailRecovery_DOWN!B3&gt;0,TailRecovery_DOWN!B3,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
@@ -1571,7 +1653,7 @@
           <t>Расчётный лот закрытия</t>
         </is>
       </c>
-      <c r="B27">
+      <c r="B27" s="4">
         <f>IFERROR(TailRecovery_DOWN!B9,0)</f>
         <v/>
       </c>
@@ -1582,7 +1664,7 @@
           <t>Округлённый лот закрытия</t>
         </is>
       </c>
-      <c r="B28">
+      <c r="B28" s="4">
         <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
@@ -1593,7 +1675,7 @@
           <t>Итоговый лот закрытия</t>
         </is>
       </c>
-      <c r="B29">
+      <c r="B29" s="4">
         <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
@@ -1604,7 +1686,7 @@
           <t>Остаток хвоста</t>
         </is>
       </c>
-      <c r="B30">
+      <c r="B30" s="4">
         <f>IF(OR(B24="Хвост не найден",NOT(ISNUMBER(B24))),"Хвост не найден",MAX(B24-B29,0))</f>
         <v/>
       </c>
@@ -1616,18 +1698,20 @@
         </is>
       </c>
       <c r="B31">
-        <f>IF(B13="ДА","ОТКРЫТЬ СЕКЦИЮ",IF(B15="ДА",IF(B16="ДА","ЗАКРЫТЬ СЕКЦИЮ + ЗАКРЫТЬ ХВОСТ","ЗАКРЫТЬ СЕКЦИЮ"),"ЖДАТЬ / НИЧЕГО НЕ ДЕЛАТЬ"))</f>
+        <f>IF(BasketSummary!C13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(BasketSummary!C13="CLOSE_SECTION+CLOSE_TAIL","ЗАКРЫТЬ СЕКЦИЮ + ЗАКРЫТЬ ХВОСТ",IF(BasketSummary!C13="CLOSE_SECTION","ЗАКРЫТЬ СЕКЦИЮ",IF(BasketSummary!C13="OPEN_SECTION","ОТКРЫТЬ СЕКЦИЮ",IF(BasketSummary!C13="SAFE","SAFE",IF(BasketSummary!C13="WAIT","ЖДАТЬ","BLOCKED"))))))</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2">
+      <c r="A32" s="5">
         <f>B46</f>
         <v/>
       </c>
     </row>
     <row r="33"/>
-    <row r="34"/>
+    <row r="34">
+      <c r="B34" s="4" t="n"/>
+    </row>
     <row r="35"/>
     <row r="36"/>
     <row r="37"/>
@@ -1641,7 +1725,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", до="&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;", закрыть="&amp;TEXT(B29,"0.00")&amp;", остаток="&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B26,"0.00")&amp;" / "&amp;TEXT(B34,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1659,7 +1743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1683,6 +1767,11 @@
           <t>UsedBy</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1729,21 +1818,338 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Scenario_UP!B2</t>
+        </is>
+      </c>
+      <c r="B4">
+        <f>CurrentPositions!F2</f>
+        <v/>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CurrentPositions!F2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CurrentPrice</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B4</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>B2+B3*Settings!B3</f>
+        <v/>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B2,B3,Settings!B3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B12</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ScenarioPrice</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Scenario_UP!N1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <f>...</f>
+        <v/>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Scenario_UP positions</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Scenario_UP!N3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AverageBuyPrice</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Scenario_UP!N2</t>
+        </is>
+      </c>
+      <c r="B7">
+        <f>...</f>
+        <v/>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Scenario_UP positions</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Scenario_UP!N3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AverageSellPrice</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Scenario_UP!N3</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>(N1+N2)/2</f>
+        <v/>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>N1,N2</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Scenario_UP!N4:N12</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B221</t>
+        </is>
+      </c>
+      <c r="B9">
+        <f>MINIFS(...)</f>
+        <v/>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>H7:H206,B7:B206</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B222</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TailWorstPnL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B222</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>MINIFS(...)</f>
+        <v/>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>A7:A206,H7:H206,B221</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Scenario_UP!B223</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>TailTicket</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B7</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>IF(B3&lt;=0,0,FLOOR(...))</f>
+        <v/>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>B3,B5</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B14</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BigLot</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B8</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>IF(B3&lt;=0,0,FLOOR(...))</f>
+        <v/>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>B3,B6</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B14</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>SmallLot</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SectionCalculator_UP!B14</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>IF(...)</f>
+        <v/>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>B3,B7,B8,B12,B13</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ScenarioText_UP!B13</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>CanOpenSection</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>TailRecovery_UP!B10</t>
         </is>
       </c>
-      <c r="B4">
+      <c r="B14">
         <f>IF(B6="YES",MIN(B9,B4),0)</f>
         <v/>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>TailRecovery_UP!B9, TailRecovery_UP!B4, TailRecovery_UP!B6</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>BasketSummary!B7, Log!F2</t>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>B6,B9,B4</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Log!F2</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>CloseLotFinal</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>BasketSummary!B13</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(...)</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>B8,B9,B10</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>ScenarioText_UP!B31</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>NextAction</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ScenarioText_UP!B31</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>IF(BasketSummary!B13...)</f>
+        <v/>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BasketSummary!B13</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ScenarioText_UP!B46</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>HumanReadableAction</t>
         </is>
       </c>
     </row>
@@ -10603,7 +11009,7 @@
         </is>
       </c>
       <c r="B221">
-        <f>IFERROR(MIN(IF((B7:B206="SELL")*(H7:H206&lt;0),H7:H206)),0)</f>
+        <f>IFERROR(MINIFS(H7:H206,B7:B206,"SELL",H7:H206,"&lt;0"),0)</f>
         <v/>
       </c>
     </row>
@@ -10614,7 +11020,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IFERROR(MIN(IF((B7:B206="SELL")*(H7:H206=B221),A7:A206)),"N/A")</f>
+        <f>IFERROR(MINIFS(A7:A206,B7:B206,"SELL",H7:H206,B221),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -19281,7 +19687,7 @@
         </is>
       </c>
       <c r="B221">
-        <f>IFERROR(MIN(IF((B7:B206="BUY")*(H7:H206&lt;0),H7:H206)),0)</f>
+        <f>IFERROR(MINIFS(H7:H206,B7:B206,"BUY",H7:H206,"&lt;0"),0)</f>
         <v/>
       </c>
     </row>
@@ -19292,7 +19698,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IFERROR(MIN(IF((B7:B206="BUY")*(H7:H206=B221),A7:A206)),"N/A")</f>
+        <f>IFERROR(MINIFS(A7:A206,B7:B206,"BUY",H7:H206,B221),"N/A")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ScenarioText tail field mapping and add strict tail-lot validation checks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -719,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -886,6 +886,51 @@
       </c>
       <c r="C11">
         <f>IF(AND(ScenarioText_DOWN!B31&lt;&gt;"",ISNUMBER(ScenarioText_DOWN!B4)),"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TailTicket not mapped as lot</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Tail lot reasonable</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tail остаток &lt;= исходного</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B37),ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B37&gt;ScenarioText_UP!B25),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
@@ -1279,29 +1324,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Лот хвоста</t>
-        </is>
-      </c>
-      <c r="B24" s="4">
-        <f>IFERROR(IF(TailRecovery_UP!B3&gt;0,TailRecovery_UP!B3,"Хвост не найден"),"Хвост не найден")</f>
+          <t>Тикет хвоста</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>IFERROR(TailRecovery_UP!B3,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Убыток хвоста</t>
-        </is>
-      </c>
-      <c r="B25">
-        <f>IFERROR(TailRecovery_UP!B12,0)</f>
+          <t>Лот хвоста</t>
+        </is>
+      </c>
+      <c r="B25" s="4">
+        <f>IFERROR(IF(TailRecovery_UP!B4&gt;0,TailRecovery_UP!B4,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RecoveryFund до закрытия</t>
+          <t>Убыток хвоста на 1 лот</t>
         </is>
       </c>
       <c r="B26">
@@ -1312,44 +1357,44 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Расчётный лот закрытия</t>
-        </is>
-      </c>
-      <c r="B27" s="4">
-        <f>IFERROR(TailRecovery_UP!B9,0)</f>
+          <t>RecoveryFund до закрытия</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>IFERROR(TailRecovery_UP!B7,0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Округлённый лот закрытия</t>
+          <t>Расчётный лот закрытия</t>
         </is>
       </c>
       <c r="B28" s="4">
-        <f>IFERROR(TailRecovery_UP!B10,0)</f>
+        <f>IFERROR(TailRecovery_UP!B8,0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Итоговый лот закрытия</t>
+          <t>Округлённый лот закрытия</t>
         </is>
       </c>
       <c r="B29" s="4">
-        <f>IFERROR(TailRecovery_UP!B10,0)</f>
+        <f>IFERROR(TailRecovery_UP!B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Остаток хвоста</t>
+          <t>Итоговый лот закрытия</t>
         </is>
       </c>
       <c r="B30" s="4">
-        <f>IF(OR(B24="Хвост не найден",NOT(ISNUMBER(B24))),"Хвост не найден",MAX(B24-B29,0))</f>
+        <f>IFERROR(TailRecovery_UP!B10,0)</f>
         <v/>
       </c>
     </row>
@@ -1371,12 +1416,16 @@
       </c>
     </row>
     <row r="33"/>
-    <row r="34">
-      <c r="B34" s="4" t="n"/>
-    </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
+    <row r="34"/>
+    <row r="35">
+      <c r="B35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="n"/>
+    </row>
     <row r="38"/>
     <row r="39"/>
     <row r="40"/>
@@ -1387,7 +1436,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(B24="Хвост не найден","N/A",TEXT(Scenario_UP!B222,"0"))&amp;", до="&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;", закрыть="&amp;TEXT(B29,"0.00")&amp;", остаток="&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B26,"0.00")&amp;" / "&amp;TEXT(B34,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;IF(ISNUMBER(B37),TEXT(B37,"0.00"),B37)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(B37,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(B36,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1617,29 +1666,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Лот хвоста</t>
-        </is>
-      </c>
-      <c r="B24" s="4">
-        <f>IFERROR(IF(TailRecovery_DOWN!B3&gt;0,TailRecovery_DOWN!B3,"Хвост не найден"),"Хвост не найден")</f>
+          <t>Тикет хвоста</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>IFERROR(TailRecovery_DOWN!B3,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Убыток хвоста</t>
-        </is>
-      </c>
-      <c r="B25">
-        <f>IFERROR(TailRecovery_DOWN!B12,0)</f>
+          <t>Лот хвоста</t>
+        </is>
+      </c>
+      <c r="B25" s="4">
+        <f>IFERROR(IF(TailRecovery_DOWN!B4&gt;0,TailRecovery_DOWN!B4,"Хвост не найден"),"Хвост не найден")</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RecoveryFund до закрытия</t>
+          <t>Убыток хвоста на 1 лот</t>
         </is>
       </c>
       <c r="B26">
@@ -1650,44 +1699,44 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Расчётный лот закрытия</t>
-        </is>
-      </c>
-      <c r="B27" s="4">
-        <f>IFERROR(TailRecovery_DOWN!B9,0)</f>
+          <t>RecoveryFund до закрытия</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>IFERROR(TailRecovery_DOWN!B7,0)</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Округлённый лот закрытия</t>
+          <t>Расчётный лот закрытия</t>
         </is>
       </c>
       <c r="B28" s="4">
-        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B8,0)</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Итоговый лот закрытия</t>
+          <t>Округлённый лот закрытия</t>
         </is>
       </c>
       <c r="B29" s="4">
-        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B9,0)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Остаток хвоста</t>
+          <t>Итоговый лот закрытия</t>
         </is>
       </c>
       <c r="B30" s="4">
-        <f>IF(OR(B24="Хвост не найден",NOT(ISNUMBER(B24))),"Хвост не найден",MAX(B24-B29,0))</f>
+        <f>IFERROR(TailRecovery_DOWN!B10,0)</f>
         <v/>
       </c>
     </row>
@@ -1709,12 +1758,16 @@
       </c>
     </row>
     <row r="33"/>
-    <row r="34">
-      <c r="B34" s="4" t="n"/>
-    </row>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
+    <row r="34"/>
+    <row r="35">
+      <c r="B35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="B36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="B37" s="4" t="n"/>
+    </row>
     <row r="38"/>
     <row r="39"/>
     <row r="40"/>
@@ -1725,7 +1778,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Лот хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B29),TEXT(B29,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(B24="Хвост не найден","N/A",TEXT(Scenario_DOWN!B222,"0"))&amp;", до="&amp;IF(ISNUMBER(B24),TEXT(B24,"0.00"),B24)&amp;", закрыть="&amp;TEXT(B29,"0.00")&amp;", остаток="&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),B30)&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B26,"0.00")&amp;" / "&amp;TEXT(B34,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;IF(ISNUMBER(B37),TEXT(B37,"0.00"),B37)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(B37,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(B36,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ScenarioText/Log tail residue and recovery fund mappings
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -1021,11 +1021,11 @@
         </is>
       </c>
       <c r="D2">
-        <f>IF(BasketSummary!B13="WAIT","ЖДАТЬ",IF(BasketSummary!B13="SAFE","SAFE",IF(BasketSummary!B13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(AND(TailRecovery_UP!B10&gt;0,TailRecovery_UP!B10&lt;TailRecovery_UP!B3),"ЗАКРЫТЬ ХВОСТ ЧАСТИЧНО","ЗАКРЫТЬ СЕКЦИЮ"))))</f>
+        <f>IF(BasketSummary!B13="WAIT","ЖДАТЬ",IF(BasketSummary!B13="SAFE","SAFE",IF(BasketSummary!B13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(AND(TailRecovery_UP!B10&gt;0,TailRecovery_UP!B10&lt;TailRecovery_UP!B4),"ЗАКРЫТЬ ХВОСТ ЧАСТИЧНО","ЗАКРЫТЬ СЕКЦИЮ"))))</f>
         <v/>
       </c>
       <c r="E2">
-        <f>IFERROR(TailRecovery_UP!B3,0)</f>
+        <f>IFERROR(TailRecovery_UP!B4,0)</f>
         <v/>
       </c>
       <c r="F2">
@@ -1033,15 +1033,15 @@
         <v/>
       </c>
       <c r="G2">
-        <f>IF(OR(NOT(ISNUMBER(E2)),NOT(ISNUMBER(F2))),"Хвост не найден",MAX(E2-F2,0))</f>
+        <f>IFERROR(TailRecovery_UP!B14,0)</f>
         <v/>
       </c>
       <c r="H2">
-        <f>IFERROR(TailRecovery_UP!B5,0)</f>
+        <f>IFERROR(TailRecovery_UP!B7,0)</f>
         <v/>
       </c>
       <c r="I2">
-        <f>IFERROR(TailRecovery_UP!B7,0)</f>
+        <f>IFERROR(TailRecovery_UP!B13,0)</f>
         <v/>
       </c>
       <c r="J2">
@@ -1069,11 +1069,11 @@
         </is>
       </c>
       <c r="D3">
-        <f>IF(BasketSummary!C13="WAIT","ЖДАТЬ",IF(BasketSummary!C13="SAFE","SAFE",IF(BasketSummary!C13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(AND(TailRecovery_DOWN!B10&gt;0,TailRecovery_DOWN!B10&lt;TailRecovery_DOWN!B3),"ЗАКРЫТЬ ХВОСТ ЧАСТИЧНО","ЗАКРЫТЬ СЕКЦИЮ"))))</f>
+        <f>IF(BasketSummary!C13="WAIT","ЖДАТЬ",IF(BasketSummary!C13="SAFE","SAFE",IF(BasketSummary!C13="BASKET_CLOSE","ЗАКРЫТЬ ВСЮ КОРЗИНУ",IF(AND(TailRecovery_DOWN!B10&gt;0,TailRecovery_DOWN!B10&lt;TailRecovery_DOWN!B4),"ЗАКРЫТЬ ХВОСТ ЧАСТИЧНО","ЗАКРЫТЬ СЕКЦИЮ"))))</f>
         <v/>
       </c>
       <c r="E3">
-        <f>IFERROR(TailRecovery_DOWN!B3,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B4,0)</f>
         <v/>
       </c>
       <c r="F3">
@@ -1081,15 +1081,15 @@
         <v/>
       </c>
       <c r="G3">
-        <f>IF(OR(NOT(ISNUMBER(E3)),NOT(ISNUMBER(F3))),"Хвост не найден",MAX(E3-F3,0))</f>
+        <f>IFERROR(TailRecovery_DOWN!B14,0)</f>
         <v/>
       </c>
       <c r="H3">
-        <f>IFERROR(TailRecovery_DOWN!B5,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B7,0)</f>
         <v/>
       </c>
       <c r="I3">
-        <f>IFERROR(TailRecovery_DOWN!B7,0)</f>
+        <f>IFERROR(TailRecovery_DOWN!B13,0)</f>
         <v/>
       </c>
       <c r="J3">
@@ -1436,7 +1436,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;IF(ISNUMBER(B37),TEXT(B37,"0.00"),B37)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(B37,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(B36,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;IF(ISNUMBER(B37),TEXT(B37,"0.00"),B37)&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(B34,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(B37,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(B36,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix reserve/recovery mapping in ScenarioText and add sync validations
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -719,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -892,44 +892,74 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TailTicket not mapped as lot</t>
+          <t>ReserveAdd mapping sync</t>
         </is>
       </c>
       <c r="B12">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B19=SectionCalculator_UP!B33,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B19=SectionCalculator_DOWN!B33,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tail lot reasonable</t>
+          <t>RecoveryAdd mapping sync</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B20=SectionCalculator_UP!B34,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B20=SectionCalculator_DOWN!B34,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>TailTicket not mapped as lot</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tail lot reasonable</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Tail остаток &lt;= исходного</t>
         </is>
       </c>
-      <c r="B14">
+      <c r="B16">
         <f>IF(AND(ISNUMBER(ScenarioText_UP!B37),ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B37&gt;ScenarioText_UP!B25),"ERROR","OK")</f>
         <v/>
       </c>
-      <c r="C14">
+      <c r="C16">
         <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
         <v/>
       </c>
@@ -1295,7 +1325,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>IFERROR(TailRecovery_UP!B6,0)</f>
+        <f>IFERROR(SectionCalculator_UP!B33,0)</f>
         <v/>
       </c>
     </row>
@@ -1306,7 +1336,29 @@
         </is>
       </c>
       <c r="B20">
-        <f>IFERROR(TailRecovery_UP!B8,0)</f>
+        <f>IFERROR(SectionCalculator_UP!B34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Резерв после</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>IFERROR(SectionCalculator_UP!B35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RecoveryFund после цикла</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>IFERROR(SectionCalculator_UP!B36,0)</f>
         <v/>
       </c>
     </row>
@@ -1436,7 +1488,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1637,7 +1689,7 @@
         </is>
       </c>
       <c r="B19">
-        <f>IFERROR(TailRecovery_DOWN!B6,0)</f>
+        <f>IFERROR(SectionCalculator_DOWN!B33,0)</f>
         <v/>
       </c>
     </row>
@@ -1648,7 +1700,29 @@
         </is>
       </c>
       <c r="B20">
-        <f>IFERROR(TailRecovery_DOWN!B8,0)</f>
+        <f>IFERROR(SectionCalculator_DOWN!B34,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Резерв после</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>IFERROR(SectionCalculator_DOWN!B35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RecoveryFund после цикла</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>IFERROR(SectionCalculator_DOWN!B36,0)</f>
         <v/>
       </c>
     </row>
@@ -1778,7 +1852,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;"; Резерв после: "&amp;TEXT(B19,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Add financial safety guards and stricter validation for recovery constraints
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -719,7 +719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -961,6 +961,51 @@
       </c>
       <c r="C16">
         <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>RecoveryFundAfter &gt;= 0</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>IF(TailRecovery_UP!B13&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>IF(TailRecovery_DOWN!B13&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>CloseLotFinal &lt;= TailLot</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>IF(TailRecovery_UP!B10&gt;TailRecovery_UP!B4,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>IF(TailRecovery_DOWN!B10&gt;TailRecovery_DOWN!B4,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TailLotAfter &gt;= 0</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>IF(TailRecovery_UP!B14&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>IF(TailRecovery_DOWN!B14&lt;0,"ERROR","OK")</f>
         <v/>
       </c>
     </row>
@@ -1488,7 +1533,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1852,7 +1897,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"Решение: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -24536,7 +24581,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>B4-B10</f>
+        <f>MAX(0,B4-B10)</f>
         <v/>
       </c>
     </row>
@@ -24738,7 +24783,7 @@
         </is>
       </c>
       <c r="B14">
-        <f>B4-B10</f>
+        <f>MAX(0,B4-B10)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ScenarioText semantic mapping for trigger/distance and add ScenarioSpread checks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -912,11 +912,11 @@
         </is>
       </c>
       <c r="B9">
-        <f>IF(OR(ISNUMBER(ScenarioText_UP!B5),ScenarioText_UP!B5="Уровень не рассчитан"),"OK","ERROR")</f>
+        <f>IF(OR(ISNUMBER(ScenarioText_UP!B9),ScenarioText_UP!B9="Уровень не рассчитан"),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C9">
-        <f>IF(OR(ISNUMBER(ScenarioText_DOWN!B5),ScenarioText_DOWN!B5="Уровень не рассчитан"),"OK","ERROR")</f>
+        <f>IF(OR(ISNUMBER(ScenarioText_DOWN!B9),ScenarioText_DOWN!B9="Уровень не рассчитан"),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -927,145 +927,220 @@
         </is>
       </c>
       <c r="B10">
-        <f>IF(OR(ISNUMBER(ScenarioText_UP!B6),ScenarioText_UP!B6="Расстояние не рассчитано"),"OK","ERROR")</f>
+        <f>IF(OR(ISNUMBER(ScenarioText_UP!B10),ScenarioText_UP!B10="Расстояние не рассчитано"),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C10">
-        <f>IF(OR(ISNUMBER(ScenarioText_DOWN!B6),ScenarioText_DOWN!B6="Расстояние не рассчитано"),"OK","ERROR")</f>
+        <f>IF(OR(ISNUMBER(ScenarioText_DOWN!B10),ScenarioText_DOWN!B10="Расстояние не рассчитано"),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>HumanReadableAction not empty</t>
+          <t>ScenarioMid is numeric</t>
         </is>
       </c>
       <c r="B11">
-        <f>IF(AND(ScenarioText_UP!B31&lt;&gt;"",ISNUMBER(ScenarioText_UP!B4)),"OK","ERROR")</f>
+        <f>IF(ISNUMBER(ScenarioText_UP!B7),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C11">
-        <f>IF(AND(ScenarioText_DOWN!B31&lt;&gt;"",ISNUMBER(ScenarioText_DOWN!B4)),"OK","ERROR")</f>
+        <f>IF(ISNUMBER(ScenarioText_DOWN!B7),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ReserveAdd mapping sync</t>
+          <t>ScenarioSpread is numeric</t>
         </is>
       </c>
       <c r="B12">
-        <f>IF(ScenarioText_UP!B19=SectionCalculator_UP!B33,"OK","ERROR")</f>
+        <f>IF(ISNUMBER(ScenarioText_UP!B8),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>IF(ScenarioText_DOWN!B19=SectionCalculator_DOWN!B33,"OK","ERROR")</f>
+        <f>IF(ISNUMBER(ScenarioText_DOWN!B8),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>RecoveryAdd mapping sync</t>
+          <t>Scenario_* B8 not empty</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(ScenarioText_UP!B20=SectionCalculator_UP!B34,"OK","ERROR")</f>
+        <f>IF(Scenario_UP!B8&lt;&gt;"","OK","ERROR")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>IF(ScenarioText_DOWN!B20=SectionCalculator_DOWN!B34,"OK","ERROR")</f>
+        <f>IF(Scenario_DOWN!B8&lt;&gt;"","OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TailTicket not mapped as lot</t>
+          <t>ScenarioText B9!=B5</t>
         </is>
       </c>
       <c r="B14">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B9&lt;&gt;ScenarioText_UP!B5,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B9&lt;&gt;ScenarioText_DOWN!B5,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tail lot reasonable</t>
+          <t>ScenarioText B10!=B6</t>
         </is>
       </c>
       <c r="B15">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B10&lt;&gt;ScenarioText_UP!B6,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B10&lt;&gt;ScenarioText_DOWN!B6,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tail остаток &lt;= исходного</t>
+          <t>HumanReadableAction not empty</t>
         </is>
       </c>
       <c r="B16">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B37),ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B37&gt;ScenarioText_UP!B25),"ERROR","OK")</f>
+        <f>IF(AND(ScenarioText_UP!B31&lt;&gt;"",ISNUMBER(ScenarioText_UP!B4)),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
+        <f>IF(AND(ScenarioText_DOWN!B31&lt;&gt;"",ISNUMBER(ScenarioText_DOWN!B4)),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RecoveryFundAfter &gt;= 0</t>
+          <t>ReserveAdd mapping sync</t>
         </is>
       </c>
       <c r="B17">
-        <f>IF(TailRecovery_UP!B13&lt;0,"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B19=SectionCalculator_UP!B33,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>IF(TailRecovery_DOWN!B13&lt;0,"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B19=SectionCalculator_DOWN!B33,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CloseLotFinal &lt;= TailLot</t>
+          <t>RecoveryAdd mapping sync</t>
         </is>
       </c>
       <c r="B18">
-        <f>IF(TailRecovery_UP!B10&gt;TailRecovery_UP!B4,"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B20=SectionCalculator_UP!B34,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>IF(TailRecovery_DOWN!B10&gt;TailRecovery_DOWN!B4,"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B20=SectionCalculator_DOWN!B34,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>TailTicket not mapped as lot</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tail lot reasonable</t>
+        </is>
+      </c>
+      <c r="B20">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tail остаток &lt;= исходного</t>
+        </is>
+      </c>
+      <c r="B21">
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B37),ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B37&gt;ScenarioText_UP!B25),"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>RecoveryFundAfter &gt;= 0</t>
+        </is>
+      </c>
+      <c r="B22">
+        <f>IF(TailRecovery_UP!B13&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>IF(TailRecovery_DOWN!B13&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CloseLotFinal &lt;= TailLot</t>
+        </is>
+      </c>
+      <c r="B23">
+        <f>IF(TailRecovery_UP!B10&gt;TailRecovery_UP!B4,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>IF(TailRecovery_DOWN!B10&gt;TailRecovery_DOWN!B4,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>TailLotAfter &gt;= 0</t>
         </is>
       </c>
-      <c r="B19">
+      <c r="B24">
         <f>IF(TailRecovery_UP!B14&lt;0,"ERROR","OK")</f>
         <v/>
       </c>
-      <c r="C19">
+      <c r="C24">
         <f>IF(TailRecovery_DOWN!B14&lt;0,"ERROR","OK")</f>
         <v/>
       </c>
@@ -1330,46 +1405,38 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Следующий уровень открытия</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!N4,IF(SectionCalculator_UP!B4=2,Scenario_UP!N5,IF(SectionCalculator_UP!B4=3,Scenario_UP!N6,IF(SectionCalculator_UP!B4=4,Scenario_UP!N7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
-        <v/>
-      </c>
+      <c r="B8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Уровень секции</t>
+          <t>Следующий уровень открытия</t>
         </is>
       </c>
       <c r="B9">
-        <f>IFERROR(SectionCalculator_UP!B4,0)</f>
+        <f>IFERROR(IF(SectionCalculator_UP!B4=1,Scenario_UP!N4,IF(SectionCalculator_UP!B4=2,Scenario_UP!N5,IF(SectionCalculator_UP!B4=3,Scenario_UP!N6,IF(SectionCalculator_UP!B4=4,Scenario_UP!N7,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Причина</t>
+          <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
       <c r="B10">
-        <f>IF(SectionCalculator_UP!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция недоступна: уровень/риск-гейт/хвост")</f>
+        <f>IF(OR(B9="Уровень не рассчитан",B7=""),"Расстояние не рассчитано",ROUND(ABS(B9-B7)/Settings!$B$3,0))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Малая защитная позиция</t>
+          <t>Большая позиция</t>
         </is>
       </c>
       <c r="B11">
-        <f>IFERROR(IF(TailRecovery_UP!B17&gt;0,IF("UP"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_UP!B17,"0.00"),"Не открывать"),"Не открывать")</f>
+        <f>IFERROR(IF(TailRecovery_UP!B16&gt;0,IF("UP"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_UP!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
@@ -1378,6 +1445,10 @@
         <is>
           <t>Проверки риска</t>
         </is>
+      </c>
+      <c r="B12">
+        <f>IFERROR(IF(TailRecovery_UP!B17&gt;0,IF("UP"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_UP!B17,"0.00"),"Не открывать"),"Не открывать")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1705,46 +1776,38 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Следующий уровень открытия</t>
-        </is>
-      </c>
-      <c r="B8" s="4">
-        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!N9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!N10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!N11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!N12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
-        <v/>
-      </c>
+      <c r="B8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Уровень секции</t>
+          <t>Следующий уровень открытия</t>
         </is>
       </c>
       <c r="B9">
-        <f>IFERROR(SectionCalculator_DOWN!B4,0)</f>
+        <f>IFERROR(IF(SectionCalculator_DOWN!B4=1,Scenario_DOWN!N9,IF(SectionCalculator_DOWN!B4=2,Scenario_DOWN!N10,IF(SectionCalculator_DOWN!B4=3,Scenario_DOWN!N11,IF(SectionCalculator_DOWN!B4=4,Scenario_DOWN!N12,"Уровень не рассчитан")))),"Уровень не рассчитан")</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Причина</t>
+          <t>Расстояние до уровня, пунктов</t>
         </is>
       </c>
       <c r="B10">
-        <f>IF(SectionCalculator_DOWN!B14="YES","цена достигла уровня; хвост найден; риск-лимиты OK","секция недоступна: уровень/риск-гейт/хвост")</f>
+        <f>IF(OR(B9="Уровень не рассчитан",B7=""),"Расстояние не рассчитано",ROUND(ABS(B9-B7)/Settings!$B$3,0))</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Малая защитная позиция</t>
+          <t>Большая позиция</t>
         </is>
       </c>
       <c r="B11">
-        <f>IFERROR(IF(TailRecovery_DOWN!B17&gt;0,IF("DOWN"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_DOWN!B17,"0.00"),"Не открывать"),"Не открывать")</f>
+        <f>IFERROR(IF(TailRecovery_DOWN!B16&gt;0,IF("DOWN"="UP","SELL ","BUY ")&amp;TEXT(TailRecovery_DOWN!B16,"0.00"),"Не открывать"),"Не открывать")</f>
         <v/>
       </c>
     </row>
@@ -1753,6 +1816,10 @@
         <is>
           <t>Проверки риска</t>
         </is>
+      </c>
+      <c r="B12">
+        <f>IFERROR(IF(TailRecovery_DOWN!B17&gt;0,IF("DOWN"="UP","BUY ","SELL ")&amp;TEXT(TailRecovery_DOWN!B17,"0.00"),"Не открывать"),"Не открывать")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -2807,6 +2874,17 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ScenarioSpread</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>(B6-B5)/Settings!$B$3</f>
+        <v/>
+      </c>
+    </row>
     <row r="9">
       <c r="M9" t="inlineStr">
         <is>
@@ -13130,6 +13208,17 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ScenarioSpread</t>
+        </is>
+      </c>
+      <c r="B8">
+        <f>(B6-B5)/Settings!$B$3</f>
+        <v/>
+      </c>
+    </row>
     <row r="9">
       <c r="M9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Correct ScenarioText Bid/Ask/Mid/Spread semantic mapping and recommendation text
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -1396,16 +1396,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Spread, пунктов</t>
+          <t>Сценарный Mid</t>
         </is>
       </c>
       <c r="B7" s="4">
-        <f>IFERROR(Settings!B34,0)</f>
+        <f>IFERROR(Scenario_UP!B7,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Сценарный Spread</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>IFERROR(Scenario_UP!B8,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1443,7 +1451,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Проверки риска</t>
+          <t>Малая защитная позиция</t>
         </is>
       </c>
       <c r="B12">
@@ -1454,11 +1462,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Можно открыть секцию</t>
+          <t>Уровень секции</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")</f>
+        <f>IFERROR(SectionCalculator_UP!B4,0)</f>
         <v/>
       </c>
     </row>
@@ -1676,7 +1684,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1767,16 +1775,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Spread, пунктов</t>
+          <t>Сценарный Mid</t>
         </is>
       </c>
       <c r="B7" s="4">
-        <f>IFERROR(Settings!B34,0)</f>
+        <f>IFERROR(Scenario_DOWN!B7,0)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="4" t="n"/>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Сценарный Spread</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>IFERROR(Scenario_DOWN!B8,0)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1814,7 +1830,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Проверки риска</t>
+          <t>Малая защитная позиция</t>
         </is>
       </c>
       <c r="B12">
@@ -1825,11 +1841,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Можно открыть секцию</t>
+          <t>Уровень секции</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")</f>
+        <f>IFERROR(SectionCalculator_DOWN!B4,0)</f>
         <v/>
       </c>
     </row>
@@ -2047,7 +2063,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущая расчетная цена: "&amp;TEXT(B3,"0.00000")&amp;"."&amp;CHAR(10)&amp;"Сценарий: "&amp;B2&amp;CHAR(10)&amp;"Текущая цена: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Сценарная цена: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B5),TEXT(B5,"0.00000"),B5)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B6),TEXT(B6,"0")&amp;" пунктов",B6)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Finalize ScenarioSpread points semantics and remove legacy single-price references
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,179 +968,209 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Scenario_* B8 not empty</t>
+          <t>ScenarioSpread bounds</t>
         </is>
       </c>
       <c r="B13">
-        <f>IF(Scenario_UP!B8&lt;&gt;"","OK","ERROR")</f>
+        <f>IF(AND(ScenarioText_UP!B8&gt;0,ScenarioText_UP!B8&lt;1000),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C13">
-        <f>IF(Scenario_DOWN!B8&lt;&gt;"","OK","ERROR")</f>
+        <f>IF(AND(ScenarioText_DOWN!B8&gt;0,ScenarioText_DOWN!B8&lt;1000),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ScenarioText B9!=B5</t>
+          <t>Scenario_* B8 not empty</t>
         </is>
       </c>
       <c r="B14">
-        <f>IF(ScenarioText_UP!B9&lt;&gt;ScenarioText_UP!B5,"OK","ERROR")</f>
+        <f>IF(Scenario_UP!B8&lt;&gt;"","OK","ERROR")</f>
         <v/>
       </c>
       <c r="C14">
-        <f>IF(ScenarioText_DOWN!B9&lt;&gt;ScenarioText_DOWN!B5,"OK","ERROR")</f>
+        <f>IF(Scenario_DOWN!B8&lt;&gt;"","OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ScenarioText B10!=B6</t>
+          <t>No legacy single-price wording</t>
         </is>
       </c>
       <c r="B15">
-        <f>IF(ScenarioText_UP!B10&lt;&gt;ScenarioText_UP!B6,"OK","ERROR")</f>
+        <f>IF(ISERROR(SEARCH("Сценарная цена",ScenarioText_UP!B46)),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C15">
-        <f>IF(ScenarioText_DOWN!B10&lt;&gt;ScenarioText_DOWN!B6,"OK","ERROR")</f>
+        <f>IF(ISERROR(SEARCH("Сценарная цена",ScenarioText_DOWN!B46)),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HumanReadableAction not empty</t>
+          <t>ScenarioText B9!=B5</t>
         </is>
       </c>
       <c r="B16">
-        <f>IF(AND(ScenarioText_UP!B31&lt;&gt;"",ISNUMBER(ScenarioText_UP!B4)),"OK","ERROR")</f>
+        <f>IF(ScenarioText_UP!B9&lt;&gt;ScenarioText_UP!B5,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C16">
-        <f>IF(AND(ScenarioText_DOWN!B31&lt;&gt;"",ISNUMBER(ScenarioText_DOWN!B4)),"OK","ERROR")</f>
+        <f>IF(ScenarioText_DOWN!B9&lt;&gt;ScenarioText_DOWN!B5,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ReserveAdd mapping sync</t>
+          <t>ScenarioText B10!=B6</t>
         </is>
       </c>
       <c r="B17">
-        <f>IF(ScenarioText_UP!B19=SectionCalculator_UP!B33,"OK","ERROR")</f>
+        <f>IF(ScenarioText_UP!B10&lt;&gt;ScenarioText_UP!B6,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C17">
-        <f>IF(ScenarioText_DOWN!B19=SectionCalculator_DOWN!B33,"OK","ERROR")</f>
+        <f>IF(ScenarioText_DOWN!B10&lt;&gt;ScenarioText_DOWN!B6,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>RecoveryAdd mapping sync</t>
+          <t>HumanReadableAction not empty</t>
         </is>
       </c>
       <c r="B18">
-        <f>IF(ScenarioText_UP!B20=SectionCalculator_UP!B34,"OK","ERROR")</f>
+        <f>IF(AND(ScenarioText_UP!B31&lt;&gt;"",ISNUMBER(ScenarioText_UP!B4)),"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C18">
-        <f>IF(ScenarioText_DOWN!B20=SectionCalculator_DOWN!B34,"OK","ERROR")</f>
+        <f>IF(AND(ScenarioText_DOWN!B31&lt;&gt;"",ISNUMBER(ScenarioText_DOWN!B4)),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TailTicket not mapped as lot</t>
+          <t>ReserveAdd mapping sync</t>
         </is>
       </c>
       <c r="B19">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B19=SectionCalculator_UP!B33,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C19">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B19=SectionCalculator_DOWN!B33,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tail lot reasonable</t>
+          <t>RecoveryAdd mapping sync</t>
         </is>
       </c>
       <c r="B20">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_UP!B20=SectionCalculator_UP!B34,"OK","ERROR")</f>
         <v/>
       </c>
       <c r="C20">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
+        <f>IF(ScenarioText_DOWN!B20=SectionCalculator_DOWN!B34,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tail остаток &lt;= исходного</t>
+          <t>TailTicket not mapped as lot</t>
         </is>
       </c>
       <c r="B21">
-        <f>IF(AND(ISNUMBER(ScenarioText_UP!B37),ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B37&gt;ScenarioText_UP!B25),"ERROR","OK")</f>
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B24),ScenarioText_UP!B24&gt;1000,ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
         <v/>
       </c>
       <c r="C21">
-        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B24),ScenarioText_DOWN!B24&gt;1000,ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RecoveryFundAfter &gt;= 0</t>
+          <t>Tail lot reasonable</t>
         </is>
       </c>
       <c r="B22">
-        <f>IF(TailRecovery_UP!B13&lt;0,"ERROR","OK")</f>
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B25&gt;100),"ERROR","OK")</f>
         <v/>
       </c>
       <c r="C22">
-        <f>IF(TailRecovery_DOWN!B13&lt;0,"ERROR","OK")</f>
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B25&gt;100),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CloseLotFinal &lt;= TailLot</t>
+          <t>Tail остаток &lt;= исходного</t>
         </is>
       </c>
       <c r="B23">
-        <f>IF(TailRecovery_UP!B10&gt;TailRecovery_UP!B4,"ERROR","OK")</f>
+        <f>IF(AND(ISNUMBER(ScenarioText_UP!B37),ISNUMBER(ScenarioText_UP!B25),ScenarioText_UP!B37&gt;ScenarioText_UP!B25),"ERROR","OK")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>IF(TailRecovery_DOWN!B10&gt;TailRecovery_DOWN!B4,"ERROR","OK")</f>
+        <f>IF(AND(ISNUMBER(ScenarioText_DOWN!B37),ISNUMBER(ScenarioText_DOWN!B25),ScenarioText_DOWN!B37&gt;ScenarioText_DOWN!B25),"ERROR","OK")</f>
         <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>RecoveryFundAfter &gt;= 0</t>
+        </is>
+      </c>
+      <c r="B24">
+        <f>IF(TailRecovery_UP!B13&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>IF(TailRecovery_DOWN!B13&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CloseLotFinal &lt;= TailLot</t>
+        </is>
+      </c>
+      <c r="B25">
+        <f>IF(TailRecovery_UP!B10&gt;TailRecovery_UP!B4,"ERROR","OK")</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>IF(TailRecovery_DOWN!B10&gt;TailRecovery_DOWN!B4,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>TailLotAfter &gt;= 0</t>
         </is>
       </c>
-      <c r="B24">
+      <c r="B26">
         <f>IF(TailRecovery_UP!B14&lt;0,"ERROR","OK")</f>
         <v/>
       </c>
-      <c r="C24">
+      <c r="C26">
         <f>IF(TailRecovery_DOWN!B14&lt;0,"ERROR","OK")</f>
         <v/>
       </c>
@@ -1399,7 +1429,7 @@
           <t>Сценарный Mid</t>
         </is>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <f>IFERROR(Scenario_UP!B7,0)</f>
         <v/>
       </c>
@@ -1410,7 +1440,7 @@
           <t>Сценарный Spread</t>
         </is>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <f>IFERROR(Scenario_UP!B8,0)</f>
         <v/>
       </c>
@@ -1684,7 +1714,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -1778,7 +1808,7 @@
           <t>Сценарный Mid</t>
         </is>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <f>IFERROR(Scenario_DOWN!B7,0)</f>
         <v/>
       </c>
@@ -1789,7 +1819,7 @@
           <t>Сценарный Spread</t>
         </is>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <f>IFERROR(Scenario_DOWN!B8,0)</f>
         <v/>
       </c>
@@ -2063,7 +2093,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B7&amp;" / "&amp;B8&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix UX/Log consistency and refresh FormulaDependencyMap for Bid-Ask architecture
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -1290,7 +1290,7 @@
         <v/>
       </c>
       <c r="K2">
-        <f>IF(OR(SectionCalculator_UP!B14&lt;&gt;"YES",SectionCalculator_UP!B13&lt;&gt;"YES"),"YES","NO")</f>
+        <f>IF(OR(SectionCalculator_UP!B14&lt;&gt;"YES",SectionCalculator_UP!B13&lt;&gt;"YES"),"ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
       <c r="K3">
-        <f>IF(OR(SectionCalculator_DOWN!B14&lt;&gt;"YES",SectionCalculator_DOWN!B13&lt;&gt;"YES"),"YES","NO")</f>
+        <f>IF(OR(SectionCalculator_DOWN!B14&lt;&gt;"YES",SectionCalculator_DOWN!B13&lt;&gt;"YES"),"ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;B13&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -2111,7 +2111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2188,349 +2188,268 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Scenario_UP!B2</t>
+          <t>Scenario_UP!B5</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>'=CurrentPositions!F2</t>
+          <t>'=B2+B4*Settings!B3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CurrentPositions!F2</t>
+          <t>Scenario_UP!B2,B4,Settings!B3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Scenario_UP!B4</t>
+          <t>Scenario_UP!B6:B8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>CurrentPrice</t>
+          <t>ScenarioBid</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Scenario_UP!B4</t>
+          <t>Scenario_UP!B6</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>'=B2+B3*Settings!B3</t>
+          <t>'=B3+B4*Settings!B3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Scenario_UP!B2,B3,Settings!B3</t>
+          <t>Scenario_UP!B3,B4,Settings!B3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B12</t>
+          <t>Scenario_UP!B8,F12:F211</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ScenarioPrice</t>
+          <t>ScenarioAsk</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Scenario_UP!N1</t>
+          <t>Scenario_UP!B7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>'=...</t>
+          <t>'=(B5+B6)/2</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Scenario_UP positions</t>
+          <t>B5,B6</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Scenario_UP!N3</t>
+          <t>SectionCalculator_UP!B12,ScenarioText_UP!B7</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AverageBuyPrice</t>
+          <t>ScenarioMid</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Scenario_UP!N2</t>
+          <t>Scenario_UP!B8</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>'=...</t>
+          <t>'=(B6-B5)/Settings!B3</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Scenario_UP positions</t>
+          <t>B6,B5,Settings!B3</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Scenario_UP!N3</t>
+          <t>ScenarioText_UP!B8</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AverageSellPrice</t>
+          <t>ScenarioSpread</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Scenario_UP!N3</t>
+          <t>Scenario_UP!B221</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>'=(N1+N2)/2</t>
+          <t>'=IF(COUNT(K12:K211)=0,0,MIN(K12:K211))</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>N1,N2</t>
+          <t>K12:K211</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Scenario_UP!N4:N12</t>
+          <t>Scenario_UP!B222</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Center</t>
+          <t>TailWorstPnL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Scenario_UP!B221</t>
+          <t>Scenario_UP!B222</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>'=MINIFS(...)</t>
+          <t>'=IF(B221=0,"N/A",MIN(L12:L211))</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>H7:H206,B7:B206</t>
+          <t>B221,L12:L211</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Scenario_UP!B222</t>
+          <t>Scenario_UP!B223</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TailWorstPnL</t>
+          <t>TailTicket</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Scenario_UP!B222</t>
+          <t>SectionCalculator_UP!B14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>'=MINIFS(...)</t>
+          <t>'=IF(...)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A7:A206,H7:H206,B221</t>
+          <t>B3,B7,B8,B12,B13</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Scenario_UP!B223</t>
+          <t>ScenarioText_UP!B13</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>TailTicket</t>
+          <t>CanOpenSection</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B7</t>
+          <t>TailRecovery_UP!B10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>'=IF(B3&lt;=0,0,FLOOR(...))</t>
+          <t>'=IF(B6="YES",MIN(B9,B4),0)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>B3,B5</t>
+          <t>B6,B9,B4</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B14</t>
+          <t>Log!F2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>BigLot</t>
+          <t>CloseLotFinal</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B8</t>
+          <t>BasketSummary!B13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>'=IF(B3&lt;=0,0,FLOOR(...))</t>
+          <t>'=IF(...)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B3,B6</t>
+          <t>B8,B9,B10</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B14</t>
+          <t>ScenarioText_UP!B31</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SmallLot</t>
+          <t>NextAction</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B14</t>
+          <t>ScenarioText_UP!B31</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>'=IF(...)</t>
+          <t>'=IF(BasketSummary!B13...)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>B3,B7,B8,B12,B13</t>
+          <t>BasketSummary!B13</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>ScenarioText_UP!B13</t>
+          <t>ScenarioText_UP!B46</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
-        <is>
-          <t>CanOpenSection</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>TailRecovery_UP!B10</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>'=IF(B6="YES",MIN(B9,B4),0)</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>B6,B9,B4</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Log!F2</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>CloseLotFinal</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>BasketSummary!B13</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>'=IF(...)</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>B8,B9,B10</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>ScenarioText_UP!B31</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>NextAction</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>ScenarioText_UP!B31</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>'=IF(BasketSummary!B13...)</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>BasketSummary!B13</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>ScenarioText_UP!B46</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
         <is>
           <t>HumanReadableAction</t>
         </is>

</xml_diff>

<commit_message>
Update latest recovery lock workbooks
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -1290,7 +1290,7 @@
         <v/>
       </c>
       <c r="K2">
-        <f>IF(OR(SectionCalculator_UP!B14&lt;&gt;"YES",SectionCalculator_UP!B13&lt;&gt;"YES"),"ДА","НЕТ")</f>
+        <f>IF(BasketSummary!B13="SAFE","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
       <c r="K3">
-        <f>IF(OR(SectionCalculator_DOWN!B14&lt;&gt;"YES",SectionCalculator_DOWN!B13&lt;&gt;"YES"),"ДА","НЕТ")</f>
+        <f>IF(BasketSummary!C13="SAFE","ДА","НЕТ")</f>
         <v/>
       </c>
     </row>
@@ -1714,7 +1714,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;B38&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
     <row r="45"/>
     <row r="46">
       <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;IF(B14="ДА","НЕТ","ДА")&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;B38&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ScenarioText SAFE mapping and refresh dependency map
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1172,6 +1172,36 @@
       </c>
       <c r="C26">
         <f>IF(TailRecovery_DOWN!B14&lt;0,"ERROR","OK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ScenarioText SAFE not empty</t>
+        </is>
+      </c>
+      <c r="B27">
+        <f>IF(ScenarioText_UP!B38&lt;&gt;"","OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C27">
+        <f>IF(ScenarioText_DOWN!B38&lt;&gt;"","OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ScenarioText SAFE equals Log SAFE</t>
+        </is>
+      </c>
+      <c r="B28">
+        <f>IF(ScenarioText_UP!B38=Log!K2,"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C28">
+        <f>IF(ScenarioText_DOWN!B38=Log!K3,"OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -2111,7 +2141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2144,314 +2174,270 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Scenario_UP!B4</t>
+          <t>Scenario_UP!B5</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>'=Scenario_UP!B2+Scenario_UP!B3*Settings!B3</t>
+          <t>'=B2+B4*Settings!B3</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Scenario_UP!B2, Scenario_UP!B3, Settings!B3</t>
+          <t>Scenario_UP!B2, Scenario_UP!B4, Settings!B3</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B12, ScenarioText_UP!B4</t>
+          <t>Scenario_UP!B7:B8, SectionCalculator_UP!B12, ScenarioText_UP!B5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ScenarioBid</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Scenario_DOWN!B4</t>
+          <t>Scenario_UP!B6</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>'=Scenario_DOWN!B2-Scenario_DOWN!B3*Settings!B3</t>
+          <t>'=B3+B4*Settings!B3</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Scenario_DOWN!B2, Scenario_DOWN!B3, Settings!B3</t>
+          <t>Scenario_UP!B3, Scenario_UP!B4, Settings!B3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>SectionCalculator_DOWN!B12, ScenarioText_DOWN!B4</t>
+          <t>Scenario_UP!B7:B8, Scenario_UP!F12:F211, ScenarioText_UP!B6</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ScenarioAsk</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Scenario_UP!B5</t>
+          <t>Scenario_UP!B7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>'=B2+B4*Settings!B3</t>
+          <t>'=(B5+B6)/2</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Scenario_UP!B2,B4,Settings!B3</t>
+          <t>Scenario_UP!B5, Scenario_UP!B6</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Scenario_UP!B6:B8</t>
+          <t>SectionCalculator_UP!B12, ScenarioText_UP!B7</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ScenarioBid</t>
+          <t>ScenarioMid</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Scenario_UP!B6</t>
+          <t>Scenario_UP!B8</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>'=B3+B4*Settings!B3</t>
+          <t>'=(B6-B5)/Settings!B3</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Scenario_UP!B3,B4,Settings!B3</t>
+          <t>Scenario_UP!B6, Scenario_UP!B5, Settings!B3</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Scenario_UP!B8,F12:F211</t>
+          <t>ScenarioText_UP!B8</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ScenarioAsk</t>
+          <t>ScenarioSpread</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Scenario_UP!B7</t>
+          <t>Scenario_UP!K12:L211</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>'=(B5+B6)/2</t>
+          <t>PnL helper range</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>B5,B6</t>
+          <t>Scenario_UP!C12:F211, Settings!B3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B12,ScenarioText_UP!B7</t>
+          <t>Scenario_UP!B221:B223</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>ScenarioMid</t>
+          <t>Tail helper range</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Scenario_UP!B8</t>
+          <t>Scenario_UP!B221</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>'=(B6-B5)/Settings!B3</t>
+          <t>'=IF(COUNT(K12:K211)=0,0,MIN(K12:K211))</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B6,B5,Settings!B3</t>
+          <t>Scenario_UP!K12:K211</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ScenarioText_UP!B8</t>
+          <t>Scenario_UP!B222</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>ScenarioSpread</t>
+          <t>TailWorstPnL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Scenario_UP!B221</t>
+          <t>Scenario_UP!B222</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>'=IF(COUNT(K12:K211)=0,0,MIN(K12:K211))</t>
+          <t>'=IF(B221=0,"N/A",MIN(L12:L211))</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>K12:K211</t>
+          <t>Scenario_UP!B221, Scenario_UP!L12:L211</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Scenario_UP!B222</t>
+          <t>Scenario_UP!B223, ScenarioText_UP!B24</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TailWorstPnL</t>
+          <t>TailTicket</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Scenario_UP!B222</t>
+          <t>BasketSummary!B13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>'=IF(B221=0,"N/A",MIN(L12:L211))</t>
+          <t>'=IF(...)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B221,L12:L211</t>
+          <t>BasketSummary!B8, BasketSummary!B9, BasketSummary!B10</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Scenario_UP!B223</t>
+          <t>ScenarioText_UP!B31, ScenarioText_UP!B38, Log!D2, Log!K2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>TailTicket</t>
+          <t>NextAction</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SectionCalculator_UP!B14</t>
+          <t>ScenarioText_UP!B31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>'=IF(...)</t>
+          <t>'=IF(BasketSummary!B13...)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B3,B7,B8,B12,B13</t>
+          <t>BasketSummary!B13</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ScenarioText_UP!B13</t>
+          <t>ScenarioText_UP!B46</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>CanOpenSection</t>
+          <t>HumanReadableAction</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TailRecovery_UP!B10</t>
+          <t>ScenarioText_UP!B38</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>'=IF(B6="YES",MIN(B9,B4),0)</t>
+          <t>'=IF(BasketSummary!B13="SAFE","ДА","НЕТ")</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>B6,B9,B4</t>
+          <t>BasketSummary!B13</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Log!F2</t>
+          <t>ScenarioText_UP!B46, Validation</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>CloseLotFinal</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>BasketSummary!B13</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>'=IF(...)</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>B8,B9,B10</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>ScenarioText_UP!B31</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>NextAction</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ScenarioText_UP!B31</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>'=IF(BasketSummary!B13...)</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>BasketSummary!B13</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>ScenarioText_UP!B46</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>HumanReadableAction</t>
+          <t>SAFE flag</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix ScenarioText SAFE cells by moving merged recommendation block
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -1383,7 +1383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1717,40 +1717,83 @@
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5">
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Разрешено закрытие хвоста</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>IF(TailRecovery_UP!B11="YES","ДА","НЕТ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Убыток закрываемой части</t>
+        </is>
+      </c>
+      <c r="B35" s="4">
+        <f>IFERROR(TailRecovery_UP!B12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RecoveryFund после закрытия</t>
+        </is>
+      </c>
+      <c r="B36" s="4">
+        <f>IFERROR(TailRecovery_UP!B13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Остаток хвоста</t>
+        </is>
+      </c>
+      <c r="B37" s="4">
+        <f>IFERROR(TailRecovery_UP!B14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>IF(BasketSummary!B13="SAFE","ДА","НЕТ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5">
         <f>B46</f>
         <v/>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35">
-      <c r="B35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="4" t="n"/>
-    </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40"/>
     <row r="41"/>
     <row r="42"/>
     <row r="43"/>
     <row r="44"/>
     <row r="45"/>
-    <row r="46">
-      <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;B38&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
-        <v/>
-      </c>
-    </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A32:H45"/>
+    <mergeCell ref="A39:H52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1762,7 +1805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2096,40 +2139,83 @@
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5">
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Разрешено закрытие хвоста</t>
+        </is>
+      </c>
+      <c r="B34">
+        <f>IF(TailRecovery_DOWN!B11="YES","ДА","НЕТ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Убыток закрываемой части</t>
+        </is>
+      </c>
+      <c r="B35" s="4">
+        <f>IFERROR(TailRecovery_DOWN!B12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RecoveryFund после закрытия</t>
+        </is>
+      </c>
+      <c r="B36" s="4">
+        <f>IFERROR(TailRecovery_DOWN!B13,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Остаток хвоста</t>
+        </is>
+      </c>
+      <c r="B37" s="4">
+        <f>IFERROR(TailRecovery_DOWN!B14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SAFE</t>
+        </is>
+      </c>
+      <c r="B38">
+        <f>IF(BasketSummary!C13="SAFE","ДА","НЕТ")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5">
         <f>B46</f>
         <v/>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35">
-      <c r="B35" s="4" t="n"/>
-    </row>
-    <row r="36">
-      <c r="B36" s="4" t="n"/>
-    </row>
-    <row r="37">
-      <c r="B37" s="4" t="n"/>
-    </row>
-    <row r="38"/>
-    <row r="39"/>
     <row r="40"/>
     <row r="41"/>
     <row r="42"/>
     <row r="43"/>
     <row r="44"/>
     <row r="45"/>
-    <row r="46">
-      <c r="B46">
-        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;B38&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
-        <v/>
-      </c>
-    </row>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A32:H45"/>
+    <mergeCell ref="A39:H52"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix detailed recommendation block rendering in ScenarioText
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1202,6 +1202,21 @@
       </c>
       <c r="C28">
         <f>IF(ScenarioText_DOWN!B38=Log!K3,"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Detailed recommendation block not empty</t>
+        </is>
+      </c>
+      <c r="B29">
+        <f>IF(AND(ScenarioText_UP!A39&lt;&gt;"",ScenarioText_UP!A39&lt;&gt;0),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C29">
+        <f>IF(AND(ScenarioText_DOWN!A39&lt;&gt;"",ScenarioText_DOWN!A39&lt;&gt;0),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -1774,7 +1789,7 @@
     </row>
     <row r="39">
       <c r="A39" s="5">
-        <f>B46</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вверх."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_UP!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_UP!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_UP!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;B38&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>
@@ -2196,7 +2211,7 @@
     </row>
     <row r="39">
       <c r="A39" s="5">
-        <f>B46</f>
+        <f>"ПОДРОБНАЯ РЕКОМЕНДАЦИЯ"&amp;CHAR(10)&amp;CHAR(10)&amp;"Сценарий: цена идет вниз."&amp;CHAR(10)&amp;"Текущий Bid: "&amp;TEXT(B3,"0.00000")&amp;CHAR(10)&amp;"Текущий Ask: "&amp;TEXT(B4,"0.00000")&amp;CHAR(10)&amp;"Сценарный Bid: "&amp;TEXT(B5,"0.00000")&amp;CHAR(10)&amp;"Сценарный Ask: "&amp;TEXT(B6,"0.00000")&amp;CHAR(10)&amp;"Сценарный Mid: "&amp;TEXT(B7,"0.00000")&amp;CHAR(10)&amp;"Spread: "&amp;TEXT(B8,"0")&amp;" пунктов"&amp;CHAR(10)&amp;"Следующий уровень: "&amp;IF(ISNUMBER(B9),TEXT(B9,"0.00000"),B9)&amp;CHAR(10)&amp;"Расстояние до уровня: "&amp;IF(ISNUMBER(B10),TEXT(B10,"0")&amp;" пунктов",B10)&amp;CHAR(10)&amp;CHAR(10)&amp;"Рекомендация по секции: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Можно открыть секцию: "&amp;IF(SectionCalculator_DOWN!B14="YES","ДА","НЕТ")&amp;CHAR(10)&amp;"Можно закрыть секцию: "&amp;B15&amp;CHAR(10)&amp;"Можно закрыть хвост: "&amp;B16&amp;CHAR(10)&amp;CHAR(10)&amp;"Тип хвоста: "&amp;B23&amp;CHAR(10)&amp;"Тикет хвоста: "&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;CHAR(10)&amp;"Лот хвоста до закрытия: "&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;CHAR(10)&amp;"Итоговый лот закрытия: "&amp;IF(ISNUMBER(B30),TEXT(B30,"0.00"),"0.00")&amp;CHAR(10)&amp;"Остаток хвоста после закрытия: "&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;CHAR(10)&amp;"RecoveryFund после: "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"ДЕЙСТВИЕ: "&amp;B31&amp;CHAR(10)&amp;"Если открывать секцию: "&amp;B11&amp;" / "&amp;B12&amp;CHAR(10)&amp;"Если закрывать хвост: тип="&amp;B23&amp;", тикет="&amp;IF(ISNUMBER(B24),TEXT(B24,"0"),B24)&amp;", до="&amp;IF(ISNUMBER(B25),TEXT(B25,"0.00"),B25)&amp;", закрыть="&amp;TEXT(B30,"0.00")&amp;", остаток="&amp;TEXT(TailRecovery_DOWN!B14,"0.00")&amp;CHAR(10)&amp;"Добавить в резерв: "&amp;TEXT(B19,"0.00")&amp;"; Добавить в RecoveryFund: "&amp;TEXT(B20,"0.00")&amp;CHAR(10)&amp;"Резерв после: "&amp;TEXT(B21,"0.00")&amp;"; RecoveryFund после цикла: "&amp;TEXT(B22,"0.00")&amp;CHAR(10)&amp;"RecoveryFund до/после закрытия хвоста: "&amp;TEXT(B27,"0.00")&amp;" / "&amp;TEXT(TailRecovery_DOWN!B13,"0.00")&amp;CHAR(10)&amp;"SAFE: "&amp;B38&amp;CHAR(10)&amp;"ИТОГОВОЕ ДЕЙСТВИЕ: "&amp;B31</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix TailTicket selection to match TailWorstPnL
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -780,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1217,6 +1217,21 @@
       </c>
       <c r="C29">
         <f>IF(AND(ScenarioText_DOWN!A39&lt;&gt;"",ScenarioText_DOWN!A39&lt;&gt;0),"OK","ERROR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TailTicket belongs to TailWorstPnL</t>
+        </is>
+      </c>
+      <c r="B30">
+        <f>IF(OR(Scenario_UP!B222="N/A",INDEX(Scenario_UP!K12:K211,MATCH(Scenario_UP!B222,Scenario_UP!A12:A211,0))=Scenario_UP!B221),"OK","ERROR")</f>
+        <v/>
+      </c>
+      <c r="C30">
+        <f>IF(OR(Scenario_DOWN!B222="N/A",INDEX(Scenario_DOWN!K12:K211,MATCH(Scenario_DOWN!B222,Scenario_DOWN!A12:A211,0))=Scenario_DOWN!B221),"OK","ERROR")</f>
         <v/>
       </c>
     </row>
@@ -2442,12 +2457,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>'=IF(B221=0,"N/A",MIN(L12:L211))</t>
+          <t>'=IF(B221=0,"N/A",MINIFS(L12:L211,K12:K211,B221))</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Scenario_UP!B221, Scenario_UP!L12:L211</t>
+          <t>Scenario_UP!B221, Scenario_UP!K12:K211, Scenario_UP!L12:L211</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -13069,7 +13084,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IF(B221=0,"N/A",MIN(L12:L211))</f>
+        <f>IF(B221=0,"N/A",MINIFS(L12:L211,K12:K211,B221))</f>
         <v/>
       </c>
     </row>
@@ -23403,7 +23418,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IF(B221=0,"N/A",MIN(L12:L211))</f>
+        <f>IF(B221=0,"N/A",MINIFS(L12:L211,K12:K211,B221))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Use LibreOffice-safe helper for TailTicket selection
</commit_message>
<xml_diff>
--- a/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
+++ b/recovery_lock_cascade_next_step/recovery_lock_cascade_next_step.xlsx
@@ -2257,7 +2257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2452,106 +2452,133 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>Scenario_UP!O12:O211</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>'=IF(Krow=$B$221,Lrow,"")</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Scenario_UP!K12:K211, Scenario_UP!L12:L211, Scenario_UP!B221</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
           <t>Scenario_UP!B222</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>'=IF(B221=0,"N/A",MINIFS(L12:L211,K12:K211,B221))</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Scenario_UP!B221, Scenario_UP!K12:K211, Scenario_UP!L12:L211</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Scenario_UP!B223, ScenarioText_UP!B24</t>
-        </is>
-      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>TailTicket</t>
+          <t>TailFinalTicketCandidates</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BasketSummary!B13</t>
+          <t>Scenario_UP!B222</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>'=IF(...)</t>
+          <t>'=IF(B221=0,"N/A",MIN(O12:O211))</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BasketSummary!B8, BasketSummary!B9, BasketSummary!B10</t>
+          <t>Scenario_UP!B221, Scenario_UP!O12:O211</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ScenarioText_UP!B31, ScenarioText_UP!B38, Log!D2, Log!K2</t>
+          <t>Scenario_UP!B223, ScenarioText_UP!B24</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>NextAction</t>
+          <t>TailTicket</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ScenarioText_UP!B31</t>
+          <t>BasketSummary!B13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>'=IF(BasketSummary!B13...)</t>
+          <t>'=IF(...)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BasketSummary!B13</t>
+          <t>BasketSummary!B8, BasketSummary!B9, BasketSummary!B10</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ScenarioText_UP!B46</t>
+          <t>ScenarioText_UP!B31, ScenarioText_UP!B38, Log!D2, Log!K2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>HumanReadableAction</t>
+          <t>NextAction</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>ScenarioText_UP!B31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>'=IF(BasketSummary!B13...)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>BasketSummary!B13</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ScenarioText_UP!B46</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HumanReadableAction</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>ScenarioText_UP!B38</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>'=IF(BasketSummary!B13="SAFE","ДА","НЕТ")</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>BasketSummary!B13</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>ScenarioText_UP!B46, Validation</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>SAFE flag</t>
         </is>
@@ -2798,7 +2825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N225"/>
+  <dimension ref="A1:O225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3103,6 +3130,10 @@
         <f>IF(N3=0,"Уровень не рассчитан",N3-4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
+      <c r="O12">
+        <f>IF(K12=$B$221,L12,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -3153,6 +3184,10 @@
         <f>IF(K13&lt;&gt;"",A13,"")</f>
         <v/>
       </c>
+      <c r="O13">
+        <f>IF(K13=$B$221,L13,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -3203,6 +3238,10 @@
         <f>IF(K14&lt;&gt;"",A14,"")</f>
         <v/>
       </c>
+      <c r="O14">
+        <f>IF(K14=$B$221,L14,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -3253,6 +3292,10 @@
         <f>IF(K15&lt;&gt;"",A15,"")</f>
         <v/>
       </c>
+      <c r="O15">
+        <f>IF(K15=$B$221,L15,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -3303,6 +3346,10 @@
         <f>IF(K16&lt;&gt;"",A16,"")</f>
         <v/>
       </c>
+      <c r="O16">
+        <f>IF(K16=$B$221,L16,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -3353,6 +3400,10 @@
         <f>IF(K17&lt;&gt;"",A17,"")</f>
         <v/>
       </c>
+      <c r="O17">
+        <f>IF(K17=$B$221,L17,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -3403,6 +3454,10 @@
         <f>IF(K18&lt;&gt;"",A18,"")</f>
         <v/>
       </c>
+      <c r="O18">
+        <f>IF(K18=$B$221,L18,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -3453,6 +3508,10 @@
         <f>IF(K19&lt;&gt;"",A19,"")</f>
         <v/>
       </c>
+      <c r="O19">
+        <f>IF(K19=$B$221,L19,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -3503,6 +3562,10 @@
         <f>IF(K20&lt;&gt;"",A20,"")</f>
         <v/>
       </c>
+      <c r="O20">
+        <f>IF(K20=$B$221,L20,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -3553,6 +3616,10 @@
         <f>IF(K21&lt;&gt;"",A21,"")</f>
         <v/>
       </c>
+      <c r="O21">
+        <f>IF(K21=$B$221,L21,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -3603,6 +3670,10 @@
         <f>IF(K22&lt;&gt;"",A22,"")</f>
         <v/>
       </c>
+      <c r="O22">
+        <f>IF(K22=$B$221,L22,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -3653,6 +3724,10 @@
         <f>IF(K23&lt;&gt;"",A23,"")</f>
         <v/>
       </c>
+      <c r="O23">
+        <f>IF(K23=$B$221,L23,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -3703,6 +3778,10 @@
         <f>IF(K24&lt;&gt;"",A24,"")</f>
         <v/>
       </c>
+      <c r="O24">
+        <f>IF(K24=$B$221,L24,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -3753,6 +3832,10 @@
         <f>IF(K25&lt;&gt;"",A25,"")</f>
         <v/>
       </c>
+      <c r="O25">
+        <f>IF(K25=$B$221,L25,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -3803,6 +3886,10 @@
         <f>IF(K26&lt;&gt;"",A26,"")</f>
         <v/>
       </c>
+      <c r="O26">
+        <f>IF(K26=$B$221,L26,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -3853,6 +3940,10 @@
         <f>IF(K27&lt;&gt;"",A27,"")</f>
         <v/>
       </c>
+      <c r="O27">
+        <f>IF(K27=$B$221,L27,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -3903,6 +3994,10 @@
         <f>IF(K28&lt;&gt;"",A28,"")</f>
         <v/>
       </c>
+      <c r="O28">
+        <f>IF(K28=$B$221,L28,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -3953,6 +4048,10 @@
         <f>IF(K29&lt;&gt;"",A29,"")</f>
         <v/>
       </c>
+      <c r="O29">
+        <f>IF(K29=$B$221,L29,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -4003,6 +4102,10 @@
         <f>IF(K30&lt;&gt;"",A30,"")</f>
         <v/>
       </c>
+      <c r="O30">
+        <f>IF(K30=$B$221,L30,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -4053,6 +4156,10 @@
         <f>IF(K31&lt;&gt;"",A31,"")</f>
         <v/>
       </c>
+      <c r="O31">
+        <f>IF(K31=$B$221,L31,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -4103,6 +4210,10 @@
         <f>IF(K32&lt;&gt;"",A32,"")</f>
         <v/>
       </c>
+      <c r="O32">
+        <f>IF(K32=$B$221,L32,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -4153,6 +4264,10 @@
         <f>IF(K33&lt;&gt;"",A33,"")</f>
         <v/>
       </c>
+      <c r="O33">
+        <f>IF(K33=$B$221,L33,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -4203,6 +4318,10 @@
         <f>IF(K34&lt;&gt;"",A34,"")</f>
         <v/>
       </c>
+      <c r="O34">
+        <f>IF(K34=$B$221,L34,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -4253,6 +4372,10 @@
         <f>IF(K35&lt;&gt;"",A35,"")</f>
         <v/>
       </c>
+      <c r="O35">
+        <f>IF(K35=$B$221,L35,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -4303,6 +4426,10 @@
         <f>IF(K36&lt;&gt;"",A36,"")</f>
         <v/>
       </c>
+      <c r="O36">
+        <f>IF(K36=$B$221,L36,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -4353,6 +4480,10 @@
         <f>IF(K37&lt;&gt;"",A37,"")</f>
         <v/>
       </c>
+      <c r="O37">
+        <f>IF(K37=$B$221,L37,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -4403,6 +4534,10 @@
         <f>IF(K38&lt;&gt;"",A38,"")</f>
         <v/>
       </c>
+      <c r="O38">
+        <f>IF(K38=$B$221,L38,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -4453,6 +4588,10 @@
         <f>IF(K39&lt;&gt;"",A39,"")</f>
         <v/>
       </c>
+      <c r="O39">
+        <f>IF(K39=$B$221,L39,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -4503,6 +4642,10 @@
         <f>IF(K40&lt;&gt;"",A40,"")</f>
         <v/>
       </c>
+      <c r="O40">
+        <f>IF(K40=$B$221,L40,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -4553,6 +4696,10 @@
         <f>IF(K41&lt;&gt;"",A41,"")</f>
         <v/>
       </c>
+      <c r="O41">
+        <f>IF(K41=$B$221,L41,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -4603,6 +4750,10 @@
         <f>IF(K42&lt;&gt;"",A42,"")</f>
         <v/>
       </c>
+      <c r="O42">
+        <f>IF(K42=$B$221,L42,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -4653,6 +4804,10 @@
         <f>IF(K43&lt;&gt;"",A43,"")</f>
         <v/>
       </c>
+      <c r="O43">
+        <f>IF(K43=$B$221,L43,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -4703,6 +4858,10 @@
         <f>IF(K44&lt;&gt;"",A44,"")</f>
         <v/>
       </c>
+      <c r="O44">
+        <f>IF(K44=$B$221,L44,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -4753,6 +4912,10 @@
         <f>IF(K45&lt;&gt;"",A45,"")</f>
         <v/>
       </c>
+      <c r="O45">
+        <f>IF(K45=$B$221,L45,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -4803,6 +4966,10 @@
         <f>IF(K46&lt;&gt;"",A46,"")</f>
         <v/>
       </c>
+      <c r="O46">
+        <f>IF(K46=$B$221,L46,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -4853,6 +5020,10 @@
         <f>IF(K47&lt;&gt;"",A47,"")</f>
         <v/>
       </c>
+      <c r="O47">
+        <f>IF(K47=$B$221,L47,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -4903,6 +5074,10 @@
         <f>IF(K48&lt;&gt;"",A48,"")</f>
         <v/>
       </c>
+      <c r="O48">
+        <f>IF(K48=$B$221,L48,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -4953,6 +5128,10 @@
         <f>IF(K49&lt;&gt;"",A49,"")</f>
         <v/>
       </c>
+      <c r="O49">
+        <f>IF(K49=$B$221,L49,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -5003,6 +5182,10 @@
         <f>IF(K50&lt;&gt;"",A50,"")</f>
         <v/>
       </c>
+      <c r="O50">
+        <f>IF(K50=$B$221,L50,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -5053,6 +5236,10 @@
         <f>IF(K51&lt;&gt;"",A51,"")</f>
         <v/>
       </c>
+      <c r="O51">
+        <f>IF(K51=$B$221,L51,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -5103,6 +5290,10 @@
         <f>IF(K52&lt;&gt;"",A52,"")</f>
         <v/>
       </c>
+      <c r="O52">
+        <f>IF(K52=$B$221,L52,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -5153,6 +5344,10 @@
         <f>IF(K53&lt;&gt;"",A53,"")</f>
         <v/>
       </c>
+      <c r="O53">
+        <f>IF(K53=$B$221,L53,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -5203,6 +5398,10 @@
         <f>IF(K54&lt;&gt;"",A54,"")</f>
         <v/>
       </c>
+      <c r="O54">
+        <f>IF(K54=$B$221,L54,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -5253,6 +5452,10 @@
         <f>IF(K55&lt;&gt;"",A55,"")</f>
         <v/>
       </c>
+      <c r="O55">
+        <f>IF(K55=$B$221,L55,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -5303,6 +5506,10 @@
         <f>IF(K56&lt;&gt;"",A56,"")</f>
         <v/>
       </c>
+      <c r="O56">
+        <f>IF(K56=$B$221,L56,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -5353,6 +5560,10 @@
         <f>IF(K57&lt;&gt;"",A57,"")</f>
         <v/>
       </c>
+      <c r="O57">
+        <f>IF(K57=$B$221,L57,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -5403,6 +5614,10 @@
         <f>IF(K58&lt;&gt;"",A58,"")</f>
         <v/>
       </c>
+      <c r="O58">
+        <f>IF(K58=$B$221,L58,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -5453,6 +5668,10 @@
         <f>IF(K59&lt;&gt;"",A59,"")</f>
         <v/>
       </c>
+      <c r="O59">
+        <f>IF(K59=$B$221,L59,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -5503,6 +5722,10 @@
         <f>IF(K60&lt;&gt;"",A60,"")</f>
         <v/>
       </c>
+      <c r="O60">
+        <f>IF(K60=$B$221,L60,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -5553,6 +5776,10 @@
         <f>IF(K61&lt;&gt;"",A61,"")</f>
         <v/>
       </c>
+      <c r="O61">
+        <f>IF(K61=$B$221,L61,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -5603,6 +5830,10 @@
         <f>IF(K62&lt;&gt;"",A62,"")</f>
         <v/>
       </c>
+      <c r="O62">
+        <f>IF(K62=$B$221,L62,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -5653,6 +5884,10 @@
         <f>IF(K63&lt;&gt;"",A63,"")</f>
         <v/>
       </c>
+      <c r="O63">
+        <f>IF(K63=$B$221,L63,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -5703,6 +5938,10 @@
         <f>IF(K64&lt;&gt;"",A64,"")</f>
         <v/>
       </c>
+      <c r="O64">
+        <f>IF(K64=$B$221,L64,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -5753,6 +5992,10 @@
         <f>IF(K65&lt;&gt;"",A65,"")</f>
         <v/>
       </c>
+      <c r="O65">
+        <f>IF(K65=$B$221,L65,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -5803,6 +6046,10 @@
         <f>IF(K66&lt;&gt;"",A66,"")</f>
         <v/>
       </c>
+      <c r="O66">
+        <f>IF(K66=$B$221,L66,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -5853,6 +6100,10 @@
         <f>IF(K67&lt;&gt;"",A67,"")</f>
         <v/>
       </c>
+      <c r="O67">
+        <f>IF(K67=$B$221,L67,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -5903,6 +6154,10 @@
         <f>IF(K68&lt;&gt;"",A68,"")</f>
         <v/>
       </c>
+      <c r="O68">
+        <f>IF(K68=$B$221,L68,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -5953,6 +6208,10 @@
         <f>IF(K69&lt;&gt;"",A69,"")</f>
         <v/>
       </c>
+      <c r="O69">
+        <f>IF(K69=$B$221,L69,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -6003,6 +6262,10 @@
         <f>IF(K70&lt;&gt;"",A70,"")</f>
         <v/>
       </c>
+      <c r="O70">
+        <f>IF(K70=$B$221,L70,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -6053,6 +6316,10 @@
         <f>IF(K71&lt;&gt;"",A71,"")</f>
         <v/>
       </c>
+      <c r="O71">
+        <f>IF(K71=$B$221,L71,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -6103,6 +6370,10 @@
         <f>IF(K72&lt;&gt;"",A72,"")</f>
         <v/>
       </c>
+      <c r="O72">
+        <f>IF(K72=$B$221,L72,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -6153,6 +6424,10 @@
         <f>IF(K73&lt;&gt;"",A73,"")</f>
         <v/>
       </c>
+      <c r="O73">
+        <f>IF(K73=$B$221,L73,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -6203,6 +6478,10 @@
         <f>IF(K74&lt;&gt;"",A74,"")</f>
         <v/>
       </c>
+      <c r="O74">
+        <f>IF(K74=$B$221,L74,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -6253,6 +6532,10 @@
         <f>IF(K75&lt;&gt;"",A75,"")</f>
         <v/>
       </c>
+      <c r="O75">
+        <f>IF(K75=$B$221,L75,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -6303,6 +6586,10 @@
         <f>IF(K76&lt;&gt;"",A76,"")</f>
         <v/>
       </c>
+      <c r="O76">
+        <f>IF(K76=$B$221,L76,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77">
@@ -6353,6 +6640,10 @@
         <f>IF(K77&lt;&gt;"",A77,"")</f>
         <v/>
       </c>
+      <c r="O77">
+        <f>IF(K77=$B$221,L77,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78">
@@ -6403,6 +6694,10 @@
         <f>IF(K78&lt;&gt;"",A78,"")</f>
         <v/>
       </c>
+      <c r="O78">
+        <f>IF(K78=$B$221,L78,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -6453,6 +6748,10 @@
         <f>IF(K79&lt;&gt;"",A79,"")</f>
         <v/>
       </c>
+      <c r="O79">
+        <f>IF(K79=$B$221,L79,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80">
@@ -6503,6 +6802,10 @@
         <f>IF(K80&lt;&gt;"",A80,"")</f>
         <v/>
       </c>
+      <c r="O80">
+        <f>IF(K80=$B$221,L80,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81">
@@ -6553,6 +6856,10 @@
         <f>IF(K81&lt;&gt;"",A81,"")</f>
         <v/>
       </c>
+      <c r="O81">
+        <f>IF(K81=$B$221,L81,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82">
@@ -6603,6 +6910,10 @@
         <f>IF(K82&lt;&gt;"",A82,"")</f>
         <v/>
       </c>
+      <c r="O82">
+        <f>IF(K82=$B$221,L82,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83">
@@ -6653,6 +6964,10 @@
         <f>IF(K83&lt;&gt;"",A83,"")</f>
         <v/>
       </c>
+      <c r="O83">
+        <f>IF(K83=$B$221,L83,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84">
@@ -6703,6 +7018,10 @@
         <f>IF(K84&lt;&gt;"",A84,"")</f>
         <v/>
       </c>
+      <c r="O84">
+        <f>IF(K84=$B$221,L84,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85">
@@ -6753,6 +7072,10 @@
         <f>IF(K85&lt;&gt;"",A85,"")</f>
         <v/>
       </c>
+      <c r="O85">
+        <f>IF(K85=$B$221,L85,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86">
@@ -6803,6 +7126,10 @@
         <f>IF(K86&lt;&gt;"",A86,"")</f>
         <v/>
       </c>
+      <c r="O86">
+        <f>IF(K86=$B$221,L86,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87">
@@ -6853,6 +7180,10 @@
         <f>IF(K87&lt;&gt;"",A87,"")</f>
         <v/>
       </c>
+      <c r="O87">
+        <f>IF(K87=$B$221,L87,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88">
@@ -6903,6 +7234,10 @@
         <f>IF(K88&lt;&gt;"",A88,"")</f>
         <v/>
       </c>
+      <c r="O88">
+        <f>IF(K88=$B$221,L88,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89">
@@ -6953,6 +7288,10 @@
         <f>IF(K89&lt;&gt;"",A89,"")</f>
         <v/>
       </c>
+      <c r="O89">
+        <f>IF(K89=$B$221,L89,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90">
@@ -7003,6 +7342,10 @@
         <f>IF(K90&lt;&gt;"",A90,"")</f>
         <v/>
       </c>
+      <c r="O90">
+        <f>IF(K90=$B$221,L90,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91">
@@ -7053,6 +7396,10 @@
         <f>IF(K91&lt;&gt;"",A91,"")</f>
         <v/>
       </c>
+      <c r="O91">
+        <f>IF(K91=$B$221,L91,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92">
@@ -7103,6 +7450,10 @@
         <f>IF(K92&lt;&gt;"",A92,"")</f>
         <v/>
       </c>
+      <c r="O92">
+        <f>IF(K92=$B$221,L92,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93">
@@ -7153,6 +7504,10 @@
         <f>IF(K93&lt;&gt;"",A93,"")</f>
         <v/>
       </c>
+      <c r="O93">
+        <f>IF(K93=$B$221,L93,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94">
@@ -7203,6 +7558,10 @@
         <f>IF(K94&lt;&gt;"",A94,"")</f>
         <v/>
       </c>
+      <c r="O94">
+        <f>IF(K94=$B$221,L94,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95">
@@ -7253,6 +7612,10 @@
         <f>IF(K95&lt;&gt;"",A95,"")</f>
         <v/>
       </c>
+      <c r="O95">
+        <f>IF(K95=$B$221,L95,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96">
@@ -7303,6 +7666,10 @@
         <f>IF(K96&lt;&gt;"",A96,"")</f>
         <v/>
       </c>
+      <c r="O96">
+        <f>IF(K96=$B$221,L96,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97">
@@ -7353,6 +7720,10 @@
         <f>IF(K97&lt;&gt;"",A97,"")</f>
         <v/>
       </c>
+      <c r="O97">
+        <f>IF(K97=$B$221,L97,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98">
@@ -7403,6 +7774,10 @@
         <f>IF(K98&lt;&gt;"",A98,"")</f>
         <v/>
       </c>
+      <c r="O98">
+        <f>IF(K98=$B$221,L98,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99">
@@ -7453,6 +7828,10 @@
         <f>IF(K99&lt;&gt;"",A99,"")</f>
         <v/>
       </c>
+      <c r="O99">
+        <f>IF(K99=$B$221,L99,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100">
@@ -7503,6 +7882,10 @@
         <f>IF(K100&lt;&gt;"",A100,"")</f>
         <v/>
       </c>
+      <c r="O100">
+        <f>IF(K100=$B$221,L100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101">
@@ -7553,6 +7936,10 @@
         <f>IF(K101&lt;&gt;"",A101,"")</f>
         <v/>
       </c>
+      <c r="O101">
+        <f>IF(K101=$B$221,L101,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102">
@@ -7603,6 +7990,10 @@
         <f>IF(K102&lt;&gt;"",A102,"")</f>
         <v/>
       </c>
+      <c r="O102">
+        <f>IF(K102=$B$221,L102,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103">
@@ -7653,6 +8044,10 @@
         <f>IF(K103&lt;&gt;"",A103,"")</f>
         <v/>
       </c>
+      <c r="O103">
+        <f>IF(K103=$B$221,L103,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104">
@@ -7703,6 +8098,10 @@
         <f>IF(K104&lt;&gt;"",A104,"")</f>
         <v/>
       </c>
+      <c r="O104">
+        <f>IF(K104=$B$221,L104,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105">
@@ -7753,6 +8152,10 @@
         <f>IF(K105&lt;&gt;"",A105,"")</f>
         <v/>
       </c>
+      <c r="O105">
+        <f>IF(K105=$B$221,L105,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106">
@@ -7803,6 +8206,10 @@
         <f>IF(K106&lt;&gt;"",A106,"")</f>
         <v/>
       </c>
+      <c r="O106">
+        <f>IF(K106=$B$221,L106,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107">
@@ -7853,6 +8260,10 @@
         <f>IF(K107&lt;&gt;"",A107,"")</f>
         <v/>
       </c>
+      <c r="O107">
+        <f>IF(K107=$B$221,L107,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108">
@@ -7903,6 +8314,10 @@
         <f>IF(K108&lt;&gt;"",A108,"")</f>
         <v/>
       </c>
+      <c r="O108">
+        <f>IF(K108=$B$221,L108,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109">
@@ -7953,6 +8368,10 @@
         <f>IF(K109&lt;&gt;"",A109,"")</f>
         <v/>
       </c>
+      <c r="O109">
+        <f>IF(K109=$B$221,L109,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110">
@@ -8003,6 +8422,10 @@
         <f>IF(K110&lt;&gt;"",A110,"")</f>
         <v/>
       </c>
+      <c r="O110">
+        <f>IF(K110=$B$221,L110,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111">
@@ -8053,6 +8476,10 @@
         <f>IF(K111&lt;&gt;"",A111,"")</f>
         <v/>
       </c>
+      <c r="O111">
+        <f>IF(K111=$B$221,L111,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112">
@@ -8103,6 +8530,10 @@
         <f>IF(K112&lt;&gt;"",A112,"")</f>
         <v/>
       </c>
+      <c r="O112">
+        <f>IF(K112=$B$221,L112,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113">
@@ -8153,6 +8584,10 @@
         <f>IF(K113&lt;&gt;"",A113,"")</f>
         <v/>
       </c>
+      <c r="O113">
+        <f>IF(K113=$B$221,L113,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114">
@@ -8203,6 +8638,10 @@
         <f>IF(K114&lt;&gt;"",A114,"")</f>
         <v/>
       </c>
+      <c r="O114">
+        <f>IF(K114=$B$221,L114,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115">
@@ -8253,6 +8692,10 @@
         <f>IF(K115&lt;&gt;"",A115,"")</f>
         <v/>
       </c>
+      <c r="O115">
+        <f>IF(K115=$B$221,L115,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116">
@@ -8303,6 +8746,10 @@
         <f>IF(K116&lt;&gt;"",A116,"")</f>
         <v/>
       </c>
+      <c r="O116">
+        <f>IF(K116=$B$221,L116,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117">
@@ -8353,6 +8800,10 @@
         <f>IF(K117&lt;&gt;"",A117,"")</f>
         <v/>
       </c>
+      <c r="O117">
+        <f>IF(K117=$B$221,L117,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118">
@@ -8403,6 +8854,10 @@
         <f>IF(K118&lt;&gt;"",A118,"")</f>
         <v/>
       </c>
+      <c r="O118">
+        <f>IF(K118=$B$221,L118,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119">
@@ -8453,6 +8908,10 @@
         <f>IF(K119&lt;&gt;"",A119,"")</f>
         <v/>
       </c>
+      <c r="O119">
+        <f>IF(K119=$B$221,L119,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120">
@@ -8503,6 +8962,10 @@
         <f>IF(K120&lt;&gt;"",A120,"")</f>
         <v/>
       </c>
+      <c r="O120">
+        <f>IF(K120=$B$221,L120,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121">
@@ -8553,6 +9016,10 @@
         <f>IF(K121&lt;&gt;"",A121,"")</f>
         <v/>
       </c>
+      <c r="O121">
+        <f>IF(K121=$B$221,L121,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122">
@@ -8603,6 +9070,10 @@
         <f>IF(K122&lt;&gt;"",A122,"")</f>
         <v/>
       </c>
+      <c r="O122">
+        <f>IF(K122=$B$221,L122,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123">
@@ -8653,6 +9124,10 @@
         <f>IF(K123&lt;&gt;"",A123,"")</f>
         <v/>
       </c>
+      <c r="O123">
+        <f>IF(K123=$B$221,L123,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124">
@@ -8703,6 +9178,10 @@
         <f>IF(K124&lt;&gt;"",A124,"")</f>
         <v/>
       </c>
+      <c r="O124">
+        <f>IF(K124=$B$221,L124,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125">
@@ -8753,6 +9232,10 @@
         <f>IF(K125&lt;&gt;"",A125,"")</f>
         <v/>
       </c>
+      <c r="O125">
+        <f>IF(K125=$B$221,L125,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126">
@@ -8803,6 +9286,10 @@
         <f>IF(K126&lt;&gt;"",A126,"")</f>
         <v/>
       </c>
+      <c r="O126">
+        <f>IF(K126=$B$221,L126,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127">
@@ -8853,6 +9340,10 @@
         <f>IF(K127&lt;&gt;"",A127,"")</f>
         <v/>
       </c>
+      <c r="O127">
+        <f>IF(K127=$B$221,L127,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128">
@@ -8903,6 +9394,10 @@
         <f>IF(K128&lt;&gt;"",A128,"")</f>
         <v/>
       </c>
+      <c r="O128">
+        <f>IF(K128=$B$221,L128,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129">
@@ -8953,6 +9448,10 @@
         <f>IF(K129&lt;&gt;"",A129,"")</f>
         <v/>
       </c>
+      <c r="O129">
+        <f>IF(K129=$B$221,L129,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130">
@@ -9003,6 +9502,10 @@
         <f>IF(K130&lt;&gt;"",A130,"")</f>
         <v/>
       </c>
+      <c r="O130">
+        <f>IF(K130=$B$221,L130,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131">
@@ -9053,6 +9556,10 @@
         <f>IF(K131&lt;&gt;"",A131,"")</f>
         <v/>
       </c>
+      <c r="O131">
+        <f>IF(K131=$B$221,L131,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132">
@@ -9103,6 +9610,10 @@
         <f>IF(K132&lt;&gt;"",A132,"")</f>
         <v/>
       </c>
+      <c r="O132">
+        <f>IF(K132=$B$221,L132,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133">
@@ -9153,6 +9664,10 @@
         <f>IF(K133&lt;&gt;"",A133,"")</f>
         <v/>
       </c>
+      <c r="O133">
+        <f>IF(K133=$B$221,L133,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134">
@@ -9203,6 +9718,10 @@
         <f>IF(K134&lt;&gt;"",A134,"")</f>
         <v/>
       </c>
+      <c r="O134">
+        <f>IF(K134=$B$221,L134,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135">
@@ -9253,6 +9772,10 @@
         <f>IF(K135&lt;&gt;"",A135,"")</f>
         <v/>
       </c>
+      <c r="O135">
+        <f>IF(K135=$B$221,L135,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136">
@@ -9303,6 +9826,10 @@
         <f>IF(K136&lt;&gt;"",A136,"")</f>
         <v/>
       </c>
+      <c r="O136">
+        <f>IF(K136=$B$221,L136,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137">
@@ -9353,6 +9880,10 @@
         <f>IF(K137&lt;&gt;"",A137,"")</f>
         <v/>
       </c>
+      <c r="O137">
+        <f>IF(K137=$B$221,L137,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138">
@@ -9403,6 +9934,10 @@
         <f>IF(K138&lt;&gt;"",A138,"")</f>
         <v/>
       </c>
+      <c r="O138">
+        <f>IF(K138=$B$221,L138,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139">
@@ -9453,6 +9988,10 @@
         <f>IF(K139&lt;&gt;"",A139,"")</f>
         <v/>
       </c>
+      <c r="O139">
+        <f>IF(K139=$B$221,L139,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140">
@@ -9503,6 +10042,10 @@
         <f>IF(K140&lt;&gt;"",A140,"")</f>
         <v/>
       </c>
+      <c r="O140">
+        <f>IF(K140=$B$221,L140,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141">
@@ -9553,6 +10096,10 @@
         <f>IF(K141&lt;&gt;"",A141,"")</f>
         <v/>
       </c>
+      <c r="O141">
+        <f>IF(K141=$B$221,L141,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142">
@@ -9603,6 +10150,10 @@
         <f>IF(K142&lt;&gt;"",A142,"")</f>
         <v/>
       </c>
+      <c r="O142">
+        <f>IF(K142=$B$221,L142,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143">
@@ -9653,6 +10204,10 @@
         <f>IF(K143&lt;&gt;"",A143,"")</f>
         <v/>
       </c>
+      <c r="O143">
+        <f>IF(K143=$B$221,L143,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144">
@@ -9703,6 +10258,10 @@
         <f>IF(K144&lt;&gt;"",A144,"")</f>
         <v/>
       </c>
+      <c r="O144">
+        <f>IF(K144=$B$221,L144,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145">
@@ -9753,6 +10312,10 @@
         <f>IF(K145&lt;&gt;"",A145,"")</f>
         <v/>
       </c>
+      <c r="O145">
+        <f>IF(K145=$B$221,L145,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146">
@@ -9803,6 +10366,10 @@
         <f>IF(K146&lt;&gt;"",A146,"")</f>
         <v/>
       </c>
+      <c r="O146">
+        <f>IF(K146=$B$221,L146,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147">
@@ -9853,6 +10420,10 @@
         <f>IF(K147&lt;&gt;"",A147,"")</f>
         <v/>
       </c>
+      <c r="O147">
+        <f>IF(K147=$B$221,L147,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148">
@@ -9903,6 +10474,10 @@
         <f>IF(K148&lt;&gt;"",A148,"")</f>
         <v/>
       </c>
+      <c r="O148">
+        <f>IF(K148=$B$221,L148,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149">
@@ -9953,6 +10528,10 @@
         <f>IF(K149&lt;&gt;"",A149,"")</f>
         <v/>
       </c>
+      <c r="O149">
+        <f>IF(K149=$B$221,L149,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150">
@@ -10003,6 +10582,10 @@
         <f>IF(K150&lt;&gt;"",A150,"")</f>
         <v/>
       </c>
+      <c r="O150">
+        <f>IF(K150=$B$221,L150,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151">
@@ -10053,6 +10636,10 @@
         <f>IF(K151&lt;&gt;"",A151,"")</f>
         <v/>
       </c>
+      <c r="O151">
+        <f>IF(K151=$B$221,L151,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152">
@@ -10103,6 +10690,10 @@
         <f>IF(K152&lt;&gt;"",A152,"")</f>
         <v/>
       </c>
+      <c r="O152">
+        <f>IF(K152=$B$221,L152,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153">
@@ -10153,6 +10744,10 @@
         <f>IF(K153&lt;&gt;"",A153,"")</f>
         <v/>
       </c>
+      <c r="O153">
+        <f>IF(K153=$B$221,L153,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154">
@@ -10203,6 +10798,10 @@
         <f>IF(K154&lt;&gt;"",A154,"")</f>
         <v/>
       </c>
+      <c r="O154">
+        <f>IF(K154=$B$221,L154,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155">
@@ -10253,6 +10852,10 @@
         <f>IF(K155&lt;&gt;"",A155,"")</f>
         <v/>
       </c>
+      <c r="O155">
+        <f>IF(K155=$B$221,L155,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156">
@@ -10303,6 +10906,10 @@
         <f>IF(K156&lt;&gt;"",A156,"")</f>
         <v/>
       </c>
+      <c r="O156">
+        <f>IF(K156=$B$221,L156,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157">
@@ -10353,6 +10960,10 @@
         <f>IF(K157&lt;&gt;"",A157,"")</f>
         <v/>
       </c>
+      <c r="O157">
+        <f>IF(K157=$B$221,L157,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158">
@@ -10403,6 +11014,10 @@
         <f>IF(K158&lt;&gt;"",A158,"")</f>
         <v/>
       </c>
+      <c r="O158">
+        <f>IF(K158=$B$221,L158,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159">
@@ -10453,6 +11068,10 @@
         <f>IF(K159&lt;&gt;"",A159,"")</f>
         <v/>
       </c>
+      <c r="O159">
+        <f>IF(K159=$B$221,L159,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160">
@@ -10503,6 +11122,10 @@
         <f>IF(K160&lt;&gt;"",A160,"")</f>
         <v/>
       </c>
+      <c r="O160">
+        <f>IF(K160=$B$221,L160,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161">
@@ -10553,6 +11176,10 @@
         <f>IF(K161&lt;&gt;"",A161,"")</f>
         <v/>
       </c>
+      <c r="O161">
+        <f>IF(K161=$B$221,L161,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162">
@@ -10603,6 +11230,10 @@
         <f>IF(K162&lt;&gt;"",A162,"")</f>
         <v/>
       </c>
+      <c r="O162">
+        <f>IF(K162=$B$221,L162,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163">
@@ -10653,6 +11284,10 @@
         <f>IF(K163&lt;&gt;"",A163,"")</f>
         <v/>
       </c>
+      <c r="O163">
+        <f>IF(K163=$B$221,L163,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164">
@@ -10703,6 +11338,10 @@
         <f>IF(K164&lt;&gt;"",A164,"")</f>
         <v/>
       </c>
+      <c r="O164">
+        <f>IF(K164=$B$221,L164,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165">
@@ -10753,6 +11392,10 @@
         <f>IF(K165&lt;&gt;"",A165,"")</f>
         <v/>
       </c>
+      <c r="O165">
+        <f>IF(K165=$B$221,L165,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166">
@@ -10803,6 +11446,10 @@
         <f>IF(K166&lt;&gt;"",A166,"")</f>
         <v/>
       </c>
+      <c r="O166">
+        <f>IF(K166=$B$221,L166,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167">
@@ -10853,6 +11500,10 @@
         <f>IF(K167&lt;&gt;"",A167,"")</f>
         <v/>
       </c>
+      <c r="O167">
+        <f>IF(K167=$B$221,L167,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168">
@@ -10903,6 +11554,10 @@
         <f>IF(K168&lt;&gt;"",A168,"")</f>
         <v/>
       </c>
+      <c r="O168">
+        <f>IF(K168=$B$221,L168,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169">
@@ -10953,6 +11608,10 @@
         <f>IF(K169&lt;&gt;"",A169,"")</f>
         <v/>
       </c>
+      <c r="O169">
+        <f>IF(K169=$B$221,L169,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170">
@@ -11003,6 +11662,10 @@
         <f>IF(K170&lt;&gt;"",A170,"")</f>
         <v/>
       </c>
+      <c r="O170">
+        <f>IF(K170=$B$221,L170,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171">
@@ -11053,6 +11716,10 @@
         <f>IF(K171&lt;&gt;"",A171,"")</f>
         <v/>
       </c>
+      <c r="O171">
+        <f>IF(K171=$B$221,L171,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172">
@@ -11103,6 +11770,10 @@
         <f>IF(K172&lt;&gt;"",A172,"")</f>
         <v/>
       </c>
+      <c r="O172">
+        <f>IF(K172=$B$221,L172,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173">
@@ -11153,6 +11824,10 @@
         <f>IF(K173&lt;&gt;"",A173,"")</f>
         <v/>
       </c>
+      <c r="O173">
+        <f>IF(K173=$B$221,L173,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174">
@@ -11203,6 +11878,10 @@
         <f>IF(K174&lt;&gt;"",A174,"")</f>
         <v/>
       </c>
+      <c r="O174">
+        <f>IF(K174=$B$221,L174,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175">
@@ -11253,6 +11932,10 @@
         <f>IF(K175&lt;&gt;"",A175,"")</f>
         <v/>
       </c>
+      <c r="O175">
+        <f>IF(K175=$B$221,L175,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176">
@@ -11303,6 +11986,10 @@
         <f>IF(K176&lt;&gt;"",A176,"")</f>
         <v/>
       </c>
+      <c r="O176">
+        <f>IF(K176=$B$221,L176,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177">
@@ -11353,6 +12040,10 @@
         <f>IF(K177&lt;&gt;"",A177,"")</f>
         <v/>
       </c>
+      <c r="O177">
+        <f>IF(K177=$B$221,L177,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178">
@@ -11403,6 +12094,10 @@
         <f>IF(K178&lt;&gt;"",A178,"")</f>
         <v/>
       </c>
+      <c r="O178">
+        <f>IF(K178=$B$221,L178,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179">
@@ -11453,6 +12148,10 @@
         <f>IF(K179&lt;&gt;"",A179,"")</f>
         <v/>
       </c>
+      <c r="O179">
+        <f>IF(K179=$B$221,L179,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180">
@@ -11503,6 +12202,10 @@
         <f>IF(K180&lt;&gt;"",A180,"")</f>
         <v/>
       </c>
+      <c r="O180">
+        <f>IF(K180=$B$221,L180,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181">
@@ -11553,6 +12256,10 @@
         <f>IF(K181&lt;&gt;"",A181,"")</f>
         <v/>
       </c>
+      <c r="O181">
+        <f>IF(K181=$B$221,L181,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182">
@@ -11603,6 +12310,10 @@
         <f>IF(K182&lt;&gt;"",A182,"")</f>
         <v/>
       </c>
+      <c r="O182">
+        <f>IF(K182=$B$221,L182,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183">
@@ -11653,6 +12364,10 @@
         <f>IF(K183&lt;&gt;"",A183,"")</f>
         <v/>
       </c>
+      <c r="O183">
+        <f>IF(K183=$B$221,L183,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184">
@@ -11703,6 +12418,10 @@
         <f>IF(K184&lt;&gt;"",A184,"")</f>
         <v/>
       </c>
+      <c r="O184">
+        <f>IF(K184=$B$221,L184,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185">
@@ -11753,6 +12472,10 @@
         <f>IF(K185&lt;&gt;"",A185,"")</f>
         <v/>
       </c>
+      <c r="O185">
+        <f>IF(K185=$B$221,L185,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186">
@@ -11803,6 +12526,10 @@
         <f>IF(K186&lt;&gt;"",A186,"")</f>
         <v/>
       </c>
+      <c r="O186">
+        <f>IF(K186=$B$221,L186,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187">
@@ -11853,6 +12580,10 @@
         <f>IF(K187&lt;&gt;"",A187,"")</f>
         <v/>
       </c>
+      <c r="O187">
+        <f>IF(K187=$B$221,L187,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188">
@@ -11903,6 +12634,10 @@
         <f>IF(K188&lt;&gt;"",A188,"")</f>
         <v/>
       </c>
+      <c r="O188">
+        <f>IF(K188=$B$221,L188,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189">
@@ -11953,6 +12688,10 @@
         <f>IF(K189&lt;&gt;"",A189,"")</f>
         <v/>
       </c>
+      <c r="O189">
+        <f>IF(K189=$B$221,L189,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190">
@@ -12003,6 +12742,10 @@
         <f>IF(K190&lt;&gt;"",A190,"")</f>
         <v/>
       </c>
+      <c r="O190">
+        <f>IF(K190=$B$221,L190,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191">
@@ -12053,6 +12796,10 @@
         <f>IF(K191&lt;&gt;"",A191,"")</f>
         <v/>
       </c>
+      <c r="O191">
+        <f>IF(K191=$B$221,L191,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192">
@@ -12103,6 +12850,10 @@
         <f>IF(K192&lt;&gt;"",A192,"")</f>
         <v/>
       </c>
+      <c r="O192">
+        <f>IF(K192=$B$221,L192,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193">
@@ -12153,6 +12904,10 @@
         <f>IF(K193&lt;&gt;"",A193,"")</f>
         <v/>
       </c>
+      <c r="O193">
+        <f>IF(K193=$B$221,L193,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194">
@@ -12203,6 +12958,10 @@
         <f>IF(K194&lt;&gt;"",A194,"")</f>
         <v/>
       </c>
+      <c r="O194">
+        <f>IF(K194=$B$221,L194,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195">
@@ -12253,6 +13012,10 @@
         <f>IF(K195&lt;&gt;"",A195,"")</f>
         <v/>
       </c>
+      <c r="O195">
+        <f>IF(K195=$B$221,L195,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196">
@@ -12303,6 +13066,10 @@
         <f>IF(K196&lt;&gt;"",A196,"")</f>
         <v/>
       </c>
+      <c r="O196">
+        <f>IF(K196=$B$221,L196,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197">
@@ -12353,6 +13120,10 @@
         <f>IF(K197&lt;&gt;"",A197,"")</f>
         <v/>
       </c>
+      <c r="O197">
+        <f>IF(K197=$B$221,L197,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198">
@@ -12403,6 +13174,10 @@
         <f>IF(K198&lt;&gt;"",A198,"")</f>
         <v/>
       </c>
+      <c r="O198">
+        <f>IF(K198=$B$221,L198,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199">
@@ -12453,6 +13228,10 @@
         <f>IF(K199&lt;&gt;"",A199,"")</f>
         <v/>
       </c>
+      <c r="O199">
+        <f>IF(K199=$B$221,L199,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200">
@@ -12503,6 +13282,10 @@
         <f>IF(K200&lt;&gt;"",A200,"")</f>
         <v/>
       </c>
+      <c r="O200">
+        <f>IF(K200=$B$221,L200,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201">
@@ -12553,6 +13336,10 @@
         <f>IF(K201&lt;&gt;"",A201,"")</f>
         <v/>
       </c>
+      <c r="O201">
+        <f>IF(K201=$B$221,L201,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202">
@@ -12603,6 +13390,10 @@
         <f>IF(K202&lt;&gt;"",A202,"")</f>
         <v/>
       </c>
+      <c r="O202">
+        <f>IF(K202=$B$221,L202,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203">
@@ -12653,6 +13444,10 @@
         <f>IF(K203&lt;&gt;"",A203,"")</f>
         <v/>
       </c>
+      <c r="O203">
+        <f>IF(K203=$B$221,L203,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204">
@@ -12703,6 +13498,10 @@
         <f>IF(K204&lt;&gt;"",A204,"")</f>
         <v/>
       </c>
+      <c r="O204">
+        <f>IF(K204=$B$221,L204,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205">
@@ -12753,6 +13552,10 @@
         <f>IF(K205&lt;&gt;"",A205,"")</f>
         <v/>
       </c>
+      <c r="O205">
+        <f>IF(K205=$B$221,L205,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206">
@@ -12803,6 +13606,10 @@
         <f>IF(K206&lt;&gt;"",A206,"")</f>
         <v/>
       </c>
+      <c r="O206">
+        <f>IF(K206=$B$221,L206,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="A207">
@@ -12853,6 +13660,10 @@
         <f>IF(K207&lt;&gt;"",A207,"")</f>
         <v/>
       </c>
+      <c r="O207">
+        <f>IF(K207=$B$221,L207,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="208">
       <c r="A208">
@@ -12903,6 +13714,10 @@
         <f>IF(K208&lt;&gt;"",A208,"")</f>
         <v/>
       </c>
+      <c r="O208">
+        <f>IF(K208=$B$221,L208,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="A209">
@@ -12953,6 +13768,10 @@
         <f>IF(K209&lt;&gt;"",A209,"")</f>
         <v/>
       </c>
+      <c r="O209">
+        <f>IF(K209=$B$221,L209,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="A210">
@@ -13003,6 +13822,10 @@
         <f>IF(K210&lt;&gt;"",A210,"")</f>
         <v/>
       </c>
+      <c r="O210">
+        <f>IF(K210=$B$221,L210,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="A211">
@@ -13053,6 +13876,10 @@
         <f>IF(K211&lt;&gt;"",A211,"")</f>
         <v/>
       </c>
+      <c r="O211">
+        <f>IF(K211=$B$221,L211,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -13084,7 +13911,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IF(B221=0,"N/A",MINIFS(L12:L211,K12:K211,B221))</f>
+        <f>IF(B221=0,"N/A",MIN(O12:O211))</f>
         <v/>
       </c>
     </row>
@@ -13132,7 +13959,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N225"/>
+  <dimension ref="A1:O225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13437,6 +14264,10 @@
         <f>IF(N3=0,"Уровень не рассчитан",N3-4*Settings!$B$5*Settings!$B$3)</f>
         <v/>
       </c>
+      <c r="O12">
+        <f>IF(K12=$B$221,L12,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13">
@@ -13487,6 +14318,10 @@
         <f>IF(K13&lt;&gt;"",A13,"")</f>
         <v/>
       </c>
+      <c r="O13">
+        <f>IF(K13=$B$221,L13,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14">
@@ -13537,6 +14372,10 @@
         <f>IF(K14&lt;&gt;"",A14,"")</f>
         <v/>
       </c>
+      <c r="O14">
+        <f>IF(K14=$B$221,L14,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15">
@@ -13587,6 +14426,10 @@
         <f>IF(K15&lt;&gt;"",A15,"")</f>
         <v/>
       </c>
+      <c r="O15">
+        <f>IF(K15=$B$221,L15,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16">
@@ -13637,6 +14480,10 @@
         <f>IF(K16&lt;&gt;"",A16,"")</f>
         <v/>
       </c>
+      <c r="O16">
+        <f>IF(K16=$B$221,L16,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17">
@@ -13687,6 +14534,10 @@
         <f>IF(K17&lt;&gt;"",A17,"")</f>
         <v/>
       </c>
+      <c r="O17">
+        <f>IF(K17=$B$221,L17,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18">
@@ -13737,6 +14588,10 @@
         <f>IF(K18&lt;&gt;"",A18,"")</f>
         <v/>
       </c>
+      <c r="O18">
+        <f>IF(K18=$B$221,L18,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19">
@@ -13787,6 +14642,10 @@
         <f>IF(K19&lt;&gt;"",A19,"")</f>
         <v/>
       </c>
+      <c r="O19">
+        <f>IF(K19=$B$221,L19,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20">
@@ -13837,6 +14696,10 @@
         <f>IF(K20&lt;&gt;"",A20,"")</f>
         <v/>
       </c>
+      <c r="O20">
+        <f>IF(K20=$B$221,L20,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21">
@@ -13887,6 +14750,10 @@
         <f>IF(K21&lt;&gt;"",A21,"")</f>
         <v/>
       </c>
+      <c r="O21">
+        <f>IF(K21=$B$221,L21,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22">
@@ -13937,6 +14804,10 @@
         <f>IF(K22&lt;&gt;"",A22,"")</f>
         <v/>
       </c>
+      <c r="O22">
+        <f>IF(K22=$B$221,L22,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23">
@@ -13987,6 +14858,10 @@
         <f>IF(K23&lt;&gt;"",A23,"")</f>
         <v/>
       </c>
+      <c r="O23">
+        <f>IF(K23=$B$221,L23,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24">
@@ -14037,6 +14912,10 @@
         <f>IF(K24&lt;&gt;"",A24,"")</f>
         <v/>
       </c>
+      <c r="O24">
+        <f>IF(K24=$B$221,L24,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25">
@@ -14087,6 +14966,10 @@
         <f>IF(K25&lt;&gt;"",A25,"")</f>
         <v/>
       </c>
+      <c r="O25">
+        <f>IF(K25=$B$221,L25,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26">
@@ -14137,6 +15020,10 @@
         <f>IF(K26&lt;&gt;"",A26,"")</f>
         <v/>
       </c>
+      <c r="O26">
+        <f>IF(K26=$B$221,L26,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27">
@@ -14187,6 +15074,10 @@
         <f>IF(K27&lt;&gt;"",A27,"")</f>
         <v/>
       </c>
+      <c r="O27">
+        <f>IF(K27=$B$221,L27,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28">
@@ -14237,6 +15128,10 @@
         <f>IF(K28&lt;&gt;"",A28,"")</f>
         <v/>
       </c>
+      <c r="O28">
+        <f>IF(K28=$B$221,L28,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29">
@@ -14287,6 +15182,10 @@
         <f>IF(K29&lt;&gt;"",A29,"")</f>
         <v/>
       </c>
+      <c r="O29">
+        <f>IF(K29=$B$221,L29,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30">
@@ -14337,6 +15236,10 @@
         <f>IF(K30&lt;&gt;"",A30,"")</f>
         <v/>
       </c>
+      <c r="O30">
+        <f>IF(K30=$B$221,L30,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31">
@@ -14387,6 +15290,10 @@
         <f>IF(K31&lt;&gt;"",A31,"")</f>
         <v/>
       </c>
+      <c r="O31">
+        <f>IF(K31=$B$221,L31,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
@@ -14437,6 +15344,10 @@
         <f>IF(K32&lt;&gt;"",A32,"")</f>
         <v/>
       </c>
+      <c r="O32">
+        <f>IF(K32=$B$221,L32,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33">
@@ -14487,6 +15398,10 @@
         <f>IF(K33&lt;&gt;"",A33,"")</f>
         <v/>
       </c>
+      <c r="O33">
+        <f>IF(K33=$B$221,L33,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34">
@@ -14537,6 +15452,10 @@
         <f>IF(K34&lt;&gt;"",A34,"")</f>
         <v/>
       </c>
+      <c r="O34">
+        <f>IF(K34=$B$221,L34,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
@@ -14587,6 +15506,10 @@
         <f>IF(K35&lt;&gt;"",A35,"")</f>
         <v/>
       </c>
+      <c r="O35">
+        <f>IF(K35=$B$221,L35,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36">
@@ -14637,6 +15560,10 @@
         <f>IF(K36&lt;&gt;"",A36,"")</f>
         <v/>
       </c>
+      <c r="O36">
+        <f>IF(K36=$B$221,L36,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37">
@@ -14687,6 +15614,10 @@
         <f>IF(K37&lt;&gt;"",A37,"")</f>
         <v/>
       </c>
+      <c r="O37">
+        <f>IF(K37=$B$221,L37,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38">
@@ -14737,6 +15668,10 @@
         <f>IF(K38&lt;&gt;"",A38,"")</f>
         <v/>
       </c>
+      <c r="O38">
+        <f>IF(K38=$B$221,L38,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39">
@@ -14787,6 +15722,10 @@
         <f>IF(K39&lt;&gt;"",A39,"")</f>
         <v/>
       </c>
+      <c r="O39">
+        <f>IF(K39=$B$221,L39,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40">
@@ -14837,6 +15776,10 @@
         <f>IF(K40&lt;&gt;"",A40,"")</f>
         <v/>
       </c>
+      <c r="O40">
+        <f>IF(K40=$B$221,L40,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41">
@@ -14887,6 +15830,10 @@
         <f>IF(K41&lt;&gt;"",A41,"")</f>
         <v/>
       </c>
+      <c r="O41">
+        <f>IF(K41=$B$221,L41,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42">
@@ -14937,6 +15884,10 @@
         <f>IF(K42&lt;&gt;"",A42,"")</f>
         <v/>
       </c>
+      <c r="O42">
+        <f>IF(K42=$B$221,L42,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43">
@@ -14987,6 +15938,10 @@
         <f>IF(K43&lt;&gt;"",A43,"")</f>
         <v/>
       </c>
+      <c r="O43">
+        <f>IF(K43=$B$221,L43,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44">
@@ -15037,6 +15992,10 @@
         <f>IF(K44&lt;&gt;"",A44,"")</f>
         <v/>
       </c>
+      <c r="O44">
+        <f>IF(K44=$B$221,L44,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45">
@@ -15087,6 +16046,10 @@
         <f>IF(K45&lt;&gt;"",A45,"")</f>
         <v/>
       </c>
+      <c r="O45">
+        <f>IF(K45=$B$221,L45,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46">
@@ -15137,6 +16100,10 @@
         <f>IF(K46&lt;&gt;"",A46,"")</f>
         <v/>
       </c>
+      <c r="O46">
+        <f>IF(K46=$B$221,L46,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47">
@@ -15187,6 +16154,10 @@
         <f>IF(K47&lt;&gt;"",A47,"")</f>
         <v/>
       </c>
+      <c r="O47">
+        <f>IF(K47=$B$221,L47,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48">
@@ -15237,6 +16208,10 @@
         <f>IF(K48&lt;&gt;"",A48,"")</f>
         <v/>
       </c>
+      <c r="O48">
+        <f>IF(K48=$B$221,L48,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49">
@@ -15287,6 +16262,10 @@
         <f>IF(K49&lt;&gt;"",A49,"")</f>
         <v/>
       </c>
+      <c r="O49">
+        <f>IF(K49=$B$221,L49,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50">
@@ -15337,6 +16316,10 @@
         <f>IF(K50&lt;&gt;"",A50,"")</f>
         <v/>
       </c>
+      <c r="O50">
+        <f>IF(K50=$B$221,L50,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51">
@@ -15387,6 +16370,10 @@
         <f>IF(K51&lt;&gt;"",A51,"")</f>
         <v/>
       </c>
+      <c r="O51">
+        <f>IF(K51=$B$221,L51,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52">
@@ -15437,6 +16424,10 @@
         <f>IF(K52&lt;&gt;"",A52,"")</f>
         <v/>
       </c>
+      <c r="O52">
+        <f>IF(K52=$B$221,L52,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53">
@@ -15487,6 +16478,10 @@
         <f>IF(K53&lt;&gt;"",A53,"")</f>
         <v/>
       </c>
+      <c r="O53">
+        <f>IF(K53=$B$221,L53,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54">
@@ -15537,6 +16532,10 @@
         <f>IF(K54&lt;&gt;"",A54,"")</f>
         <v/>
       </c>
+      <c r="O54">
+        <f>IF(K54=$B$221,L54,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55">
@@ -15587,6 +16586,10 @@
         <f>IF(K55&lt;&gt;"",A55,"")</f>
         <v/>
       </c>
+      <c r="O55">
+        <f>IF(K55=$B$221,L55,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56">
@@ -15637,6 +16640,10 @@
         <f>IF(K56&lt;&gt;"",A56,"")</f>
         <v/>
       </c>
+      <c r="O56">
+        <f>IF(K56=$B$221,L56,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57">
@@ -15687,6 +16694,10 @@
         <f>IF(K57&lt;&gt;"",A57,"")</f>
         <v/>
       </c>
+      <c r="O57">
+        <f>IF(K57=$B$221,L57,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58">
@@ -15737,6 +16748,10 @@
         <f>IF(K58&lt;&gt;"",A58,"")</f>
         <v/>
       </c>
+      <c r="O58">
+        <f>IF(K58=$B$221,L58,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59">
@@ -15787,6 +16802,10 @@
         <f>IF(K59&lt;&gt;"",A59,"")</f>
         <v/>
       </c>
+      <c r="O59">
+        <f>IF(K59=$B$221,L59,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60">
@@ -15837,6 +16856,10 @@
         <f>IF(K60&lt;&gt;"",A60,"")</f>
         <v/>
       </c>
+      <c r="O60">
+        <f>IF(K60=$B$221,L60,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61">
@@ -15887,6 +16910,10 @@
         <f>IF(K61&lt;&gt;"",A61,"")</f>
         <v/>
       </c>
+      <c r="O61">
+        <f>IF(K61=$B$221,L61,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62">
@@ -15937,6 +16964,10 @@
         <f>IF(K62&lt;&gt;"",A62,"")</f>
         <v/>
       </c>
+      <c r="O62">
+        <f>IF(K62=$B$221,L62,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63">
@@ -15987,6 +17018,10 @@
         <f>IF(K63&lt;&gt;"",A63,"")</f>
         <v/>
       </c>
+      <c r="O63">
+        <f>IF(K63=$B$221,L63,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64">
@@ -16037,6 +17072,10 @@
         <f>IF(K64&lt;&gt;"",A64,"")</f>
         <v/>
       </c>
+      <c r="O64">
+        <f>IF(K64=$B$221,L64,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65">
@@ -16087,6 +17126,10 @@
         <f>IF(K65&lt;&gt;"",A65,"")</f>
         <v/>
       </c>
+      <c r="O65">
+        <f>IF(K65=$B$221,L65,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66">
@@ -16137,6 +17180,10 @@
         <f>IF(K66&lt;&gt;"",A66,"")</f>
         <v/>
       </c>
+      <c r="O66">
+        <f>IF(K66=$B$221,L66,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67">
@@ -16187,6 +17234,10 @@
         <f>IF(K67&lt;&gt;"",A67,"")</f>
         <v/>
       </c>
+      <c r="O67">
+        <f>IF(K67=$B$221,L67,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68">
@@ -16237,6 +17288,10 @@
         <f>IF(K68&lt;&gt;"",A68,"")</f>
         <v/>
       </c>
+      <c r="O68">
+        <f>IF(K68=$B$221,L68,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69">
@@ -16287,6 +17342,10 @@
         <f>IF(K69&lt;&gt;"",A69,"")</f>
         <v/>
       </c>
+      <c r="O69">
+        <f>IF(K69=$B$221,L69,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70">
@@ -16337,6 +17396,10 @@
         <f>IF(K70&lt;&gt;"",A70,"")</f>
         <v/>
       </c>
+      <c r="O70">
+        <f>IF(K70=$B$221,L70,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71">
@@ -16387,6 +17450,10 @@
         <f>IF(K71&lt;&gt;"",A71,"")</f>
         <v/>
       </c>
+      <c r="O71">
+        <f>IF(K71=$B$221,L71,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72">
@@ -16437,6 +17504,10 @@
         <f>IF(K72&lt;&gt;"",A72,"")</f>
         <v/>
       </c>
+      <c r="O72">
+        <f>IF(K72=$B$221,L72,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73">
@@ -16487,6 +17558,10 @@
         <f>IF(K73&lt;&gt;"",A73,"")</f>
         <v/>
       </c>
+      <c r="O73">
+        <f>IF(K73=$B$221,L73,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74">
@@ -16537,6 +17612,10 @@
         <f>IF(K74&lt;&gt;"",A74,"")</f>
         <v/>
       </c>
+      <c r="O74">
+        <f>IF(K74=$B$221,L74,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75">
@@ -16587,6 +17666,10 @@
         <f>IF(K75&lt;&gt;"",A75,"")</f>
         <v/>
       </c>
+      <c r="O75">
+        <f>IF(K75=$B$221,L75,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76">
@@ -16637,6 +17720,10 @@
         <f>IF(K76&lt;&gt;"",A76,"")</f>
         <v/>
       </c>
+      <c r="O76">
+        <f>IF(K76=$B$221,L76,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77">
@@ -16687,6 +17774,10 @@
         <f>IF(K77&lt;&gt;"",A77,"")</f>
         <v/>
       </c>
+      <c r="O77">
+        <f>IF(K77=$B$221,L77,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78">
@@ -16737,6 +17828,10 @@
         <f>IF(K78&lt;&gt;"",A78,"")</f>
         <v/>
       </c>
+      <c r="O78">
+        <f>IF(K78=$B$221,L78,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79">
@@ -16787,6 +17882,10 @@
         <f>IF(K79&lt;&gt;"",A79,"")</f>
         <v/>
       </c>
+      <c r="O79">
+        <f>IF(K79=$B$221,L79,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80">
@@ -16837,6 +17936,10 @@
         <f>IF(K80&lt;&gt;"",A80,"")</f>
         <v/>
       </c>
+      <c r="O80">
+        <f>IF(K80=$B$221,L80,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81">
@@ -16887,6 +17990,10 @@
         <f>IF(K81&lt;&gt;"",A81,"")</f>
         <v/>
       </c>
+      <c r="O81">
+        <f>IF(K81=$B$221,L81,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82">
@@ -16937,6 +18044,10 @@
         <f>IF(K82&lt;&gt;"",A82,"")</f>
         <v/>
       </c>
+      <c r="O82">
+        <f>IF(K82=$B$221,L82,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83">
@@ -16987,6 +18098,10 @@
         <f>IF(K83&lt;&gt;"",A83,"")</f>
         <v/>
       </c>
+      <c r="O83">
+        <f>IF(K83=$B$221,L83,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84">
@@ -17037,6 +18152,10 @@
         <f>IF(K84&lt;&gt;"",A84,"")</f>
         <v/>
       </c>
+      <c r="O84">
+        <f>IF(K84=$B$221,L84,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85">
@@ -17087,6 +18206,10 @@
         <f>IF(K85&lt;&gt;"",A85,"")</f>
         <v/>
       </c>
+      <c r="O85">
+        <f>IF(K85=$B$221,L85,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86">
@@ -17137,6 +18260,10 @@
         <f>IF(K86&lt;&gt;"",A86,"")</f>
         <v/>
       </c>
+      <c r="O86">
+        <f>IF(K86=$B$221,L86,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87">
@@ -17187,6 +18314,10 @@
         <f>IF(K87&lt;&gt;"",A87,"")</f>
         <v/>
       </c>
+      <c r="O87">
+        <f>IF(K87=$B$221,L87,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88">
@@ -17237,6 +18368,10 @@
         <f>IF(K88&lt;&gt;"",A88,"")</f>
         <v/>
       </c>
+      <c r="O88">
+        <f>IF(K88=$B$221,L88,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89">
@@ -17287,6 +18422,10 @@
         <f>IF(K89&lt;&gt;"",A89,"")</f>
         <v/>
       </c>
+      <c r="O89">
+        <f>IF(K89=$B$221,L89,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90">
@@ -17337,6 +18476,10 @@
         <f>IF(K90&lt;&gt;"",A90,"")</f>
         <v/>
       </c>
+      <c r="O90">
+        <f>IF(K90=$B$221,L90,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91">
@@ -17387,6 +18530,10 @@
         <f>IF(K91&lt;&gt;"",A91,"")</f>
         <v/>
       </c>
+      <c r="O91">
+        <f>IF(K91=$B$221,L91,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92">
@@ -17437,6 +18584,10 @@
         <f>IF(K92&lt;&gt;"",A92,"")</f>
         <v/>
       </c>
+      <c r="O92">
+        <f>IF(K92=$B$221,L92,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93">
@@ -17487,6 +18638,10 @@
         <f>IF(K93&lt;&gt;"",A93,"")</f>
         <v/>
       </c>
+      <c r="O93">
+        <f>IF(K93=$B$221,L93,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94">
@@ -17537,6 +18692,10 @@
         <f>IF(K94&lt;&gt;"",A94,"")</f>
         <v/>
       </c>
+      <c r="O94">
+        <f>IF(K94=$B$221,L94,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95">
@@ -17587,6 +18746,10 @@
         <f>IF(K95&lt;&gt;"",A95,"")</f>
         <v/>
       </c>
+      <c r="O95">
+        <f>IF(K95=$B$221,L95,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96">
@@ -17637,6 +18800,10 @@
         <f>IF(K96&lt;&gt;"",A96,"")</f>
         <v/>
       </c>
+      <c r="O96">
+        <f>IF(K96=$B$221,L96,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="97">
       <c r="A97">
@@ -17687,6 +18854,10 @@
         <f>IF(K97&lt;&gt;"",A97,"")</f>
         <v/>
       </c>
+      <c r="O97">
+        <f>IF(K97=$B$221,L97,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="98">
       <c r="A98">
@@ -17737,6 +18908,10 @@
         <f>IF(K98&lt;&gt;"",A98,"")</f>
         <v/>
       </c>
+      <c r="O98">
+        <f>IF(K98=$B$221,L98,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="99">
       <c r="A99">
@@ -17787,6 +18962,10 @@
         <f>IF(K99&lt;&gt;"",A99,"")</f>
         <v/>
       </c>
+      <c r="O99">
+        <f>IF(K99=$B$221,L99,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="100">
       <c r="A100">
@@ -17837,6 +19016,10 @@
         <f>IF(K100&lt;&gt;"",A100,"")</f>
         <v/>
       </c>
+      <c r="O100">
+        <f>IF(K100=$B$221,L100,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="101">
       <c r="A101">
@@ -17887,6 +19070,10 @@
         <f>IF(K101&lt;&gt;"",A101,"")</f>
         <v/>
       </c>
+      <c r="O101">
+        <f>IF(K101=$B$221,L101,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="102">
       <c r="A102">
@@ -17937,6 +19124,10 @@
         <f>IF(K102&lt;&gt;"",A102,"")</f>
         <v/>
       </c>
+      <c r="O102">
+        <f>IF(K102=$B$221,L102,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="103">
       <c r="A103">
@@ -17987,6 +19178,10 @@
         <f>IF(K103&lt;&gt;"",A103,"")</f>
         <v/>
       </c>
+      <c r="O103">
+        <f>IF(K103=$B$221,L103,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="104">
       <c r="A104">
@@ -18037,6 +19232,10 @@
         <f>IF(K104&lt;&gt;"",A104,"")</f>
         <v/>
       </c>
+      <c r="O104">
+        <f>IF(K104=$B$221,L104,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="105">
       <c r="A105">
@@ -18087,6 +19286,10 @@
         <f>IF(K105&lt;&gt;"",A105,"")</f>
         <v/>
       </c>
+      <c r="O105">
+        <f>IF(K105=$B$221,L105,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="106">
       <c r="A106">
@@ -18137,6 +19340,10 @@
         <f>IF(K106&lt;&gt;"",A106,"")</f>
         <v/>
       </c>
+      <c r="O106">
+        <f>IF(K106=$B$221,L106,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="107">
       <c r="A107">
@@ -18187,6 +19394,10 @@
         <f>IF(K107&lt;&gt;"",A107,"")</f>
         <v/>
       </c>
+      <c r="O107">
+        <f>IF(K107=$B$221,L107,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="108">
       <c r="A108">
@@ -18237,6 +19448,10 @@
         <f>IF(K108&lt;&gt;"",A108,"")</f>
         <v/>
       </c>
+      <c r="O108">
+        <f>IF(K108=$B$221,L108,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="109">
       <c r="A109">
@@ -18287,6 +19502,10 @@
         <f>IF(K109&lt;&gt;"",A109,"")</f>
         <v/>
       </c>
+      <c r="O109">
+        <f>IF(K109=$B$221,L109,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="110">
       <c r="A110">
@@ -18337,6 +19556,10 @@
         <f>IF(K110&lt;&gt;"",A110,"")</f>
         <v/>
       </c>
+      <c r="O110">
+        <f>IF(K110=$B$221,L110,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="111">
       <c r="A111">
@@ -18387,6 +19610,10 @@
         <f>IF(K111&lt;&gt;"",A111,"")</f>
         <v/>
       </c>
+      <c r="O111">
+        <f>IF(K111=$B$221,L111,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="112">
       <c r="A112">
@@ -18437,6 +19664,10 @@
         <f>IF(K112&lt;&gt;"",A112,"")</f>
         <v/>
       </c>
+      <c r="O112">
+        <f>IF(K112=$B$221,L112,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="113">
       <c r="A113">
@@ -18487,6 +19718,10 @@
         <f>IF(K113&lt;&gt;"",A113,"")</f>
         <v/>
       </c>
+      <c r="O113">
+        <f>IF(K113=$B$221,L113,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="114">
       <c r="A114">
@@ -18537,6 +19772,10 @@
         <f>IF(K114&lt;&gt;"",A114,"")</f>
         <v/>
       </c>
+      <c r="O114">
+        <f>IF(K114=$B$221,L114,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="115">
       <c r="A115">
@@ -18587,6 +19826,10 @@
         <f>IF(K115&lt;&gt;"",A115,"")</f>
         <v/>
       </c>
+      <c r="O115">
+        <f>IF(K115=$B$221,L115,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="116">
       <c r="A116">
@@ -18637,6 +19880,10 @@
         <f>IF(K116&lt;&gt;"",A116,"")</f>
         <v/>
       </c>
+      <c r="O116">
+        <f>IF(K116=$B$221,L116,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="117">
       <c r="A117">
@@ -18687,6 +19934,10 @@
         <f>IF(K117&lt;&gt;"",A117,"")</f>
         <v/>
       </c>
+      <c r="O117">
+        <f>IF(K117=$B$221,L117,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="118">
       <c r="A118">
@@ -18737,6 +19988,10 @@
         <f>IF(K118&lt;&gt;"",A118,"")</f>
         <v/>
       </c>
+      <c r="O118">
+        <f>IF(K118=$B$221,L118,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="119">
       <c r="A119">
@@ -18787,6 +20042,10 @@
         <f>IF(K119&lt;&gt;"",A119,"")</f>
         <v/>
       </c>
+      <c r="O119">
+        <f>IF(K119=$B$221,L119,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="120">
       <c r="A120">
@@ -18837,6 +20096,10 @@
         <f>IF(K120&lt;&gt;"",A120,"")</f>
         <v/>
       </c>
+      <c r="O120">
+        <f>IF(K120=$B$221,L120,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="121">
       <c r="A121">
@@ -18887,6 +20150,10 @@
         <f>IF(K121&lt;&gt;"",A121,"")</f>
         <v/>
       </c>
+      <c r="O121">
+        <f>IF(K121=$B$221,L121,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="122">
       <c r="A122">
@@ -18937,6 +20204,10 @@
         <f>IF(K122&lt;&gt;"",A122,"")</f>
         <v/>
       </c>
+      <c r="O122">
+        <f>IF(K122=$B$221,L122,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="123">
       <c r="A123">
@@ -18987,6 +20258,10 @@
         <f>IF(K123&lt;&gt;"",A123,"")</f>
         <v/>
       </c>
+      <c r="O123">
+        <f>IF(K123=$B$221,L123,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="124">
       <c r="A124">
@@ -19037,6 +20312,10 @@
         <f>IF(K124&lt;&gt;"",A124,"")</f>
         <v/>
       </c>
+      <c r="O124">
+        <f>IF(K124=$B$221,L124,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="125">
       <c r="A125">
@@ -19087,6 +20366,10 @@
         <f>IF(K125&lt;&gt;"",A125,"")</f>
         <v/>
       </c>
+      <c r="O125">
+        <f>IF(K125=$B$221,L125,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="126">
       <c r="A126">
@@ -19137,6 +20420,10 @@
         <f>IF(K126&lt;&gt;"",A126,"")</f>
         <v/>
       </c>
+      <c r="O126">
+        <f>IF(K126=$B$221,L126,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="127">
       <c r="A127">
@@ -19187,6 +20474,10 @@
         <f>IF(K127&lt;&gt;"",A127,"")</f>
         <v/>
       </c>
+      <c r="O127">
+        <f>IF(K127=$B$221,L127,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="128">
       <c r="A128">
@@ -19237,6 +20528,10 @@
         <f>IF(K128&lt;&gt;"",A128,"")</f>
         <v/>
       </c>
+      <c r="O128">
+        <f>IF(K128=$B$221,L128,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="129">
       <c r="A129">
@@ -19287,6 +20582,10 @@
         <f>IF(K129&lt;&gt;"",A129,"")</f>
         <v/>
       </c>
+      <c r="O129">
+        <f>IF(K129=$B$221,L129,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="130">
       <c r="A130">
@@ -19337,6 +20636,10 @@
         <f>IF(K130&lt;&gt;"",A130,"")</f>
         <v/>
       </c>
+      <c r="O130">
+        <f>IF(K130=$B$221,L130,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="131">
       <c r="A131">
@@ -19387,6 +20690,10 @@
         <f>IF(K131&lt;&gt;"",A131,"")</f>
         <v/>
       </c>
+      <c r="O131">
+        <f>IF(K131=$B$221,L131,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="132">
       <c r="A132">
@@ -19437,6 +20744,10 @@
         <f>IF(K132&lt;&gt;"",A132,"")</f>
         <v/>
       </c>
+      <c r="O132">
+        <f>IF(K132=$B$221,L132,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="133">
       <c r="A133">
@@ -19487,6 +20798,10 @@
         <f>IF(K133&lt;&gt;"",A133,"")</f>
         <v/>
       </c>
+      <c r="O133">
+        <f>IF(K133=$B$221,L133,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="134">
       <c r="A134">
@@ -19537,6 +20852,10 @@
         <f>IF(K134&lt;&gt;"",A134,"")</f>
         <v/>
       </c>
+      <c r="O134">
+        <f>IF(K134=$B$221,L134,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="135">
       <c r="A135">
@@ -19587,6 +20906,10 @@
         <f>IF(K135&lt;&gt;"",A135,"")</f>
         <v/>
       </c>
+      <c r="O135">
+        <f>IF(K135=$B$221,L135,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="136">
       <c r="A136">
@@ -19637,6 +20960,10 @@
         <f>IF(K136&lt;&gt;"",A136,"")</f>
         <v/>
       </c>
+      <c r="O136">
+        <f>IF(K136=$B$221,L136,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="137">
       <c r="A137">
@@ -19687,6 +21014,10 @@
         <f>IF(K137&lt;&gt;"",A137,"")</f>
         <v/>
       </c>
+      <c r="O137">
+        <f>IF(K137=$B$221,L137,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="138">
       <c r="A138">
@@ -19737,6 +21068,10 @@
         <f>IF(K138&lt;&gt;"",A138,"")</f>
         <v/>
       </c>
+      <c r="O138">
+        <f>IF(K138=$B$221,L138,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="139">
       <c r="A139">
@@ -19787,6 +21122,10 @@
         <f>IF(K139&lt;&gt;"",A139,"")</f>
         <v/>
       </c>
+      <c r="O139">
+        <f>IF(K139=$B$221,L139,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="140">
       <c r="A140">
@@ -19837,6 +21176,10 @@
         <f>IF(K140&lt;&gt;"",A140,"")</f>
         <v/>
       </c>
+      <c r="O140">
+        <f>IF(K140=$B$221,L140,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="141">
       <c r="A141">
@@ -19887,6 +21230,10 @@
         <f>IF(K141&lt;&gt;"",A141,"")</f>
         <v/>
       </c>
+      <c r="O141">
+        <f>IF(K141=$B$221,L141,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="142">
       <c r="A142">
@@ -19937,6 +21284,10 @@
         <f>IF(K142&lt;&gt;"",A142,"")</f>
         <v/>
       </c>
+      <c r="O142">
+        <f>IF(K142=$B$221,L142,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="143">
       <c r="A143">
@@ -19987,6 +21338,10 @@
         <f>IF(K143&lt;&gt;"",A143,"")</f>
         <v/>
       </c>
+      <c r="O143">
+        <f>IF(K143=$B$221,L143,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="144">
       <c r="A144">
@@ -20037,6 +21392,10 @@
         <f>IF(K144&lt;&gt;"",A144,"")</f>
         <v/>
       </c>
+      <c r="O144">
+        <f>IF(K144=$B$221,L144,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="145">
       <c r="A145">
@@ -20087,6 +21446,10 @@
         <f>IF(K145&lt;&gt;"",A145,"")</f>
         <v/>
       </c>
+      <c r="O145">
+        <f>IF(K145=$B$221,L145,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="146">
       <c r="A146">
@@ -20137,6 +21500,10 @@
         <f>IF(K146&lt;&gt;"",A146,"")</f>
         <v/>
       </c>
+      <c r="O146">
+        <f>IF(K146=$B$221,L146,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="147">
       <c r="A147">
@@ -20187,6 +21554,10 @@
         <f>IF(K147&lt;&gt;"",A147,"")</f>
         <v/>
       </c>
+      <c r="O147">
+        <f>IF(K147=$B$221,L147,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="148">
       <c r="A148">
@@ -20237,6 +21608,10 @@
         <f>IF(K148&lt;&gt;"",A148,"")</f>
         <v/>
       </c>
+      <c r="O148">
+        <f>IF(K148=$B$221,L148,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="149">
       <c r="A149">
@@ -20287,6 +21662,10 @@
         <f>IF(K149&lt;&gt;"",A149,"")</f>
         <v/>
       </c>
+      <c r="O149">
+        <f>IF(K149=$B$221,L149,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="150">
       <c r="A150">
@@ -20337,6 +21716,10 @@
         <f>IF(K150&lt;&gt;"",A150,"")</f>
         <v/>
       </c>
+      <c r="O150">
+        <f>IF(K150=$B$221,L150,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="151">
       <c r="A151">
@@ -20387,6 +21770,10 @@
         <f>IF(K151&lt;&gt;"",A151,"")</f>
         <v/>
       </c>
+      <c r="O151">
+        <f>IF(K151=$B$221,L151,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="152">
       <c r="A152">
@@ -20437,6 +21824,10 @@
         <f>IF(K152&lt;&gt;"",A152,"")</f>
         <v/>
       </c>
+      <c r="O152">
+        <f>IF(K152=$B$221,L152,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="153">
       <c r="A153">
@@ -20487,6 +21878,10 @@
         <f>IF(K153&lt;&gt;"",A153,"")</f>
         <v/>
       </c>
+      <c r="O153">
+        <f>IF(K153=$B$221,L153,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="154">
       <c r="A154">
@@ -20537,6 +21932,10 @@
         <f>IF(K154&lt;&gt;"",A154,"")</f>
         <v/>
       </c>
+      <c r="O154">
+        <f>IF(K154=$B$221,L154,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="155">
       <c r="A155">
@@ -20587,6 +21986,10 @@
         <f>IF(K155&lt;&gt;"",A155,"")</f>
         <v/>
       </c>
+      <c r="O155">
+        <f>IF(K155=$B$221,L155,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="156">
       <c r="A156">
@@ -20637,6 +22040,10 @@
         <f>IF(K156&lt;&gt;"",A156,"")</f>
         <v/>
       </c>
+      <c r="O156">
+        <f>IF(K156=$B$221,L156,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="157">
       <c r="A157">
@@ -20687,6 +22094,10 @@
         <f>IF(K157&lt;&gt;"",A157,"")</f>
         <v/>
       </c>
+      <c r="O157">
+        <f>IF(K157=$B$221,L157,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="158">
       <c r="A158">
@@ -20737,6 +22148,10 @@
         <f>IF(K158&lt;&gt;"",A158,"")</f>
         <v/>
       </c>
+      <c r="O158">
+        <f>IF(K158=$B$221,L158,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="159">
       <c r="A159">
@@ -20787,6 +22202,10 @@
         <f>IF(K159&lt;&gt;"",A159,"")</f>
         <v/>
       </c>
+      <c r="O159">
+        <f>IF(K159=$B$221,L159,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="160">
       <c r="A160">
@@ -20837,6 +22256,10 @@
         <f>IF(K160&lt;&gt;"",A160,"")</f>
         <v/>
       </c>
+      <c r="O160">
+        <f>IF(K160=$B$221,L160,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="161">
       <c r="A161">
@@ -20887,6 +22310,10 @@
         <f>IF(K161&lt;&gt;"",A161,"")</f>
         <v/>
       </c>
+      <c r="O161">
+        <f>IF(K161=$B$221,L161,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="162">
       <c r="A162">
@@ -20937,6 +22364,10 @@
         <f>IF(K162&lt;&gt;"",A162,"")</f>
         <v/>
       </c>
+      <c r="O162">
+        <f>IF(K162=$B$221,L162,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="163">
       <c r="A163">
@@ -20987,6 +22418,10 @@
         <f>IF(K163&lt;&gt;"",A163,"")</f>
         <v/>
       </c>
+      <c r="O163">
+        <f>IF(K163=$B$221,L163,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="164">
       <c r="A164">
@@ -21037,6 +22472,10 @@
         <f>IF(K164&lt;&gt;"",A164,"")</f>
         <v/>
       </c>
+      <c r="O164">
+        <f>IF(K164=$B$221,L164,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="165">
       <c r="A165">
@@ -21087,6 +22526,10 @@
         <f>IF(K165&lt;&gt;"",A165,"")</f>
         <v/>
       </c>
+      <c r="O165">
+        <f>IF(K165=$B$221,L165,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="166">
       <c r="A166">
@@ -21137,6 +22580,10 @@
         <f>IF(K166&lt;&gt;"",A166,"")</f>
         <v/>
       </c>
+      <c r="O166">
+        <f>IF(K166=$B$221,L166,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="167">
       <c r="A167">
@@ -21187,6 +22634,10 @@
         <f>IF(K167&lt;&gt;"",A167,"")</f>
         <v/>
       </c>
+      <c r="O167">
+        <f>IF(K167=$B$221,L167,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="168">
       <c r="A168">
@@ -21237,6 +22688,10 @@
         <f>IF(K168&lt;&gt;"",A168,"")</f>
         <v/>
       </c>
+      <c r="O168">
+        <f>IF(K168=$B$221,L168,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="169">
       <c r="A169">
@@ -21287,6 +22742,10 @@
         <f>IF(K169&lt;&gt;"",A169,"")</f>
         <v/>
       </c>
+      <c r="O169">
+        <f>IF(K169=$B$221,L169,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="170">
       <c r="A170">
@@ -21337,6 +22796,10 @@
         <f>IF(K170&lt;&gt;"",A170,"")</f>
         <v/>
       </c>
+      <c r="O170">
+        <f>IF(K170=$B$221,L170,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="171">
       <c r="A171">
@@ -21387,6 +22850,10 @@
         <f>IF(K171&lt;&gt;"",A171,"")</f>
         <v/>
       </c>
+      <c r="O171">
+        <f>IF(K171=$B$221,L171,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="172">
       <c r="A172">
@@ -21437,6 +22904,10 @@
         <f>IF(K172&lt;&gt;"",A172,"")</f>
         <v/>
       </c>
+      <c r="O172">
+        <f>IF(K172=$B$221,L172,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="173">
       <c r="A173">
@@ -21487,6 +22958,10 @@
         <f>IF(K173&lt;&gt;"",A173,"")</f>
         <v/>
       </c>
+      <c r="O173">
+        <f>IF(K173=$B$221,L173,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="174">
       <c r="A174">
@@ -21537,6 +23012,10 @@
         <f>IF(K174&lt;&gt;"",A174,"")</f>
         <v/>
       </c>
+      <c r="O174">
+        <f>IF(K174=$B$221,L174,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="175">
       <c r="A175">
@@ -21587,6 +23066,10 @@
         <f>IF(K175&lt;&gt;"",A175,"")</f>
         <v/>
       </c>
+      <c r="O175">
+        <f>IF(K175=$B$221,L175,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="176">
       <c r="A176">
@@ -21637,6 +23120,10 @@
         <f>IF(K176&lt;&gt;"",A176,"")</f>
         <v/>
       </c>
+      <c r="O176">
+        <f>IF(K176=$B$221,L176,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="177">
       <c r="A177">
@@ -21687,6 +23174,10 @@
         <f>IF(K177&lt;&gt;"",A177,"")</f>
         <v/>
       </c>
+      <c r="O177">
+        <f>IF(K177=$B$221,L177,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="178">
       <c r="A178">
@@ -21737,6 +23228,10 @@
         <f>IF(K178&lt;&gt;"",A178,"")</f>
         <v/>
       </c>
+      <c r="O178">
+        <f>IF(K178=$B$221,L178,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="179">
       <c r="A179">
@@ -21787,6 +23282,10 @@
         <f>IF(K179&lt;&gt;"",A179,"")</f>
         <v/>
       </c>
+      <c r="O179">
+        <f>IF(K179=$B$221,L179,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="180">
       <c r="A180">
@@ -21837,6 +23336,10 @@
         <f>IF(K180&lt;&gt;"",A180,"")</f>
         <v/>
       </c>
+      <c r="O180">
+        <f>IF(K180=$B$221,L180,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="181">
       <c r="A181">
@@ -21887,6 +23390,10 @@
         <f>IF(K181&lt;&gt;"",A181,"")</f>
         <v/>
       </c>
+      <c r="O181">
+        <f>IF(K181=$B$221,L181,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="182">
       <c r="A182">
@@ -21937,6 +23444,10 @@
         <f>IF(K182&lt;&gt;"",A182,"")</f>
         <v/>
       </c>
+      <c r="O182">
+        <f>IF(K182=$B$221,L182,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="183">
       <c r="A183">
@@ -21987,6 +23498,10 @@
         <f>IF(K183&lt;&gt;"",A183,"")</f>
         <v/>
       </c>
+      <c r="O183">
+        <f>IF(K183=$B$221,L183,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="184">
       <c r="A184">
@@ -22037,6 +23552,10 @@
         <f>IF(K184&lt;&gt;"",A184,"")</f>
         <v/>
       </c>
+      <c r="O184">
+        <f>IF(K184=$B$221,L184,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="185">
       <c r="A185">
@@ -22087,6 +23606,10 @@
         <f>IF(K185&lt;&gt;"",A185,"")</f>
         <v/>
       </c>
+      <c r="O185">
+        <f>IF(K185=$B$221,L185,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="186">
       <c r="A186">
@@ -22137,6 +23660,10 @@
         <f>IF(K186&lt;&gt;"",A186,"")</f>
         <v/>
       </c>
+      <c r="O186">
+        <f>IF(K186=$B$221,L186,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="187">
       <c r="A187">
@@ -22187,6 +23714,10 @@
         <f>IF(K187&lt;&gt;"",A187,"")</f>
         <v/>
       </c>
+      <c r="O187">
+        <f>IF(K187=$B$221,L187,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="188">
       <c r="A188">
@@ -22237,6 +23768,10 @@
         <f>IF(K188&lt;&gt;"",A188,"")</f>
         <v/>
       </c>
+      <c r="O188">
+        <f>IF(K188=$B$221,L188,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="189">
       <c r="A189">
@@ -22287,6 +23822,10 @@
         <f>IF(K189&lt;&gt;"",A189,"")</f>
         <v/>
       </c>
+      <c r="O189">
+        <f>IF(K189=$B$221,L189,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="190">
       <c r="A190">
@@ -22337,6 +23876,10 @@
         <f>IF(K190&lt;&gt;"",A190,"")</f>
         <v/>
       </c>
+      <c r="O190">
+        <f>IF(K190=$B$221,L190,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="191">
       <c r="A191">
@@ -22387,6 +23930,10 @@
         <f>IF(K191&lt;&gt;"",A191,"")</f>
         <v/>
       </c>
+      <c r="O191">
+        <f>IF(K191=$B$221,L191,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="192">
       <c r="A192">
@@ -22437,6 +23984,10 @@
         <f>IF(K192&lt;&gt;"",A192,"")</f>
         <v/>
       </c>
+      <c r="O192">
+        <f>IF(K192=$B$221,L192,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="193">
       <c r="A193">
@@ -22487,6 +24038,10 @@
         <f>IF(K193&lt;&gt;"",A193,"")</f>
         <v/>
       </c>
+      <c r="O193">
+        <f>IF(K193=$B$221,L193,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="194">
       <c r="A194">
@@ -22537,6 +24092,10 @@
         <f>IF(K194&lt;&gt;"",A194,"")</f>
         <v/>
       </c>
+      <c r="O194">
+        <f>IF(K194=$B$221,L194,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="195">
       <c r="A195">
@@ -22587,6 +24146,10 @@
         <f>IF(K195&lt;&gt;"",A195,"")</f>
         <v/>
       </c>
+      <c r="O195">
+        <f>IF(K195=$B$221,L195,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="196">
       <c r="A196">
@@ -22637,6 +24200,10 @@
         <f>IF(K196&lt;&gt;"",A196,"")</f>
         <v/>
       </c>
+      <c r="O196">
+        <f>IF(K196=$B$221,L196,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="197">
       <c r="A197">
@@ -22687,6 +24254,10 @@
         <f>IF(K197&lt;&gt;"",A197,"")</f>
         <v/>
       </c>
+      <c r="O197">
+        <f>IF(K197=$B$221,L197,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="198">
       <c r="A198">
@@ -22737,6 +24308,10 @@
         <f>IF(K198&lt;&gt;"",A198,"")</f>
         <v/>
       </c>
+      <c r="O198">
+        <f>IF(K198=$B$221,L198,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="199">
       <c r="A199">
@@ -22787,6 +24362,10 @@
         <f>IF(K199&lt;&gt;"",A199,"")</f>
         <v/>
       </c>
+      <c r="O199">
+        <f>IF(K199=$B$221,L199,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="200">
       <c r="A200">
@@ -22837,6 +24416,10 @@
         <f>IF(K200&lt;&gt;"",A200,"")</f>
         <v/>
       </c>
+      <c r="O200">
+        <f>IF(K200=$B$221,L200,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="201">
       <c r="A201">
@@ -22887,6 +24470,10 @@
         <f>IF(K201&lt;&gt;"",A201,"")</f>
         <v/>
       </c>
+      <c r="O201">
+        <f>IF(K201=$B$221,L201,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="202">
       <c r="A202">
@@ -22937,6 +24524,10 @@
         <f>IF(K202&lt;&gt;"",A202,"")</f>
         <v/>
       </c>
+      <c r="O202">
+        <f>IF(K202=$B$221,L202,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="203">
       <c r="A203">
@@ -22987,6 +24578,10 @@
         <f>IF(K203&lt;&gt;"",A203,"")</f>
         <v/>
       </c>
+      <c r="O203">
+        <f>IF(K203=$B$221,L203,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="204">
       <c r="A204">
@@ -23037,6 +24632,10 @@
         <f>IF(K204&lt;&gt;"",A204,"")</f>
         <v/>
       </c>
+      <c r="O204">
+        <f>IF(K204=$B$221,L204,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="205">
       <c r="A205">
@@ -23087,6 +24686,10 @@
         <f>IF(K205&lt;&gt;"",A205,"")</f>
         <v/>
       </c>
+      <c r="O205">
+        <f>IF(K205=$B$221,L205,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="206">
       <c r="A206">
@@ -23137,6 +24740,10 @@
         <f>IF(K206&lt;&gt;"",A206,"")</f>
         <v/>
       </c>
+      <c r="O206">
+        <f>IF(K206=$B$221,L206,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="207">
       <c r="A207">
@@ -23187,6 +24794,10 @@
         <f>IF(K207&lt;&gt;"",A207,"")</f>
         <v/>
       </c>
+      <c r="O207">
+        <f>IF(K207=$B$221,L207,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="208">
       <c r="A208">
@@ -23237,6 +24848,10 @@
         <f>IF(K208&lt;&gt;"",A208,"")</f>
         <v/>
       </c>
+      <c r="O208">
+        <f>IF(K208=$B$221,L208,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="209">
       <c r="A209">
@@ -23287,6 +24902,10 @@
         <f>IF(K209&lt;&gt;"",A209,"")</f>
         <v/>
       </c>
+      <c r="O209">
+        <f>IF(K209=$B$221,L209,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="210">
       <c r="A210">
@@ -23337,6 +24956,10 @@
         <f>IF(K210&lt;&gt;"",A210,"")</f>
         <v/>
       </c>
+      <c r="O210">
+        <f>IF(K210=$B$221,L210,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="211">
       <c r="A211">
@@ -23387,6 +25010,10 @@
         <f>IF(K211&lt;&gt;"",A211,"")</f>
         <v/>
       </c>
+      <c r="O211">
+        <f>IF(K211=$B$221,L211,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -23418,7 +25045,7 @@
         </is>
       </c>
       <c r="B222">
-        <f>IF(B221=0,"N/A",MINIFS(L12:L211,K12:K211,B221))</f>
+        <f>IF(B221=0,"N/A",MIN(O12:O211))</f>
         <v/>
       </c>
     </row>

</xml_diff>